<commit_message>
Dark UChicago theme + DnD, flagship editor, schedule, prereq/conflict warnings
- Dark mode with UChicago maroon/gold palette; maroon header band.
- Drag-and-drop: catalog course -> quarter, and move placed courses between
  quarters (re-resolves to the target term's section; blocks invalid terms).
- Flagship section: configurable (course, professor) list seeded from defaults;
  make/un-make from the Flagship modal or via a section's star toggle.
- Bidding clarity: explicit 'Est. cost N pts' and 'Your bid' labels.
- Clicking a placed course opens its detail; placed cards show the schedule
  inline (e.g. 'W 8:30-11:30').
- Prereq warning icon on placed courses -> popup listing strict (missing ones
  flagged) and recommended prereqs.
- Scheduling-conflict icon when two courses in a quarter overlap in day/time.
- Parser: reject header text leaking into a section's time field.
</commit_message>
<xml_diff>
--- a/build/curriculum.xlsx
+++ b/build/curriculum.xlsx
@@ -437,7 +437,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="41" customWidth="1" min="8" max="8"/>
     <col width="60" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
@@ -1295,11 +1295,6 @@
           <t>Heltzer, Wendy</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>FINANCIAL ACCOUNTING (30000) - KLEYMENOVA, ANYA&gt;&gt;</t>
-        </is>
-      </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
@@ -1727,11 +1722,6 @@
           <t>Le, Anthony</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>FINANCIAL ACCOUNTING (30000) - NIKOLAEV, VALERI&gt;&gt;</t>
-        </is>
-      </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
@@ -8630,11 +8620,6 @@
       <c r="F77" t="n">
         <v>2025</v>
       </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>Professor Hugh Cole</t>
-        </is>
-      </c>
       <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr"/>
       <c r="L77" t="b">
@@ -12149,11 +12134,6 @@
           <t>Misra, Sanjog</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr">
-        <is>
-          <t>MICROECONOMICS (33001) - CAMPOS, CHRISTOPHER&gt;&gt;</t>
-        </is>
-      </c>
       <c r="I113" t="inlineStr">
         <is>
           <t>43100 43800</t>
@@ -12254,11 +12234,6 @@
       <c r="G114" t="inlineStr">
         <is>
           <t>Campos, Christopher</t>
-        </is>
-      </c>
-      <c r="H114" t="inlineStr">
-        <is>
-          <t>MICROECONOMICS (33001) - DIZON-ROSS, REBECCA&gt;&gt;</t>
         </is>
       </c>
       <c r="I114" t="inlineStr"/>
@@ -20598,11 +20573,6 @@
           <t>HSIEH, CHANG-TAI</t>
         </is>
       </c>
-      <c r="H191" t="inlineStr">
-        <is>
-          <t>Day/Time: TBD</t>
-        </is>
-      </c>
       <c r="I191" t="inlineStr"/>
       <c r="J191" t="inlineStr">
         <is>
@@ -20816,11 +20786,6 @@
           <t>Hsieh, Chang-Tai</t>
         </is>
       </c>
-      <c r="H193" t="inlineStr">
-        <is>
-          <t>APPLIED ECONOMICS WORKSHOP (33610) - BERTRAND, MARIANNE&gt;&gt; ;</t>
-        </is>
-      </c>
       <c r="I193" t="inlineStr"/>
       <c r="J193" t="inlineStr">
         <is>
@@ -21033,11 +20998,6 @@
       <c r="G195" t="inlineStr">
         <is>
           <t>Conway, Jacob; Kamenica, Emir</t>
-        </is>
-      </c>
-      <c r="H195" t="inlineStr">
-        <is>
-          <t>APPLIED ECONOMICS WORKSHOP (33610) - MINNI, VIRGINIA&gt;&gt; ; ZWICK,</t>
         </is>
       </c>
       <c r="I195" t="inlineStr"/>
@@ -22838,11 +22798,6 @@
           <t>Richert, Eric</t>
         </is>
       </c>
-      <c r="H212" t="inlineStr">
-        <is>
-          <t>ECONOMICS OF EDUCATION (33930) - CAMPOS, CHRISTOPHER&gt;&gt; ; MOUNTJOY,</t>
-        </is>
-      </c>
       <c r="I212" t="inlineStr"/>
       <c r="J212" t="inlineStr">
         <is>
@@ -26933,11 +26888,6 @@
           <t>Parrish, Priya</t>
         </is>
       </c>
-      <c r="H251" t="inlineStr">
-        <is>
-          <t>includes both “non-concessionary” or “market-rate” investments that target</t>
-        </is>
-      </c>
       <c r="I251" t="inlineStr"/>
       <c r="J251" t="inlineStr"/>
       <c r="K251" t="inlineStr">
@@ -29810,11 +29760,6 @@
           <t>STROMBERG, PER</t>
         </is>
       </c>
-      <c r="H279" t="inlineStr">
-        <is>
-          <t>Day/Time: TBD</t>
-        </is>
-      </c>
       <c r="I279" t="inlineStr"/>
       <c r="J279" t="inlineStr"/>
       <c r="L279" t="b">
@@ -37259,11 +37204,6 @@
           <t>Rajan, Raghuram</t>
         </is>
       </c>
-      <c r="H347" t="inlineStr">
-        <is>
-          <t>EMERGING MARKETS FINANCE AND ENTREPRENEURSHIP (35213) - COLONNELLI,</t>
-        </is>
-      </c>
       <c r="I347" t="inlineStr">
         <is>
           <t>35200 35201 30130 34101 35902</t>
@@ -37812,11 +37752,6 @@
       <c r="G352" t="inlineStr">
         <is>
           <t>Vishny, Robert</t>
-        </is>
-      </c>
-      <c r="H352" t="inlineStr">
-        <is>
-          <t>FINANCIAL CRISES (35218) - CHABOT, BEN&gt;&gt;</t>
         </is>
       </c>
       <c r="I352" t="inlineStr"/>
@@ -38234,11 +38169,6 @@
           <t>COLONNELLI, EMANUELE</t>
         </is>
       </c>
-      <c r="H356" t="inlineStr">
-        <is>
-          <t>Day/Time: TBD</t>
-        </is>
-      </c>
       <c r="I356" t="inlineStr"/>
       <c r="J356" t="inlineStr"/>
       <c r="L356" t="b">
@@ -53133,11 +53063,6 @@
       <c r="G496" t="inlineStr">
         <is>
           <t>Wu, George</t>
-        </is>
-      </c>
-      <c r="H496" t="inlineStr">
-        <is>
-          <t>negotiation.</t>
         </is>
       </c>
       <c r="I496" t="inlineStr">

</xml_diff>

<commit_message>
Rewrite prereq classification: notation-anchored strict + OR-groups
Strict prereqs are now only those explicitly notated ('X (strict)',
'<clause>: strict', '<clause> is/are strict') and attach to the course(s)
on the left of the notation, not the whole list. Lists joined by
'or'/'at least one of' become OR-groups (any one satisfies). Everything
unnotated is recommended; anti-requisites ('cannot enroll if X taken
previously') are not-concurrent. Strict courses dropped from ~80 to 27
(14 OR-groups); e.g. 35200 strict={35000} only, 34101 strict={one of
35200/35201/35902/34106/30130}. App prereq popup/flag now group-aware.
</commit_message>
<xml_diff>
--- a/build/curriculum.xlsx
+++ b/build/curriculum.xlsx
@@ -438,7 +438,7 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="41" customWidth="1" min="8" max="8"/>
-    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
     <col width="32" customWidth="1" min="12" max="12"/>
@@ -2567,7 +2567,7 @@
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
-          <t>30000 33001 41000 41100 20101 30001</t>
+          <t>30000 33001 41000 41100</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2679,7 +2679,7 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>30000 33001 41000 41100 20101 30001</t>
+          <t>30000 33001 41000 41100</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -2791,7 +2791,7 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
-          <t>30000 33001 41000 41100 20101 30001</t>
+          <t>30000 33001 41000 41100</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2898,7 +2898,7 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>30000 33001 41000 41100 20101 30001</t>
+          <t>30000 33001 41000 41100</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -3004,7 +3004,7 @@
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
-          <t>30000 33001 41000 41100 20101 30001</t>
+          <t>30000 33001 41000 41100</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -3116,7 +3116,7 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
-          <t>30000 33001 41000 41100 20101 30001</t>
+          <t>30000 33001 41000 41100</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -3228,7 +3228,7 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
-          <t>30000 33001 41000 41100 20101 30001</t>
+          <t>30000 33001 41000 41100</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -3340,7 +3340,7 @@
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
-          <t>30000 30116 20140</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -3452,7 +3452,7 @@
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
-          <t>30000 30116 20140</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -3564,7 +3564,7 @@
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
-          <t>30000 30116 20140</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -3670,7 +3670,7 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
-          <t>30000 30116 20140</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -3776,7 +3776,7 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
-          <t>30000 35200 20170</t>
+          <t>30000 35200</t>
         </is>
       </c>
       <c r="L31" t="b">
@@ -3883,7 +3883,7 @@
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
         <is>
-          <t>30000 35200 20170</t>
+          <t>30000 35200</t>
         </is>
       </c>
       <c r="L32" t="b">
@@ -3990,7 +3990,7 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t>30000 35200 20170</t>
+          <t>30000 35200</t>
         </is>
       </c>
       <c r="L33" t="b">
@@ -4097,7 +4097,7 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
-          <t>30000 35200 20170</t>
+          <t>30000 35200</t>
         </is>
       </c>
       <c r="L34" t="b">
@@ -4204,7 +4204,7 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>30000 20160 30835</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="L35" t="b">
@@ -4311,7 +4311,7 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
-          <t>30000 20160 30835</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="L36" t="b">
@@ -4418,7 +4418,7 @@
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>30000 20160 30835</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="L37" t="b">
@@ -4525,7 +4525,7 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
-          <t>30000 20160 30835</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="L38" t="b">
@@ -4632,7 +4632,7 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>30000 20160 30835</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="L39" t="b">
@@ -4739,7 +4739,7 @@
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
-          <t>30000 20160 30835</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="L40" t="b">
@@ -4846,7 +4846,7 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
-          <t>30000 20160 30835</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="L41" t="b">
@@ -4950,12 +4950,12 @@
           <t>W 8:30 AM-11:30 AM</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
         <is>
           <t>30000 30130 30116 30118 30131</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
           <t>Financial Accounting</t>
@@ -5062,14 +5062,10 @@
           <t>F 8:30 AM-11:30 AM</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>30130 30000 35200</t>
-        </is>
-      </c>
+      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
-          <t>35000 20150</t>
+          <t>30000 35200 35000 20150</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -5178,14 +5174,10 @@
           <t>TH 6:00 PM-9:00 PM</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>30130 30000 35200</t>
-        </is>
-      </c>
+      <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
-          <t>35000 20150</t>
+          <t>30000 35200 35000 20150</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -5294,14 +5286,10 @@
           <t>W 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>30130 30000 35200</t>
-        </is>
-      </c>
+      <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>35000 20150</t>
+          <t>30000 35200 35000 20150</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -5410,14 +5398,10 @@
           <t>W 6:00 PM-9:00 PM</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>30130 30000 35200</t>
-        </is>
-      </c>
+      <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr">
         <is>
-          <t>35000 20150</t>
+          <t>30000 35200 35000 20150</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -5526,14 +5510,10 @@
           <t>M 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>30130 30000 35200</t>
-        </is>
-      </c>
+      <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
-          <t>35000 20150</t>
+          <t>30000 35200 35000 20150</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -5642,14 +5622,10 @@
           <t>T 6:00 PM-9:00 PM</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>30130 30000 35200</t>
-        </is>
-      </c>
+      <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr">
         <is>
-          <t>35000 20150</t>
+          <t>30000 35200 35000 20150</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -5758,14 +5734,10 @@
           <t>S 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>30130 30000 35200</t>
-        </is>
-      </c>
+      <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
-          <t>35000 20150</t>
+          <t>30000 35200 35000 20150</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -5874,14 +5846,10 @@
           <t>W 8:30 AM-11:30 AM</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>30130 30000 35200</t>
-        </is>
-      </c>
+      <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
-          <t>35000 20150</t>
+          <t>30000 35200 35000 20150</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -5990,14 +5958,10 @@
           <t>T 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>30130 30000 35200</t>
-        </is>
-      </c>
+      <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
-          <t>35000 20150</t>
+          <t>30000 35200 35000 20150</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -7356,11 +7320,7 @@
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>30122</t>
-        </is>
-      </c>
+      <c r="J64" t="inlineStr"/>
       <c r="L64" t="b">
         <v>0</v>
       </c>
@@ -10468,7 +10428,7 @@
       <c r="I97" t="inlineStr"/>
       <c r="J97" t="inlineStr">
         <is>
-          <t>31001 31403 31404</t>
+          <t>31001 31404</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -10580,7 +10540,7 @@
       <c r="I98" t="inlineStr"/>
       <c r="J98" t="inlineStr">
         <is>
-          <t>31001 31403 31404</t>
+          <t>31001 31404</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -10692,7 +10652,7 @@
       <c r="I99" t="inlineStr"/>
       <c r="J99" t="inlineStr">
         <is>
-          <t>31001 31403 31404</t>
+          <t>31001 31404</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -10804,7 +10764,7 @@
       <c r="I100" t="inlineStr"/>
       <c r="J100" t="inlineStr">
         <is>
-          <t>31001 31403 31404</t>
+          <t>31001 31404</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -11210,11 +11170,7 @@
           <t>M 6:00 PM-9:00 PM</t>
         </is>
       </c>
-      <c r="I104" t="inlineStr">
-        <is>
-          <t>31407 31404</t>
-        </is>
-      </c>
+      <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr"/>
       <c r="L104" t="b">
         <v>0</v>
@@ -12134,11 +12090,7 @@
           <t>Misra, Sanjog</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr">
-        <is>
-          <t>43100 43800</t>
-        </is>
-      </c>
+      <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr"/>
       <c r="L113" t="b">
         <v>0</v>
@@ -14136,12 +14088,12 @@
           <t>T 6:00 PM-9:00 PM</t>
         </is>
       </c>
-      <c r="I132" t="inlineStr">
+      <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr">
         <is>
           <t>33001</t>
         </is>
       </c>
-      <c r="J132" t="inlineStr"/>
       <c r="K132" t="inlineStr">
         <is>
           <t>People</t>
@@ -14243,12 +14195,12 @@
           <t>W 6:00 PM-9:00 PM</t>
         </is>
       </c>
-      <c r="I133" t="inlineStr">
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr">
         <is>
           <t>33001</t>
         </is>
       </c>
-      <c r="J133" t="inlineStr"/>
       <c r="K133" t="inlineStr">
         <is>
           <t>People</t>
@@ -14349,12 +14301,12 @@
           <t>T 8:30 AM-11:30 AM</t>
         </is>
       </c>
-      <c r="I134" t="inlineStr">
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr">
         <is>
           <t>33001</t>
         </is>
       </c>
-      <c r="J134" t="inlineStr"/>
       <c r="K134" t="inlineStr">
         <is>
           <t>People</t>
@@ -14461,12 +14413,12 @@
           <t>TH 8:30 AM-11:30 AM</t>
         </is>
       </c>
-      <c r="I135" t="inlineStr">
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr">
         <is>
           <t>33001</t>
         </is>
       </c>
-      <c r="J135" t="inlineStr"/>
       <c r="K135" t="inlineStr">
         <is>
           <t>People</t>
@@ -14573,12 +14525,12 @@
           <t>T 6:00 PM-9:00 PM</t>
         </is>
       </c>
-      <c r="I136" t="inlineStr">
+      <c r="I136" t="inlineStr"/>
+      <c r="J136" t="inlineStr">
         <is>
           <t>33001</t>
         </is>
       </c>
-      <c r="J136" t="inlineStr"/>
       <c r="K136" t="inlineStr">
         <is>
           <t>People</t>
@@ -14687,7 +14639,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>33001 33050 33040 20200</t>
+          <t>33001</t>
         </is>
       </c>
       <c r="J137" t="inlineStr"/>
@@ -14799,7 +14751,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>33001 33050 33040 20200</t>
+          <t>33001</t>
         </is>
       </c>
       <c r="J138" t="inlineStr"/>
@@ -14911,7 +14863,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>33001 33050 33040 20200</t>
+          <t>33001</t>
         </is>
       </c>
       <c r="J139" t="inlineStr"/>
@@ -15023,7 +14975,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>33001 33050 33040 20200</t>
+          <t>33001</t>
         </is>
       </c>
       <c r="J140" t="inlineStr"/>
@@ -15135,7 +15087,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>33001 33050 33040 20200</t>
+          <t>33001</t>
         </is>
       </c>
       <c r="J141" t="inlineStr"/>
@@ -15247,7 +15199,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>33001 33050 33040 20200</t>
+          <t>33001</t>
         </is>
       </c>
       <c r="J142" t="inlineStr"/>
@@ -15359,7 +15311,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>33001 33050 33040 20200</t>
+          <t>33001</t>
         </is>
       </c>
       <c r="J143" t="inlineStr"/>
@@ -18470,11 +18422,7 @@
           <t>M 8:30 AM-11:30 AM</t>
         </is>
       </c>
-      <c r="I172" t="inlineStr">
-        <is>
-          <t>33401 20232</t>
-        </is>
-      </c>
+      <c r="I172" t="inlineStr"/>
       <c r="J172" t="inlineStr"/>
       <c r="K172" t="inlineStr">
         <is>
@@ -18582,11 +18530,7 @@
           <t>M 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I173" t="inlineStr">
-        <is>
-          <t>33401 20232</t>
-        </is>
-      </c>
+      <c r="I173" t="inlineStr"/>
       <c r="J173" t="inlineStr"/>
       <c r="K173" t="inlineStr">
         <is>
@@ -18694,11 +18638,7 @@
           <t>T 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I174" t="inlineStr">
-        <is>
-          <t>33401 20232</t>
-        </is>
-      </c>
+      <c r="I174" t="inlineStr"/>
       <c r="J174" t="inlineStr"/>
       <c r="K174" t="inlineStr">
         <is>
@@ -18806,11 +18746,7 @@
           <t>T 6:00 PM-9:00 PM</t>
         </is>
       </c>
-      <c r="I175" t="inlineStr">
-        <is>
-          <t>33401 20232</t>
-        </is>
-      </c>
+      <c r="I175" t="inlineStr"/>
       <c r="J175" t="inlineStr"/>
       <c r="K175" t="inlineStr">
         <is>
@@ -18918,11 +18854,7 @@
           <t>T 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I176" t="inlineStr">
-        <is>
-          <t>33401 20232</t>
-        </is>
-      </c>
+      <c r="I176" t="inlineStr"/>
       <c r="J176" t="inlineStr"/>
       <c r="K176" t="inlineStr">
         <is>
@@ -19030,11 +18962,7 @@
           <t>W 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I177" t="inlineStr">
-        <is>
-          <t>33401 20232</t>
-        </is>
-      </c>
+      <c r="I177" t="inlineStr"/>
       <c r="J177" t="inlineStr"/>
       <c r="K177" t="inlineStr">
         <is>
@@ -19142,11 +19070,7 @@
           <t>T 6:00 PM-9:00 PM</t>
         </is>
       </c>
-      <c r="I178" t="inlineStr">
-        <is>
-          <t>33401 20232</t>
-        </is>
-      </c>
+      <c r="I178" t="inlineStr"/>
       <c r="J178" t="inlineStr"/>
       <c r="K178" t="inlineStr">
         <is>
@@ -19684,7 +19608,7 @@
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>20940 33471</t>
+          <t>20940</t>
         </is>
       </c>
       <c r="J183" t="inlineStr"/>
@@ -19796,7 +19720,7 @@
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>20940 33471</t>
+          <t>20940</t>
         </is>
       </c>
       <c r="J184" t="inlineStr"/>
@@ -19908,7 +19832,7 @@
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>20940 33471</t>
+          <t>20940</t>
         </is>
       </c>
       <c r="J185" t="inlineStr"/>
@@ -20020,7 +19944,7 @@
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>20940 33471</t>
+          <t>20940</t>
         </is>
       </c>
       <c r="J186" t="inlineStr"/>
@@ -20130,12 +20054,12 @@
           <t>TH 6:00 PM-9:00 PM</t>
         </is>
       </c>
-      <c r="I187" t="inlineStr">
+      <c r="I187" t="inlineStr"/>
+      <c r="J187" t="inlineStr">
         <is>
           <t>33001</t>
         </is>
       </c>
-      <c r="J187" t="inlineStr"/>
       <c r="K187" t="inlineStr">
         <is>
           <t>Economy</t>
@@ -20245,7 +20169,7 @@
       <c r="I188" t="inlineStr"/>
       <c r="J188" t="inlineStr">
         <is>
-          <t>33050 33502 20230</t>
+          <t>33050</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -20357,7 +20281,7 @@
       <c r="I189" t="inlineStr"/>
       <c r="J189" t="inlineStr">
         <is>
-          <t>33050 33502 20230</t>
+          <t>33050</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -20469,7 +20393,7 @@
       <c r="I190" t="inlineStr"/>
       <c r="J190" t="inlineStr">
         <is>
-          <t>33050 33502 20230</t>
+          <t>33050</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -20899,11 +20823,7 @@
         </is>
       </c>
       <c r="I194" t="inlineStr"/>
-      <c r="J194" t="inlineStr">
-        <is>
-          <t>33610 54300</t>
-        </is>
-      </c>
+      <c r="J194" t="inlineStr"/>
       <c r="L194" t="b">
         <v>0</v>
       </c>
@@ -21001,11 +20921,7 @@
         </is>
       </c>
       <c r="I195" t="inlineStr"/>
-      <c r="J195" t="inlineStr">
-        <is>
-          <t>33610 54300</t>
-        </is>
-      </c>
+      <c r="J195" t="inlineStr"/>
       <c r="L195" t="b">
         <v>0</v>
       </c>
@@ -21108,11 +21024,7 @@
         </is>
       </c>
       <c r="I196" t="inlineStr"/>
-      <c r="J196" t="inlineStr">
-        <is>
-          <t>33610 54300</t>
-        </is>
-      </c>
+      <c r="J196" t="inlineStr"/>
       <c r="L196" t="b">
         <v>0</v>
       </c>
@@ -21215,11 +21127,7 @@
         </is>
       </c>
       <c r="I197" t="inlineStr"/>
-      <c r="J197" t="inlineStr">
-        <is>
-          <t>33630 53000</t>
-        </is>
-      </c>
+      <c r="J197" t="inlineStr"/>
       <c r="L197" t="b">
         <v>0</v>
       </c>
@@ -21322,11 +21230,7 @@
         </is>
       </c>
       <c r="I198" t="inlineStr"/>
-      <c r="J198" t="inlineStr">
-        <is>
-          <t>33630 53000</t>
-        </is>
-      </c>
+      <c r="J198" t="inlineStr"/>
       <c r="L198" t="b">
         <v>0</v>
       </c>
@@ -21429,11 +21333,7 @@
         </is>
       </c>
       <c r="I199" t="inlineStr"/>
-      <c r="J199" t="inlineStr">
-        <is>
-          <t>33630 53000</t>
-        </is>
-      </c>
+      <c r="J199" t="inlineStr"/>
       <c r="L199" t="b">
         <v>0</v>
       </c>
@@ -21536,11 +21436,7 @@
         </is>
       </c>
       <c r="I200" t="inlineStr"/>
-      <c r="J200" t="inlineStr">
-        <is>
-          <t>33650 57000</t>
-        </is>
-      </c>
+      <c r="J200" t="inlineStr"/>
       <c r="L200" t="b">
         <v>0</v>
       </c>
@@ -21643,11 +21539,7 @@
         </is>
       </c>
       <c r="I201" t="inlineStr"/>
-      <c r="J201" t="inlineStr">
-        <is>
-          <t>33650 57000</t>
-        </is>
-      </c>
+      <c r="J201" t="inlineStr"/>
       <c r="L201" t="b">
         <v>0</v>
       </c>
@@ -21750,11 +21642,7 @@
         </is>
       </c>
       <c r="I202" t="inlineStr"/>
-      <c r="J202" t="inlineStr">
-        <is>
-          <t>33650 57000</t>
-        </is>
-      </c>
+      <c r="J202" t="inlineStr"/>
       <c r="L202" t="b">
         <v>0</v>
       </c>
@@ -22165,11 +22053,7 @@
           <t>T 8:30 AM-11:30 AM</t>
         </is>
       </c>
-      <c r="I206" t="inlineStr">
-        <is>
-          <t>33914 30680</t>
-        </is>
-      </c>
+      <c r="I206" t="inlineStr"/>
       <c r="J206" t="inlineStr"/>
       <c r="L206" t="b">
         <v>0</v>
@@ -22377,7 +22261,7 @@
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>33001 33101 33002 30000 30100 30200</t>
+          <t>30100 30200 33001 33002 33101</t>
         </is>
       </c>
       <c r="J208" t="inlineStr"/>
@@ -22484,7 +22368,7 @@
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>33001 33101 33002 30000 30100 30200</t>
+          <t>30100 30200 33001 33002 33101</t>
         </is>
       </c>
       <c r="J209" t="inlineStr"/>
@@ -22592,7 +22476,7 @@
       <c r="I210" t="inlineStr"/>
       <c r="J210" t="inlineStr">
         <is>
-          <t>33001 33002 33101 30000 30100 30200 33921 40101</t>
+          <t>33001 33002 33101 30000 30100 30200</t>
         </is>
       </c>
       <c r="L210" t="b">
@@ -22699,7 +22583,7 @@
       <c r="I211" t="inlineStr"/>
       <c r="J211" t="inlineStr">
         <is>
-          <t>33921 33922 40201</t>
+          <t>33921</t>
         </is>
       </c>
       <c r="L211" t="b">
@@ -22801,7 +22685,7 @@
       <c r="I212" t="inlineStr"/>
       <c r="J212" t="inlineStr">
         <is>
-          <t>33921 33922 33923 40301</t>
+          <t>33921 33922</t>
         </is>
       </c>
       <c r="L212" t="b">
@@ -23011,7 +22895,7 @@
       <c r="I214" t="inlineStr"/>
       <c r="J214" t="inlineStr">
         <is>
-          <t>33931 30540 30100 30200 30300</t>
+          <t>30200 30300</t>
         </is>
       </c>
       <c r="L214" t="b">
@@ -23219,11 +23103,7 @@
         </is>
       </c>
       <c r="I216" t="inlineStr"/>
-      <c r="J216" t="inlineStr">
-        <is>
-          <t>33942 38001</t>
-        </is>
-      </c>
+      <c r="J216" t="inlineStr"/>
       <c r="L216" t="b">
         <v>0</v>
       </c>
@@ -23326,11 +23206,7 @@
         </is>
       </c>
       <c r="I217" t="inlineStr"/>
-      <c r="J217" t="inlineStr">
-        <is>
-          <t>33946 35101</t>
-        </is>
-      </c>
+      <c r="J217" t="inlineStr"/>
       <c r="L217" t="b">
         <v>0</v>
       </c>
@@ -23434,7 +23310,7 @@
       </c>
       <c r="I218" t="inlineStr">
         <is>
-          <t>35200 35201 35902 34106 30130</t>
+          <t>30130 34106 35200 35201 35902</t>
         </is>
       </c>
       <c r="J218" t="inlineStr"/>
@@ -23546,7 +23422,7 @@
       </c>
       <c r="I219" t="inlineStr">
         <is>
-          <t>35200 35201 35902 34106 30130</t>
+          <t>30130 34106 35200 35201 35902</t>
         </is>
       </c>
       <c r="J219" t="inlineStr"/>
@@ -23658,7 +23534,7 @@
       </c>
       <c r="I220" t="inlineStr">
         <is>
-          <t>35200 35201 35902 34106 30130</t>
+          <t>30130 34106 35200 35201 35902</t>
         </is>
       </c>
       <c r="J220" t="inlineStr"/>
@@ -23770,7 +23646,7 @@
       </c>
       <c r="I221" t="inlineStr">
         <is>
-          <t>35200 35201 35902 34106 30130</t>
+          <t>30130 34106 35200 35201 35902</t>
         </is>
       </c>
       <c r="J221" t="inlineStr"/>
@@ -23882,7 +23758,7 @@
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t>35200 35201 35902 34106 30130</t>
+          <t>30130 34106 35200 35201 35902</t>
         </is>
       </c>
       <c r="J222" t="inlineStr"/>
@@ -23994,7 +23870,7 @@
       </c>
       <c r="I223" t="inlineStr">
         <is>
-          <t>35200 35201 35902 34106 30130</t>
+          <t>30130 34106 35200 35201 35902</t>
         </is>
       </c>
       <c r="J223" t="inlineStr"/>
@@ -24106,7 +23982,7 @@
       </c>
       <c r="I224" t="inlineStr">
         <is>
-          <t>35200 35201 35902 34106 30130</t>
+          <t>30130 34106 35200 35201 35902</t>
         </is>
       </c>
       <c r="J224" t="inlineStr"/>
@@ -24213,7 +24089,7 @@
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>35200 35201 35902 34106 30130</t>
+          <t>30130 34106 35200 35201 35902</t>
         </is>
       </c>
       <c r="J225" t="inlineStr"/>
@@ -25028,11 +24904,7 @@
         </is>
       </c>
       <c r="I233" t="inlineStr"/>
-      <c r="J233" t="inlineStr">
-        <is>
-          <t>34103 20330</t>
-        </is>
-      </c>
+      <c r="J233" t="inlineStr"/>
       <c r="L233" t="b">
         <v>0</v>
       </c>
@@ -25135,11 +25007,7 @@
         </is>
       </c>
       <c r="I234" t="inlineStr"/>
-      <c r="J234" t="inlineStr">
-        <is>
-          <t>34103 20330</t>
-        </is>
-      </c>
+      <c r="J234" t="inlineStr"/>
       <c r="L234" t="b">
         <v>0</v>
       </c>
@@ -25242,11 +25110,7 @@
         </is>
       </c>
       <c r="I235" t="inlineStr"/>
-      <c r="J235" t="inlineStr">
-        <is>
-          <t>34103 20330</t>
-        </is>
-      </c>
+      <c r="J235" t="inlineStr"/>
       <c r="L235" t="b">
         <v>0</v>
       </c>
@@ -25349,11 +25213,7 @@
         </is>
       </c>
       <c r="I236" t="inlineStr"/>
-      <c r="J236" t="inlineStr">
-        <is>
-          <t>34103 20330</t>
-        </is>
-      </c>
+      <c r="J236" t="inlineStr"/>
       <c r="L236" t="b">
         <v>0</v>
       </c>
@@ -25456,11 +25316,7 @@
         </is>
       </c>
       <c r="I237" t="inlineStr"/>
-      <c r="J237" t="inlineStr">
-        <is>
-          <t>34103 20330</t>
-        </is>
-      </c>
+      <c r="J237" t="inlineStr"/>
       <c r="L237" t="b">
         <v>0</v>
       </c>
@@ -26364,11 +26220,7 @@
           <t>T 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I246" t="inlineStr">
-        <is>
-          <t>20355 34887</t>
-        </is>
-      </c>
+      <c r="I246" t="inlineStr"/>
       <c r="J246" t="inlineStr"/>
       <c r="L246" t="b">
         <v>0</v>
@@ -26471,11 +26323,7 @@
           <t>S 9:00 AM-12:00 PM</t>
         </is>
       </c>
-      <c r="I247" t="inlineStr">
-        <is>
-          <t>20355 34887</t>
-        </is>
-      </c>
+      <c r="I247" t="inlineStr"/>
       <c r="J247" t="inlineStr"/>
       <c r="L247" t="b">
         <v>0</v>
@@ -26578,11 +26426,7 @@
           <t>T 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I248" t="inlineStr">
-        <is>
-          <t>20355 34887</t>
-        </is>
-      </c>
+      <c r="I248" t="inlineStr"/>
       <c r="J248" t="inlineStr"/>
       <c r="L248" t="b">
         <v>0</v>
@@ -26685,11 +26529,7 @@
           <t>T 8:30 AM-11:30 AM</t>
         </is>
       </c>
-      <c r="I249" t="inlineStr">
-        <is>
-          <t>20355 34887</t>
-        </is>
-      </c>
+      <c r="I249" t="inlineStr"/>
       <c r="J249" t="inlineStr"/>
       <c r="L249" t="b">
         <v>0</v>
@@ -26792,11 +26632,7 @@
           <t>T 6:00 PM-9:00 PM</t>
         </is>
       </c>
-      <c r="I250" t="inlineStr">
-        <is>
-          <t>20355 34887</t>
-        </is>
-      </c>
+      <c r="I250" t="inlineStr"/>
       <c r="J250" t="inlineStr"/>
       <c r="L250" t="b">
         <v>0</v>
@@ -27606,12 +27442,12 @@
           <t>M 5:00 PM-8:00 PM</t>
         </is>
       </c>
-      <c r="I258" t="inlineStr">
+      <c r="I258" t="inlineStr"/>
+      <c r="J258" t="inlineStr">
         <is>
           <t>34211</t>
         </is>
       </c>
-      <c r="J258" t="inlineStr"/>
       <c r="L258" t="b">
         <v>0</v>
       </c>
@@ -28022,12 +27858,12 @@
           <t>W 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I262" t="inlineStr">
-        <is>
-          <t>34101 34219 34209</t>
-        </is>
-      </c>
-      <c r="J262" t="inlineStr"/>
+      <c r="I262" t="inlineStr"/>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>34101</t>
+        </is>
+      </c>
       <c r="L262" t="b">
         <v>0</v>
       </c>
@@ -29451,11 +29287,7 @@
         </is>
       </c>
       <c r="I276" t="inlineStr"/>
-      <c r="J276" t="inlineStr">
-        <is>
-          <t>20350</t>
-        </is>
-      </c>
+      <c r="J276" t="inlineStr"/>
       <c r="L276" t="b">
         <v>0</v>
       </c>
@@ -29558,11 +29390,7 @@
         </is>
       </c>
       <c r="I277" t="inlineStr"/>
-      <c r="J277" t="inlineStr">
-        <is>
-          <t>20350</t>
-        </is>
-      </c>
+      <c r="J277" t="inlineStr"/>
       <c r="L277" t="b">
         <v>0</v>
       </c>
@@ -29664,11 +29492,7 @@
           <t>F 8:30 AM-11:30 AM</t>
         </is>
       </c>
-      <c r="I278" t="inlineStr">
-        <is>
-          <t>34709 34706</t>
-        </is>
-      </c>
+      <c r="I278" t="inlineStr"/>
       <c r="J278" t="inlineStr"/>
       <c r="L278" t="b">
         <v>0</v>
@@ -29860,7 +29684,7 @@
       <c r="I280" t="inlineStr"/>
       <c r="J280" t="inlineStr">
         <is>
-          <t>34715 53455 33830 32002</t>
+          <t>33830 32002</t>
         </is>
       </c>
       <c r="L280" t="b">
@@ -30262,10 +30086,14 @@
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t>34901 35904 31000 31100 31200 33000 33100 33200 34902 35060</t>
-        </is>
-      </c>
-      <c r="J284" t="inlineStr"/>
+          <t>34901 35904</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>31100 31200 33100 33200</t>
+        </is>
+      </c>
       <c r="K284" t="inlineStr">
         <is>
           <t>Finance</t>
@@ -30372,11 +30200,7 @@
           <t>M 3:00 PM-6:00 PM</t>
         </is>
       </c>
-      <c r="I285" t="inlineStr">
-        <is>
-          <t>30100 30200 30300 34903 35070</t>
-        </is>
-      </c>
+      <c r="I285" t="inlineStr"/>
       <c r="J285" t="inlineStr"/>
       <c r="K285" t="inlineStr">
         <is>
@@ -30486,7 +30310,7 @@
       </c>
       <c r="I286" t="inlineStr">
         <is>
-          <t>34903 35902 34904 35080</t>
+          <t>34903 35902</t>
         </is>
       </c>
       <c r="J286" t="inlineStr"/>
@@ -30598,7 +30422,7 @@
       </c>
       <c r="I287" t="inlineStr">
         <is>
-          <t>34903 34904 34906 35090</t>
+          <t>34903 34904</t>
         </is>
       </c>
       <c r="J287" t="inlineStr"/>
@@ -30705,7 +30529,7 @@
       </c>
       <c r="I288" t="inlineStr">
         <is>
-          <t>41000 41100 35000 20400</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="J288" t="inlineStr">
@@ -30821,7 +30645,7 @@
       </c>
       <c r="I289" t="inlineStr">
         <is>
-          <t>41000 41100 35000 20400</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="J289" t="inlineStr">
@@ -30937,7 +30761,7 @@
       </c>
       <c r="I290" t="inlineStr">
         <is>
-          <t>41000 41100 35000 20400</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="J290" t="inlineStr">
@@ -31053,7 +30877,7 @@
       </c>
       <c r="I291" t="inlineStr">
         <is>
-          <t>41000 41100 35000 20400</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="J291" t="inlineStr">
@@ -31169,7 +30993,7 @@
       </c>
       <c r="I292" t="inlineStr">
         <is>
-          <t>41000 41100 35000 20400</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="J292" t="inlineStr">
@@ -31285,7 +31109,7 @@
       </c>
       <c r="I293" t="inlineStr">
         <is>
-          <t>41000 41100 35000 20400</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="J293" t="inlineStr">
@@ -31401,7 +31225,7 @@
       </c>
       <c r="I294" t="inlineStr">
         <is>
-          <t>41000 41100 35000 20400</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="J294" t="inlineStr">
@@ -31512,7 +31336,7 @@
       </c>
       <c r="I295" t="inlineStr">
         <is>
-          <t>41000 41100 35000 20400</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="J295" t="inlineStr">
@@ -31622,7 +31446,7 @@
       </c>
       <c r="I296" t="inlineStr">
         <is>
-          <t>41000 41100 35000 20400</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="J296" t="inlineStr">
@@ -31738,7 +31562,7 @@
       </c>
       <c r="I297" t="inlineStr">
         <is>
-          <t>41000 41100 35000 20400</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="J297" t="inlineStr">
@@ -31854,7 +31678,7 @@
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t>41000 41100 35000 20400</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="J298" t="inlineStr">
@@ -31970,7 +31794,7 @@
       </c>
       <c r="I299" t="inlineStr">
         <is>
-          <t>41000 41100 35000 20400</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="J299" t="inlineStr">
@@ -32086,7 +31910,7 @@
       </c>
       <c r="I300" t="inlineStr">
         <is>
-          <t>41000 41100 35000 20400</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="J300" t="inlineStr">
@@ -32202,7 +32026,7 @@
       </c>
       <c r="I301" t="inlineStr">
         <is>
-          <t>41000 41100 35000 20400</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="J301" t="inlineStr">
@@ -32313,7 +32137,7 @@
       </c>
       <c r="I302" t="inlineStr">
         <is>
-          <t>41000 41100 35000 20400</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="J302" t="inlineStr">
@@ -32418,7 +32242,7 @@
       </c>
       <c r="I303" t="inlineStr">
         <is>
-          <t>41000 41100 35000 20400</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="J303" t="inlineStr">
@@ -32526,11 +32350,7 @@
           <t>TH 8:30 AM-11:30 AM</t>
         </is>
       </c>
-      <c r="I304" t="inlineStr">
-        <is>
-          <t>35001 35010</t>
-        </is>
-      </c>
+      <c r="I304" t="inlineStr"/>
       <c r="J304" t="inlineStr">
         <is>
           <t>30000</t>
@@ -32642,11 +32462,7 @@
           <t>S 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I305" t="inlineStr">
-        <is>
-          <t>35001 35010</t>
-        </is>
-      </c>
+      <c r="I305" t="inlineStr"/>
       <c r="J305" t="inlineStr">
         <is>
           <t>30000</t>
@@ -32758,12 +32574,12 @@
           <t>TH 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I306" t="inlineStr">
-        <is>
-          <t>30000 35010 35001</t>
-        </is>
-      </c>
-      <c r="J306" t="inlineStr"/>
+      <c r="I306" t="inlineStr"/>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>30000</t>
+        </is>
+      </c>
       <c r="L306" t="b">
         <v>0</v>
       </c>
@@ -32979,7 +32795,7 @@
       </c>
       <c r="I308" t="inlineStr">
         <is>
-          <t>41000 35000 35200</t>
+          <t>35000 35200 41000</t>
         </is>
       </c>
       <c r="J308" t="inlineStr"/>
@@ -33420,12 +33236,12 @@
           <t>T 8:30 AM-11:30 AM</t>
         </is>
       </c>
-      <c r="I312" t="inlineStr">
+      <c r="I312" t="inlineStr"/>
+      <c r="J312" t="inlineStr">
         <is>
           <t>35000 41100 35215</t>
         </is>
       </c>
-      <c r="J312" t="inlineStr"/>
       <c r="L312" t="b">
         <v>0</v>
       </c>
@@ -33529,10 +33345,14 @@
       </c>
       <c r="I313" t="inlineStr">
         <is>
-          <t>30000 33001 35000 41000 41100</t>
-        </is>
-      </c>
-      <c r="J313" t="inlineStr"/>
+          <t>41000 41100</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>30000 33001 35000</t>
+        </is>
+      </c>
       <c r="L313" t="b">
         <v>0</v>
       </c>
@@ -33636,10 +33456,14 @@
       </c>
       <c r="I314" t="inlineStr">
         <is>
-          <t>30000 33001 35000 41000 41100</t>
-        </is>
-      </c>
-      <c r="J314" t="inlineStr"/>
+          <t>41000 41100</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>30000 33001 35000</t>
+        </is>
+      </c>
       <c r="L314" t="b">
         <v>0</v>
       </c>
@@ -33743,10 +33567,14 @@
       </c>
       <c r="I315" t="inlineStr">
         <is>
-          <t>30000 33001 35000 41000 41100</t>
-        </is>
-      </c>
-      <c r="J315" t="inlineStr"/>
+          <t>41000 41100</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>30000 33001 35000</t>
+        </is>
+      </c>
       <c r="L315" t="b">
         <v>0</v>
       </c>
@@ -35017,12 +34845,12 @@
           <t>W 3:00 PM-6:00 PM</t>
         </is>
       </c>
-      <c r="I327" t="inlineStr">
-        <is>
-          <t>41000 41100 35000 34214</t>
-        </is>
-      </c>
-      <c r="J327" t="inlineStr"/>
+      <c r="I327" t="inlineStr"/>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>41000 41100 35000</t>
+        </is>
+      </c>
       <c r="L327" t="b">
         <v>0</v>
       </c>
@@ -35121,10 +34949,14 @@
       </c>
       <c r="I328" t="inlineStr">
         <is>
-          <t>30000 33001 35000 41000 41100</t>
-        </is>
-      </c>
-      <c r="J328" t="inlineStr"/>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>30000 33001 41000 41100</t>
+        </is>
+      </c>
       <c r="K328" t="inlineStr">
         <is>
           <t>Finance</t>
@@ -35222,10 +35054,14 @@
       </c>
       <c r="I329" t="inlineStr">
         <is>
-          <t>30000 33001 35000 41000 41100</t>
-        </is>
-      </c>
-      <c r="J329" t="inlineStr"/>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>30000 33001 41000 41100</t>
+        </is>
+      </c>
       <c r="K329" t="inlineStr">
         <is>
           <t>Finance</t>
@@ -35328,10 +35164,14 @@
       </c>
       <c r="I330" t="inlineStr">
         <is>
-          <t>30000 33001 35000 41000 41100</t>
-        </is>
-      </c>
-      <c r="J330" t="inlineStr"/>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>30000 33001 41000 41100</t>
+        </is>
+      </c>
       <c r="K330" t="inlineStr">
         <is>
           <t>Finance</t>
@@ -35440,10 +35280,14 @@
       </c>
       <c r="I331" t="inlineStr">
         <is>
-          <t>30000 33001 35000 41000 41100</t>
-        </is>
-      </c>
-      <c r="J331" t="inlineStr"/>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>30000 33001 41000 41100</t>
+        </is>
+      </c>
       <c r="K331" t="inlineStr">
         <is>
           <t>Finance</t>
@@ -35552,10 +35396,14 @@
       </c>
       <c r="I332" t="inlineStr">
         <is>
-          <t>30000 33001 35000 41000 41100</t>
-        </is>
-      </c>
-      <c r="J332" t="inlineStr"/>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>30000 33001 41000 41100</t>
+        </is>
+      </c>
       <c r="K332" t="inlineStr">
         <is>
           <t>Finance</t>
@@ -35664,10 +35512,14 @@
       </c>
       <c r="I333" t="inlineStr">
         <is>
-          <t>30000 33001 35000 41000 41100</t>
-        </is>
-      </c>
-      <c r="J333" t="inlineStr"/>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>30000 33001 41000 41100</t>
+        </is>
+      </c>
       <c r="K333" t="inlineStr">
         <is>
           <t>Finance</t>
@@ -35776,10 +35628,14 @@
       </c>
       <c r="I334" t="inlineStr">
         <is>
-          <t>30000 33001 35000 41000 41100</t>
-        </is>
-      </c>
-      <c r="J334" t="inlineStr"/>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>30000 33001 41000 41100</t>
+        </is>
+      </c>
       <c r="K334" t="inlineStr">
         <is>
           <t>Finance</t>
@@ -35888,10 +35744,14 @@
       </c>
       <c r="I335" t="inlineStr">
         <is>
-          <t>30000 33001 35000 41000 41100</t>
-        </is>
-      </c>
-      <c r="J335" t="inlineStr"/>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>30000 33001 41000 41100</t>
+        </is>
+      </c>
       <c r="K335" t="inlineStr">
         <is>
           <t>Finance</t>
@@ -36000,10 +35860,14 @@
       </c>
       <c r="I336" t="inlineStr">
         <is>
-          <t>30000 33001 35000 41000 41100</t>
-        </is>
-      </c>
-      <c r="J336" t="inlineStr"/>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>30000 33001 41000 41100</t>
+        </is>
+      </c>
       <c r="K336" t="inlineStr">
         <is>
           <t>Finance</t>
@@ -36107,10 +35971,14 @@
       </c>
       <c r="I337" t="inlineStr">
         <is>
-          <t>30000 33001 35000 41000 41100</t>
-        </is>
-      </c>
-      <c r="J337" t="inlineStr"/>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>30000 33001 41000 41100</t>
+        </is>
+      </c>
       <c r="K337" t="inlineStr">
         <is>
           <t>Finance</t>
@@ -36213,10 +36081,14 @@
       </c>
       <c r="I338" t="inlineStr">
         <is>
-          <t>30000 33001 35000 41000 41100</t>
-        </is>
-      </c>
-      <c r="J338" t="inlineStr"/>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>30000 33001 41000 41100</t>
+        </is>
+      </c>
       <c r="K338" t="inlineStr">
         <is>
           <t>Finance</t>
@@ -36325,10 +36197,14 @@
       </c>
       <c r="I339" t="inlineStr">
         <is>
-          <t>30000 33001 35000 41000 41100</t>
-        </is>
-      </c>
-      <c r="J339" t="inlineStr"/>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>30000 33001 41000 41100</t>
+        </is>
+      </c>
       <c r="K339" t="inlineStr">
         <is>
           <t>Finance</t>
@@ -36437,7 +36313,7 @@
       </c>
       <c r="I340" t="inlineStr">
         <is>
-          <t>35000 35200 35901 35902 35010</t>
+          <t>35000 35010 35200 35901 35902</t>
         </is>
       </c>
       <c r="J340" t="inlineStr"/>
@@ -36549,7 +36425,7 @@
       </c>
       <c r="I341" t="inlineStr">
         <is>
-          <t>35000 35200 35901 35902 35010</t>
+          <t>35000 35010 35200 35901 35902</t>
         </is>
       </c>
       <c r="J341" t="inlineStr"/>
@@ -36661,7 +36537,7 @@
       </c>
       <c r="I342" t="inlineStr">
         <is>
-          <t>35000 35200 35901 35902 35010</t>
+          <t>35000 35010 35200 35901 35902</t>
         </is>
       </c>
       <c r="J342" t="inlineStr"/>
@@ -36773,7 +36649,7 @@
       </c>
       <c r="I343" t="inlineStr">
         <is>
-          <t>35000 35200 35901 35902 35010</t>
+          <t>35000 35010 35200 35901 35902</t>
         </is>
       </c>
       <c r="J343" t="inlineStr"/>
@@ -36885,7 +36761,7 @@
       </c>
       <c r="I344" t="inlineStr">
         <is>
-          <t>35000 35200 35901 35902 35010</t>
+          <t>35000 35010 35200 35901 35902</t>
         </is>
       </c>
       <c r="J344" t="inlineStr"/>
@@ -36995,12 +36871,12 @@
           <t>TH 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I345" t="inlineStr">
+      <c r="I345" t="inlineStr"/>
+      <c r="J345" t="inlineStr">
         <is>
           <t>33001 35200</t>
         </is>
       </c>
-      <c r="J345" t="inlineStr"/>
       <c r="L345" t="b">
         <v>0</v>
       </c>
@@ -37102,12 +36978,12 @@
           <t>S 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I346" t="inlineStr">
+      <c r="I346" t="inlineStr"/>
+      <c r="J346" t="inlineStr">
         <is>
           <t>33001 35200</t>
         </is>
       </c>
-      <c r="J346" t="inlineStr"/>
       <c r="L346" t="b">
         <v>0</v>
       </c>
@@ -37204,12 +37080,12 @@
           <t>Rajan, Raghuram</t>
         </is>
       </c>
-      <c r="I347" t="inlineStr">
+      <c r="I347" t="inlineStr"/>
+      <c r="J347" t="inlineStr">
         <is>
           <t>35200 35201 30130 34101 35902</t>
         </is>
       </c>
-      <c r="J347" t="inlineStr"/>
       <c r="K347" t="inlineStr">
         <is>
           <t>Finance</t>
@@ -37316,12 +37192,12 @@
           <t>W 6:00 PM-9:00 PM</t>
         </is>
       </c>
-      <c r="I348" t="inlineStr">
+      <c r="I348" t="inlineStr"/>
+      <c r="J348" t="inlineStr">
         <is>
           <t>35200 35201 30130 34101 35902</t>
         </is>
       </c>
-      <c r="J348" t="inlineStr"/>
       <c r="K348" t="inlineStr">
         <is>
           <t>Finance</t>
@@ -37538,7 +37414,7 @@
       <c r="I350" t="inlineStr"/>
       <c r="J350" t="inlineStr">
         <is>
-          <t>30000 33001 41000 41100 35000 35200 35214 35824 35224</t>
+          <t>30000 33001 41000 41100 35000 35200</t>
         </is>
       </c>
       <c r="K350" t="inlineStr">
@@ -37650,7 +37526,7 @@
       <c r="I351" t="inlineStr"/>
       <c r="J351" t="inlineStr">
         <is>
-          <t>30000 33001 41000 41100 35000 35200 35214 35824 35224</t>
+          <t>30000 33001 41000 41100 35000 35200</t>
         </is>
       </c>
       <c r="K351" t="inlineStr">
@@ -38370,11 +38246,7 @@
         </is>
       </c>
       <c r="I358" t="inlineStr"/>
-      <c r="J358" t="inlineStr">
-        <is>
-          <t>35600 55600</t>
-        </is>
-      </c>
+      <c r="J358" t="inlineStr"/>
       <c r="L358" t="b">
         <v>0</v>
       </c>
@@ -38477,11 +38349,7 @@
         </is>
       </c>
       <c r="I359" t="inlineStr"/>
-      <c r="J359" t="inlineStr">
-        <is>
-          <t>35600 55600</t>
-        </is>
-      </c>
+      <c r="J359" t="inlineStr"/>
       <c r="L359" t="b">
         <v>0</v>
       </c>
@@ -38584,11 +38452,7 @@
         </is>
       </c>
       <c r="I360" t="inlineStr"/>
-      <c r="J360" t="inlineStr">
-        <is>
-          <t>35600 55600</t>
-        </is>
-      </c>
+      <c r="J360" t="inlineStr"/>
       <c r="L360" t="b">
         <v>0</v>
       </c>
@@ -39187,12 +39051,12 @@
           <t>M 1:20 PM-4:20 PM</t>
         </is>
       </c>
-      <c r="I366" t="inlineStr">
-        <is>
-          <t>35916 36330 42540</t>
-        </is>
-      </c>
-      <c r="J366" t="inlineStr"/>
+      <c r="I366" t="inlineStr"/>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>42540</t>
+        </is>
+      </c>
       <c r="L366" t="b">
         <v>0</v>
       </c>
@@ -39295,11 +39159,7 @@
         </is>
       </c>
       <c r="I367" t="inlineStr"/>
-      <c r="J367" t="inlineStr">
-        <is>
-          <t>35930 49700</t>
-        </is>
-      </c>
+      <c r="J367" t="inlineStr"/>
       <c r="L367" t="b">
         <v>0</v>
       </c>
@@ -39402,11 +39262,7 @@
         </is>
       </c>
       <c r="I368" t="inlineStr"/>
-      <c r="J368" t="inlineStr">
-        <is>
-          <t>35930 49700</t>
-        </is>
-      </c>
+      <c r="J368" t="inlineStr"/>
       <c r="L368" t="b">
         <v>0</v>
       </c>
@@ -39509,11 +39365,7 @@
         </is>
       </c>
       <c r="I369" t="inlineStr"/>
-      <c r="J369" t="inlineStr">
-        <is>
-          <t>35931 49800</t>
-        </is>
-      </c>
+      <c r="J369" t="inlineStr"/>
       <c r="L369" t="b">
         <v>0</v>
       </c>
@@ -39616,11 +39468,7 @@
         </is>
       </c>
       <c r="I370" t="inlineStr"/>
-      <c r="J370" t="inlineStr">
-        <is>
-          <t>35931 49800</t>
-        </is>
-      </c>
+      <c r="J370" t="inlineStr"/>
       <c r="L370" t="b">
         <v>0</v>
       </c>
@@ -39723,11 +39571,7 @@
         </is>
       </c>
       <c r="I371" t="inlineStr"/>
-      <c r="J371" t="inlineStr">
-        <is>
-          <t>35932 49900</t>
-        </is>
-      </c>
+      <c r="J371" t="inlineStr"/>
       <c r="L371" t="b">
         <v>0</v>
       </c>
@@ -39830,11 +39674,7 @@
         </is>
       </c>
       <c r="I372" t="inlineStr"/>
-      <c r="J372" t="inlineStr">
-        <is>
-          <t>35932 49900</t>
-        </is>
-      </c>
+      <c r="J372" t="inlineStr"/>
       <c r="L372" t="b">
         <v>0</v>
       </c>
@@ -42080,7 +41920,7 @@
       </c>
       <c r="I393" t="inlineStr">
         <is>
-          <t>36110 20550</t>
+          <t>20550 36110</t>
         </is>
       </c>
       <c r="J393" t="inlineStr"/>
@@ -43108,11 +42948,7 @@
         </is>
       </c>
       <c r="I403" t="inlineStr"/>
-      <c r="J403" t="inlineStr">
-        <is>
-          <t>37000 20600</t>
-        </is>
-      </c>
+      <c r="J403" t="inlineStr"/>
       <c r="K403" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -43209,11 +43045,7 @@
         </is>
       </c>
       <c r="I404" t="inlineStr"/>
-      <c r="J404" t="inlineStr">
-        <is>
-          <t>37000 20600</t>
-        </is>
-      </c>
+      <c r="J404" t="inlineStr"/>
       <c r="K404" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -43315,11 +43147,7 @@
         </is>
       </c>
       <c r="I405" t="inlineStr"/>
-      <c r="J405" t="inlineStr">
-        <is>
-          <t>37000 20600</t>
-        </is>
-      </c>
+      <c r="J405" t="inlineStr"/>
       <c r="K405" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -43427,11 +43255,7 @@
         </is>
       </c>
       <c r="I406" t="inlineStr"/>
-      <c r="J406" t="inlineStr">
-        <is>
-          <t>37000 20600</t>
-        </is>
-      </c>
+      <c r="J406" t="inlineStr"/>
       <c r="K406" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -43539,11 +43363,7 @@
         </is>
       </c>
       <c r="I407" t="inlineStr"/>
-      <c r="J407" t="inlineStr">
-        <is>
-          <t>37000 20600</t>
-        </is>
-      </c>
+      <c r="J407" t="inlineStr"/>
       <c r="K407" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -43651,11 +43471,7 @@
         </is>
       </c>
       <c r="I408" t="inlineStr"/>
-      <c r="J408" t="inlineStr">
-        <is>
-          <t>37000 20600</t>
-        </is>
-      </c>
+      <c r="J408" t="inlineStr"/>
       <c r="K408" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -43763,11 +43579,7 @@
         </is>
       </c>
       <c r="I409" t="inlineStr"/>
-      <c r="J409" t="inlineStr">
-        <is>
-          <t>37000 20600</t>
-        </is>
-      </c>
+      <c r="J409" t="inlineStr"/>
       <c r="K409" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -43875,11 +43687,7 @@
         </is>
       </c>
       <c r="I410" t="inlineStr"/>
-      <c r="J410" t="inlineStr">
-        <is>
-          <t>37000 20600</t>
-        </is>
-      </c>
+      <c r="J410" t="inlineStr"/>
       <c r="K410" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -43987,11 +43795,7 @@
         </is>
       </c>
       <c r="I411" t="inlineStr"/>
-      <c r="J411" t="inlineStr">
-        <is>
-          <t>37000 20600</t>
-        </is>
-      </c>
+      <c r="J411" t="inlineStr"/>
       <c r="K411" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -44099,11 +43903,7 @@
         </is>
       </c>
       <c r="I412" t="inlineStr"/>
-      <c r="J412" t="inlineStr">
-        <is>
-          <t>37000 20600</t>
-        </is>
-      </c>
+      <c r="J412" t="inlineStr"/>
       <c r="K412" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -44211,11 +44011,7 @@
         </is>
       </c>
       <c r="I413" t="inlineStr"/>
-      <c r="J413" t="inlineStr">
-        <is>
-          <t>37000 20600</t>
-        </is>
-      </c>
+      <c r="J413" t="inlineStr"/>
       <c r="K413" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -44323,11 +44119,7 @@
         </is>
       </c>
       <c r="I414" t="inlineStr"/>
-      <c r="J414" t="inlineStr">
-        <is>
-          <t>37000 20600</t>
-        </is>
-      </c>
+      <c r="J414" t="inlineStr"/>
       <c r="K414" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -44435,11 +44227,7 @@
         </is>
       </c>
       <c r="I415" t="inlineStr"/>
-      <c r="J415" t="inlineStr">
-        <is>
-          <t>37000 20600</t>
-        </is>
-      </c>
+      <c r="J415" t="inlineStr"/>
       <c r="K415" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -44547,11 +44335,7 @@
         </is>
       </c>
       <c r="I416" t="inlineStr"/>
-      <c r="J416" t="inlineStr">
-        <is>
-          <t>37000 20600</t>
-        </is>
-      </c>
+      <c r="J416" t="inlineStr"/>
       <c r="K416" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -44659,11 +44443,7 @@
         </is>
       </c>
       <c r="I417" t="inlineStr"/>
-      <c r="J417" t="inlineStr">
-        <is>
-          <t>37000 20600</t>
-        </is>
-      </c>
+      <c r="J417" t="inlineStr"/>
       <c r="K417" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -44771,11 +44551,7 @@
         </is>
       </c>
       <c r="I418" t="inlineStr"/>
-      <c r="J418" t="inlineStr">
-        <is>
-          <t>37000 20600</t>
-        </is>
-      </c>
+      <c r="J418" t="inlineStr"/>
       <c r="K418" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -45666,11 +45442,7 @@
           <t>W 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I426" t="inlineStr">
-        <is>
-          <t>37103 37105 20620</t>
-        </is>
-      </c>
+      <c r="I426" t="inlineStr"/>
       <c r="J426" t="inlineStr">
         <is>
           <t>37000 37100 41000 41100</t>
@@ -45784,7 +45556,7 @@
       </c>
       <c r="I427" t="inlineStr">
         <is>
-          <t>41000 41100 37105 37103 20620</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="J427" t="inlineStr"/>
@@ -45892,7 +45664,7 @@
       <c r="I428" t="inlineStr"/>
       <c r="J428" t="inlineStr">
         <is>
-          <t>37000 37201 37200 37810</t>
+          <t>37000</t>
         </is>
       </c>
       <c r="K428" t="inlineStr">
@@ -45993,7 +45765,7 @@
       <c r="I429" t="inlineStr"/>
       <c r="J429" t="inlineStr">
         <is>
-          <t>37000 37201 37200 37810</t>
+          <t>37000</t>
         </is>
       </c>
       <c r="K429" t="inlineStr">
@@ -46094,7 +45866,7 @@
       <c r="I430" t="inlineStr"/>
       <c r="J430" t="inlineStr">
         <is>
-          <t>37000 37201 37200 37810</t>
+          <t>37000</t>
         </is>
       </c>
       <c r="K430" t="inlineStr">
@@ -46195,7 +45967,7 @@
       <c r="I431" t="inlineStr"/>
       <c r="J431" t="inlineStr">
         <is>
-          <t>37000 37201 37200 37810</t>
+          <t>37000</t>
         </is>
       </c>
       <c r="K431" t="inlineStr">
@@ -46296,7 +46068,7 @@
       <c r="I432" t="inlineStr"/>
       <c r="J432" t="inlineStr">
         <is>
-          <t>37000 37201 37200 37810</t>
+          <t>37000</t>
         </is>
       </c>
       <c r="K432" t="inlineStr">
@@ -48022,12 +47794,12 @@
           <t>S 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I448" t="inlineStr">
+      <c r="I448" t="inlineStr"/>
+      <c r="J448" t="inlineStr">
         <is>
           <t>37000</t>
         </is>
       </c>
-      <c r="J448" t="inlineStr"/>
       <c r="K448" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -48432,11 +48204,7 @@
         </is>
       </c>
       <c r="I452" t="inlineStr"/>
-      <c r="J452" t="inlineStr">
-        <is>
-          <t>37904 40902</t>
-        </is>
-      </c>
+      <c r="J452" t="inlineStr"/>
       <c r="L452" t="b">
         <v>0</v>
       </c>
@@ -55813,11 +55581,7 @@
           <t>T 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I522" t="inlineStr">
-        <is>
-          <t>38916 41175</t>
-        </is>
-      </c>
+      <c r="I522" t="inlineStr"/>
       <c r="J522" t="inlineStr"/>
       <c r="L522" t="b">
         <v>0</v>
@@ -55921,11 +55685,7 @@
         </is>
       </c>
       <c r="I523" t="inlineStr"/>
-      <c r="J523" t="inlineStr">
-        <is>
-          <t>38917 41120</t>
-        </is>
-      </c>
+      <c r="J523" t="inlineStr"/>
       <c r="L523" t="b">
         <v>0</v>
       </c>
@@ -56027,11 +55787,7 @@
           <t>TH 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I524" t="inlineStr">
-        <is>
-          <t>39001</t>
-        </is>
-      </c>
+      <c r="I524" t="inlineStr"/>
       <c r="J524" t="inlineStr"/>
       <c r="K524" t="inlineStr">
         <is>
@@ -56139,11 +55895,7 @@
           <t>S 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I525" t="inlineStr">
-        <is>
-          <t>39001</t>
-        </is>
-      </c>
+      <c r="I525" t="inlineStr"/>
       <c r="J525" t="inlineStr"/>
       <c r="K525" t="inlineStr">
         <is>
@@ -56253,7 +56005,7 @@
       </c>
       <c r="I526" t="inlineStr">
         <is>
-          <t>42001 39001</t>
+          <t>39001 42001</t>
         </is>
       </c>
       <c r="J526" t="inlineStr"/>
@@ -56365,7 +56117,7 @@
       </c>
       <c r="I527" t="inlineStr">
         <is>
-          <t>42001 39001</t>
+          <t>39001 42001</t>
         </is>
       </c>
       <c r="J527" t="inlineStr"/>
@@ -56477,7 +56229,7 @@
       </c>
       <c r="I528" t="inlineStr">
         <is>
-          <t>42001 39001</t>
+          <t>39001 42001</t>
         </is>
       </c>
       <c r="J528" t="inlineStr"/>
@@ -56589,7 +56341,7 @@
       </c>
       <c r="I529" t="inlineStr">
         <is>
-          <t>42001 39001</t>
+          <t>39001 42001</t>
         </is>
       </c>
       <c r="J529" t="inlineStr"/>
@@ -56700,11 +56452,7 @@
         </is>
       </c>
       <c r="I530" t="inlineStr"/>
-      <c r="J530" t="inlineStr">
-        <is>
-          <t>40000 20500</t>
-        </is>
-      </c>
+      <c r="J530" t="inlineStr"/>
       <c r="K530" t="inlineStr">
         <is>
           <t>Operations</t>
@@ -56812,11 +56560,7 @@
         </is>
       </c>
       <c r="I531" t="inlineStr"/>
-      <c r="J531" t="inlineStr">
-        <is>
-          <t>40000 20500</t>
-        </is>
-      </c>
+      <c r="J531" t="inlineStr"/>
       <c r="K531" t="inlineStr">
         <is>
           <t>Operations</t>
@@ -56924,11 +56668,7 @@
         </is>
       </c>
       <c r="I532" t="inlineStr"/>
-      <c r="J532" t="inlineStr">
-        <is>
-          <t>40000 20500</t>
-        </is>
-      </c>
+      <c r="J532" t="inlineStr"/>
       <c r="K532" t="inlineStr">
         <is>
           <t>Operations</t>
@@ -57036,11 +56776,7 @@
         </is>
       </c>
       <c r="I533" t="inlineStr"/>
-      <c r="J533" t="inlineStr">
-        <is>
-          <t>40000 20500</t>
-        </is>
-      </c>
+      <c r="J533" t="inlineStr"/>
       <c r="K533" t="inlineStr">
         <is>
           <t>Operations</t>
@@ -57143,11 +56879,7 @@
         </is>
       </c>
       <c r="I534" t="inlineStr"/>
-      <c r="J534" t="inlineStr">
-        <is>
-          <t>40000 20500</t>
-        </is>
-      </c>
+      <c r="J534" t="inlineStr"/>
       <c r="K534" t="inlineStr">
         <is>
           <t>Operations</t>
@@ -57244,11 +56976,7 @@
         </is>
       </c>
       <c r="I535" t="inlineStr"/>
-      <c r="J535" t="inlineStr">
-        <is>
-          <t>40000 20500</t>
-        </is>
-      </c>
+      <c r="J535" t="inlineStr"/>
       <c r="K535" t="inlineStr">
         <is>
           <t>Operations</t>
@@ -57350,11 +57078,7 @@
         </is>
       </c>
       <c r="I536" t="inlineStr"/>
-      <c r="J536" t="inlineStr">
-        <is>
-          <t>40000 20500</t>
-        </is>
-      </c>
+      <c r="J536" t="inlineStr"/>
       <c r="K536" t="inlineStr">
         <is>
           <t>Operations</t>
@@ -57462,11 +57186,7 @@
         </is>
       </c>
       <c r="I537" t="inlineStr"/>
-      <c r="J537" t="inlineStr">
-        <is>
-          <t>40000 20500</t>
-        </is>
-      </c>
+      <c r="J537" t="inlineStr"/>
       <c r="K537" t="inlineStr">
         <is>
           <t>Operations</t>
@@ -57574,11 +57294,7 @@
         </is>
       </c>
       <c r="I538" t="inlineStr"/>
-      <c r="J538" t="inlineStr">
-        <is>
-          <t>40000 20500</t>
-        </is>
-      </c>
+      <c r="J538" t="inlineStr"/>
       <c r="K538" t="inlineStr">
         <is>
           <t>Operations</t>
@@ -58650,12 +58366,12 @@
           <t>TH 2:00 PM-5:00 PM</t>
         </is>
       </c>
-      <c r="I548" t="inlineStr">
-        <is>
-          <t>40206 40205 40201 40721</t>
-        </is>
-      </c>
-      <c r="J548" t="inlineStr"/>
+      <c r="I548" t="inlineStr"/>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>40721</t>
+        </is>
+      </c>
       <c r="L548" t="b">
         <v>1</v>
       </c>
@@ -58757,12 +58473,12 @@
           <t>TH 6:00 PM-9:00 PM</t>
         </is>
       </c>
-      <c r="I549" t="inlineStr">
-        <is>
-          <t>40206 40205 40201 40721</t>
-        </is>
-      </c>
-      <c r="J549" t="inlineStr"/>
+      <c r="I549" t="inlineStr"/>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>40721</t>
+        </is>
+      </c>
       <c r="L549" t="b">
         <v>1</v>
       </c>
@@ -58867,7 +58583,7 @@
       <c r="I550" t="inlineStr"/>
       <c r="J550" t="inlineStr">
         <is>
-          <t>40206 40721 41201 41100 41204 40000 30001 36106 32100</t>
+          <t>40206 41201 41100 41204 40000 30001 36106 32100</t>
         </is>
       </c>
       <c r="L550" t="b">
@@ -62059,11 +61775,7 @@
         </is>
       </c>
       <c r="I580" t="inlineStr"/>
-      <c r="J580" t="inlineStr">
-        <is>
-          <t>41600 51400</t>
-        </is>
-      </c>
+      <c r="J580" t="inlineStr"/>
       <c r="L580" t="b">
         <v>0</v>
       </c>
@@ -62166,11 +61878,7 @@
         </is>
       </c>
       <c r="I581" t="inlineStr"/>
-      <c r="J581" t="inlineStr">
-        <is>
-          <t>41600 51400</t>
-        </is>
-      </c>
+      <c r="J581" t="inlineStr"/>
       <c r="L581" t="b">
         <v>0</v>
       </c>
@@ -62273,11 +61981,7 @@
         </is>
       </c>
       <c r="I582" t="inlineStr"/>
-      <c r="J582" t="inlineStr">
-        <is>
-          <t>41600 51400</t>
-        </is>
-      </c>
+      <c r="J582" t="inlineStr"/>
       <c r="L582" t="b">
         <v>0</v>
       </c>
@@ -62382,7 +62086,7 @@
       <c r="I583" t="inlineStr"/>
       <c r="J583" t="inlineStr">
         <is>
-          <t>41901 32400</t>
+          <t>32400</t>
         </is>
       </c>
       <c r="K583" t="inlineStr">
@@ -62718,7 +62422,7 @@
       <c r="I586" t="inlineStr"/>
       <c r="J586" t="inlineStr">
         <is>
-          <t>41901 41910 33500</t>
+          <t>41901 33500</t>
         </is>
       </c>
       <c r="K586" t="inlineStr">
@@ -62935,12 +62639,12 @@
           <t>F 1:30 PM-4:30 PM</t>
         </is>
       </c>
-      <c r="I588" t="inlineStr">
-        <is>
-          <t>41919 32419</t>
-        </is>
-      </c>
-      <c r="J588" t="inlineStr"/>
+      <c r="I588" t="inlineStr"/>
+      <c r="J588" t="inlineStr">
+        <is>
+          <t>32419</t>
+        </is>
+      </c>
       <c r="L588" t="b">
         <v>0</v>
       </c>
@@ -64712,11 +64416,7 @@
         </is>
       </c>
       <c r="I604" t="inlineStr"/>
-      <c r="J604" t="inlineStr">
-        <is>
-          <t>42005</t>
-        </is>
-      </c>
+      <c r="J604" t="inlineStr"/>
       <c r="L604" t="b">
         <v>0</v>
       </c>
@@ -66724,11 +66424,7 @@
           <t>T 8:30 AM-11:30 AM</t>
         </is>
       </c>
-      <c r="I623" t="inlineStr">
-        <is>
-          <t>42136 42125 20930</t>
-        </is>
-      </c>
+      <c r="I623" t="inlineStr"/>
       <c r="J623" t="inlineStr"/>
       <c r="K623" t="inlineStr">
         <is>
@@ -69837,7 +69533,7 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="37" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
     <col width="80" customWidth="1" min="9" max="9"/>
   </cols>
@@ -69965,7 +69661,7 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>30000 33001 41000 41100 20101 30001</t>
+          <t>30000 33001 41000 41100</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -70017,7 +69713,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>30000 30116 20140</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -70059,7 +69755,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>30000 35200 20170</t>
+          <t>30000 35200</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -70113,7 +69809,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>30000 20160 30835</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -70160,12 +69856,12 @@
       <c r="F7" t="b">
         <v>0</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
         <is>
           <t>30000 30130 30116 30118 30131</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr">
         <is>
           <t>In previous accounting/financial analysis courses, you obtained skills important
@@ -70223,14 +69919,10 @@
       <c r="F8" t="b">
         <v>0</v>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>30130 30000 35200</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>35000 20150</t>
+          <t>30000 35200 35000 20150</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -70492,11 +70184,7 @@
         <v>0</v>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>30122</t>
-        </is>
-      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
           <t>There are many forms of “structures” in a deal such as financial structure, tax
@@ -70837,7 +70525,7 @@
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>31001 31403 31404</t>
+          <t>31001 31404</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -70931,11 +70619,7 @@
       <c r="F25" t="b">
         <v>0</v>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>31407 31404</t>
-        </is>
-      </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" s="2" t="inlineStr">
         <is>
@@ -71185,11 +70869,7 @@
       <c r="F29" t="b">
         <v>0</v>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>43100 43800</t>
-        </is>
-      </c>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" s="2" t="inlineStr">
         <is>
@@ -71306,12 +70986,12 @@
       <c r="F32" t="b">
         <v>0</v>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
         <is>
           <t>33001</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" s="2" t="inlineStr">
         <is>
           <t>This course examines foundational topics in human resource management
@@ -71352,7 +71032,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>33001 33050 33040 20200</t>
+          <t>33001</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -71839,11 +71519,7 @@
       <c r="F43" t="b">
         <v>0</v>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>33401 20232</t>
-        </is>
-      </c>
+      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
       <c r="I43" s="2" t="inlineStr">
         <is>
@@ -71987,7 +71663,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>20940 33471</t>
+          <t>20940</t>
         </is>
       </c>
       <c r="H46" t="inlineStr"/>
@@ -72047,12 +71723,12 @@
       <c r="F47" t="b">
         <v>0</v>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
         <is>
           <t>33001</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
       <c r="I47" s="2" t="inlineStr">
         <is>
           <t>SCHEDULE
@@ -72099,7 +71775,7 @@
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
-          <t>33050 33502 20230</t>
+          <t>33050</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
@@ -72180,11 +71856,7 @@
         <v>0</v>
       </c>
       <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>33610 54300</t>
-        </is>
-      </c>
+      <c r="H50" t="inlineStr"/>
       <c r="I50" s="2" t="inlineStr">
         <is>
           <t>Workshops in each academic area provide a forum for faculty, PhD students,
@@ -72211,11 +71883,7 @@
         <v>0</v>
       </c>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>33630 53000</t>
-        </is>
-      </c>
+      <c r="H51" t="inlineStr"/>
       <c r="I51" s="2" t="inlineStr">
         <is>
           <t>Workshops in each academic area provide a forum for faculty, PhD students,
@@ -72242,11 +71910,7 @@
         <v>0</v>
       </c>
       <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>33650 57000</t>
-        </is>
-      </c>
+      <c r="H52" t="inlineStr"/>
       <c r="I52" s="2" t="inlineStr">
         <is>
           <t>Workshops in each academic area provide a forum for faculty, PhD students,
@@ -72353,11 +72017,7 @@
       <c r="F56" t="b">
         <v>0</v>
       </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>33914 30680</t>
-        </is>
-      </c>
+      <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
       <c r="I56" s="2" t="inlineStr">
         <is>
@@ -72418,7 +72078,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>33001 33101 33002 30000 30100 30200</t>
+          <t>30100 30200 33001 33002 33101</t>
         </is>
       </c>
       <c r="H58" t="inlineStr"/>
@@ -72452,7 +72112,7 @@
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
-          <t>33001 33002 33101 30000 30100 30200 33921 40101</t>
+          <t>33001 33002 33101 30000 30100 30200</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
@@ -72486,7 +72146,7 @@
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
-          <t>33921 33922 40201</t>
+          <t>33921</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
@@ -72524,7 +72184,7 @@
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
-          <t>33921 33922 33923 40301</t>
+          <t>33921 33922</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
@@ -72597,7 +72257,7 @@
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>33931 30540 30100 30200 30300</t>
+          <t>30200 30300</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -72658,11 +72318,7 @@
         <v>0</v>
       </c>
       <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>33942 38001</t>
-        </is>
-      </c>
+      <c r="H65" t="inlineStr"/>
       <c r="I65" s="2" t="inlineStr">
         <is>
           <t>This course considers the use of data on households, workers and producers
@@ -72701,11 +72357,7 @@
         <v>0</v>
       </c>
       <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>33946 35101</t>
-        </is>
-      </c>
+      <c r="H66" t="inlineStr"/>
       <c r="I66" s="2" t="inlineStr">
         <is>
           <t>This is a graduate course in international trade. It introduces the fundamental
@@ -72743,7 +72395,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>35200 35201 35902 34106 30130</t>
+          <t>30130 34106 35200 35201 35902</t>
         </is>
       </c>
       <c r="H67" t="inlineStr"/>
@@ -72829,11 +72481,7 @@
         <v>0</v>
       </c>
       <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>34103 20330</t>
-        </is>
-      </c>
+      <c r="H69" t="inlineStr"/>
       <c r="I69" s="2" t="inlineStr">
         <is>
           <t>Course Description
@@ -73048,11 +72696,7 @@
       <c r="F73" t="b">
         <v>0</v>
       </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>20355 34887</t>
-        </is>
-      </c>
+      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
@@ -73347,12 +72991,12 @@
       <c r="F79" t="b">
         <v>0</v>
       </c>
-      <c r="G79" t="inlineStr">
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr">
         <is>
           <t>34211</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
       <c r="I79" s="2" t="inlineStr">
         <is>
           <t>Course Description and Learning Objectives: 
@@ -73526,12 +73170,12 @@
       <c r="F83" t="b">
         <v>0</v>
       </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>34101 34219 34209</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>34101</t>
+        </is>
+      </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
           <t>WHAT YOU LEARN
@@ -73905,11 +73549,7 @@
         <v>0</v>
       </c>
       <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>20350</t>
-        </is>
-      </c>
+      <c r="H90" t="inlineStr"/>
       <c r="I90" s="2" t="inlineStr">
         <is>
           <t>Entrepreneurial success is built with passion, execution, and leadership;
@@ -73989,11 +73629,7 @@
       <c r="F91" t="b">
         <v>0</v>
       </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>34709 34706</t>
-        </is>
-      </c>
+      <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr"/>
       <c r="I91" s="2" t="inlineStr">
         <is>
@@ -74082,7 +73718,7 @@
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
-          <t>34715 53455 33830 32002</t>
+          <t>33830 32002</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr">
@@ -74257,10 +73893,14 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>34901 35904 31000 31100 31200 33000 33100 33200 34902 35060</t>
-        </is>
-      </c>
-      <c r="H97" t="inlineStr"/>
+          <t>34901 35904</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>31100 31200 33100 33200</t>
+        </is>
+      </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
           <t>This course builds on Asset Pricing I. The course focuses on empirical asset
@@ -74306,11 +73946,7 @@
       <c r="F98" t="b">
         <v>0</v>
       </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>30100 30200 30300 34903 35070</t>
-        </is>
-      </c>
+      <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr"/>
       <c r="I98" s="2" t="inlineStr">
         <is>
@@ -74352,7 +73988,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>34903 35902 34904 35080</t>
+          <t>34903 35902</t>
         </is>
       </c>
       <c r="H99" t="inlineStr"/>
@@ -74389,7 +74025,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>34903 34904 34906 35090</t>
+          <t>34903 34904</t>
         </is>
       </c>
       <c r="H100" t="inlineStr"/>
@@ -74433,7 +74069,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>41000 41100 35000 20400</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -74476,11 +74112,7 @@
       <c r="F102" t="b">
         <v>0</v>
       </c>
-      <c r="G102" t="inlineStr">
-        <is>
-          <t>35001 35010</t>
-        </is>
-      </c>
+      <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr">
         <is>
           <t>30000</t>
@@ -74518,12 +74150,12 @@
       <c r="F103" t="b">
         <v>0</v>
       </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>30000 35010 35001</t>
-        </is>
-      </c>
-      <c r="H103" t="inlineStr"/>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>30000</t>
+        </is>
+      </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
           <t>This course introduces students to corporate finance, asset pricing, and
@@ -74618,7 +74250,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>41000 35000 35200</t>
+          <t>35000 35200 41000</t>
         </is>
       </c>
       <c r="H105" t="inlineStr"/>
@@ -74708,12 +74340,12 @@
       <c r="F107" t="b">
         <v>0</v>
       </c>
-      <c r="G107" t="inlineStr">
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr">
         <is>
           <t>35000 41100 35215</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
       <c r="I107" s="2" t="inlineStr">
         <is>
           <t>SCHEDULE
@@ -74756,10 +74388,14 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>30000 33001 35000 41000 41100</t>
-        </is>
-      </c>
-      <c r="H108" t="inlineStr"/>
+          <t>41000 41100</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>30000 33001 35000</t>
+        </is>
+      </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
           <t>This course develops a framework to build and analyze quantitative
@@ -75180,12 +74816,12 @@
       <c r="F117" t="b">
         <v>0</v>
       </c>
-      <c r="G117" t="inlineStr">
-        <is>
-          <t>41000 41100 35000 34214</t>
-        </is>
-      </c>
-      <c r="H117" t="inlineStr"/>
+      <c r="G117" t="inlineStr"/>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>41000 41100 35000</t>
+        </is>
+      </c>
       <c r="I117" s="2" t="inlineStr">
         <is>
           <t>COURSE OVERVIEW
@@ -75228,10 +74864,14 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>30000 33001 35000 41000 41100</t>
-        </is>
-      </c>
-      <c r="H118" t="inlineStr"/>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>30000 33001 41000 41100</t>
+        </is>
+      </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
           <t>This course analyzes the major decisions facing corporate financial managers.
@@ -75282,7 +74922,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>35000 35200 35901 35902 35010</t>
+          <t>35000 35010 35200 35901 35902</t>
         </is>
       </c>
       <c r="H119" t="inlineStr"/>
@@ -75328,12 +74968,12 @@
       <c r="F120" t="b">
         <v>0</v>
       </c>
-      <c r="G120" t="inlineStr">
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr">
         <is>
           <t>33001 35200</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr"/>
       <c r="I120" s="2" t="inlineStr">
         <is>
           <t>Consumer finance is ubiquitous. The US, for example, carries more consumer
@@ -75373,12 +75013,12 @@
       <c r="F121" t="b">
         <v>0</v>
       </c>
-      <c r="G121" t="inlineStr">
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr">
         <is>
           <t>35200 35201 30130 34101 35902</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr"/>
       <c r="I121" s="2" t="inlineStr">
         <is>
           <t>This course will explore the challenges of corporate finance and investment in
@@ -75481,7 +75121,7 @@
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr">
         <is>
-          <t>30000 33001 41000 41100 35000 35200 35214 35824 35224</t>
+          <t>30000 33001 41000 41100 35000 35200</t>
         </is>
       </c>
       <c r="I123" s="2" t="inlineStr">
@@ -75732,11 +75372,7 @@
         <v>0</v>
       </c>
       <c r="G129" t="inlineStr"/>
-      <c r="H129" t="inlineStr">
-        <is>
-          <t>35600 55600</t>
-        </is>
-      </c>
+      <c r="H129" t="inlineStr"/>
       <c r="I129" s="2" t="inlineStr">
         <is>
           <t>Workshops in each academic area provide a forum for faculty, PhD students,
@@ -75911,12 +75547,12 @@
       <c r="F134" t="b">
         <v>0</v>
       </c>
-      <c r="G134" t="inlineStr">
-        <is>
-          <t>35916 36330 42540</t>
-        </is>
-      </c>
-      <c r="H134" t="inlineStr"/>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>42540</t>
+        </is>
+      </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
           <t>This course provides graduate-level discussion of topics and methods in public
@@ -75958,11 +75594,7 @@
         <v>0</v>
       </c>
       <c r="G135" t="inlineStr"/>
-      <c r="H135" t="inlineStr">
-        <is>
-          <t>35930 49700</t>
-        </is>
-      </c>
+      <c r="H135" t="inlineStr"/>
       <c r="I135" s="2" t="inlineStr">
         <is>
           <t>PhD research seminar for third year students in both Finance and the joint
@@ -75991,11 +75623,7 @@
         <v>0</v>
       </c>
       <c r="G136" t="inlineStr"/>
-      <c r="H136" t="inlineStr">
-        <is>
-          <t>35931 49800</t>
-        </is>
-      </c>
+      <c r="H136" t="inlineStr"/>
       <c r="I136" s="2" t="inlineStr">
         <is>
           <t>PhD research seminar for third year students in both Finance and the joint
@@ -76024,11 +75652,7 @@
         <v>0</v>
       </c>
       <c r="G137" t="inlineStr"/>
-      <c r="H137" t="inlineStr">
-        <is>
-          <t>35932 49900</t>
-        </is>
-      </c>
+      <c r="H137" t="inlineStr"/>
       <c r="I137" s="2" t="inlineStr">
         <is>
           <t>PhD research seminar for third year students in both Finance and the joint
@@ -76268,7 +75892,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>36110 20550</t>
+          <t>20550 36110</t>
         </is>
       </c>
       <c r="H141" t="inlineStr"/>
@@ -76552,11 +76176,7 @@
         <v>0</v>
       </c>
       <c r="G149" t="inlineStr"/>
-      <c r="H149" t="inlineStr">
-        <is>
-          <t>37000 20600</t>
-        </is>
-      </c>
+      <c r="H149" t="inlineStr"/>
       <c r="I149" s="2" t="inlineStr">
         <is>
           <t>I use a framework-based approach to teach this course. The first half of the
@@ -76653,11 +76273,7 @@
       <c r="F151" t="b">
         <v>0</v>
       </c>
-      <c r="G151" t="inlineStr">
-        <is>
-          <t>37103 37105 20620</t>
-        </is>
-      </c>
+      <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr">
         <is>
           <t>37000 37100 41000 41100</t>
@@ -76719,7 +76335,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>41000 41100 37105 37103 20620</t>
+          <t>41000 41100</t>
         </is>
       </c>
       <c r="H152" t="inlineStr"/>
@@ -76784,7 +76400,7 @@
       <c r="G153" t="inlineStr"/>
       <c r="H153" t="inlineStr">
         <is>
-          <t>37000 37201 37200 37810</t>
+          <t>37000</t>
         </is>
       </c>
       <c r="I153" s="2" t="inlineStr">
@@ -77114,12 +76730,12 @@
       <c r="F160" t="b">
         <v>1</v>
       </c>
-      <c r="G160" t="inlineStr">
+      <c r="G160" t="inlineStr"/>
+      <c r="H160" t="inlineStr">
         <is>
           <t>37000</t>
         </is>
       </c>
-      <c r="H160" t="inlineStr"/>
       <c r="I160" s="2" t="inlineStr">
         <is>
           <t>Companies today expect their marketing professionals to understand what it
@@ -77263,11 +76879,7 @@
         <v>0</v>
       </c>
       <c r="G164" t="inlineStr"/>
-      <c r="H164" t="inlineStr">
-        <is>
-          <t>37904 40902</t>
-        </is>
-      </c>
+      <c r="H164" t="inlineStr"/>
       <c r="I164" s="2" t="inlineStr">
         <is>
           <t>This course covers some key topics at the research frontier in quantitative
@@ -78171,11 +77783,7 @@
       <c r="F186" t="b">
         <v>0</v>
       </c>
-      <c r="G186" t="inlineStr">
-        <is>
-          <t>38916 41175</t>
-        </is>
-      </c>
+      <c r="G186" t="inlineStr"/>
       <c r="H186" t="inlineStr"/>
       <c r="I186" s="2" t="inlineStr">
         <is>
@@ -78215,11 +77823,7 @@
         <v>0</v>
       </c>
       <c r="G187" t="inlineStr"/>
-      <c r="H187" t="inlineStr">
-        <is>
-          <t>38917 41120</t>
-        </is>
-      </c>
+      <c r="H187" t="inlineStr"/>
       <c r="I187" s="2" t="inlineStr">
         <is>
           <t>This class covers recent work in behavioral economics. Topics include social
@@ -78259,11 +77863,7 @@
       <c r="F188" t="b">
         <v>0</v>
       </c>
-      <c r="G188" t="inlineStr">
-        <is>
-          <t>39001</t>
-        </is>
-      </c>
+      <c r="G188" t="inlineStr"/>
       <c r="H188" t="inlineStr"/>
       <c r="I188" s="2" t="inlineStr">
         <is>
@@ -78321,7 +77921,7 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>42001 39001</t>
+          <t>39001 42001</t>
         </is>
       </c>
       <c r="H189" t="inlineStr"/>
@@ -78372,11 +77972,7 @@
         <v>0</v>
       </c>
       <c r="G190" t="inlineStr"/>
-      <c r="H190" t="inlineStr">
-        <is>
-          <t>40000 20500</t>
-        </is>
-      </c>
+      <c r="H190" t="inlineStr"/>
       <c r="I190" s="2" t="inlineStr">
         <is>
           <t>This core course focuses on the levers for structuring, managing, and
@@ -78602,12 +78198,12 @@
       <c r="F195" t="b">
         <v>1</v>
       </c>
-      <c r="G195" t="inlineStr">
-        <is>
-          <t>40206 40205 40201 40721</t>
-        </is>
-      </c>
-      <c r="H195" t="inlineStr"/>
+      <c r="G195" t="inlineStr"/>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>40721</t>
+        </is>
+      </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
           <t>One of the today's most exciting and important applications of Business
@@ -78671,7 +78267,7 @@
       <c r="G196" t="inlineStr"/>
       <c r="H196" t="inlineStr">
         <is>
-          <t>40206 40721 41201 41100 41204 40000 30001 36106 32100</t>
+          <t>40206 41201 41100 41204 40000 30001 36106 32100</t>
         </is>
       </c>
       <c r="I196" s="2" t="inlineStr">
@@ -79081,11 +78677,7 @@
         <v>0</v>
       </c>
       <c r="G205" t="inlineStr"/>
-      <c r="H205" t="inlineStr">
-        <is>
-          <t>41600 51400</t>
-        </is>
-      </c>
+      <c r="H205" t="inlineStr"/>
       <c r="I205" s="2" t="inlineStr">
         <is>
           <t>Workshops in each academic area provide a forum for faculty, PhD students,
@@ -79123,7 +78715,7 @@
       <c r="G206" t="inlineStr"/>
       <c r="H206" t="inlineStr">
         <is>
-          <t>41901 32400</t>
+          <t>32400</t>
         </is>
       </c>
       <c r="I206" s="2" t="inlineStr">
@@ -79256,7 +78848,7 @@
       <c r="G209" t="inlineStr"/>
       <c r="H209" t="inlineStr">
         <is>
-          <t>41901 41910 33500</t>
+          <t>41901 33500</t>
         </is>
       </c>
       <c r="I209" s="2" t="inlineStr">
@@ -79330,12 +78922,12 @@
       <c r="F211" t="b">
         <v>0</v>
       </c>
-      <c r="G211" t="inlineStr">
-        <is>
-          <t>41919 32419</t>
-        </is>
-      </c>
-      <c r="H211" t="inlineStr"/>
+      <c r="G211" t="inlineStr"/>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>32419</t>
+        </is>
+      </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
           <t>This is a course on advanced Bayesian inference in the context of
@@ -79439,11 +79031,7 @@
         <v>0</v>
       </c>
       <c r="G213" t="inlineStr"/>
-      <c r="H213" t="inlineStr">
-        <is>
-          <t>42005</t>
-        </is>
-      </c>
+      <c r="H213" t="inlineStr"/>
       <c r="I213" s="2" t="inlineStr">
         <is>
           <t>Using timeless stories and characters as case studies can illuminate leadership
@@ -80002,11 +79590,7 @@
       <c r="F224" t="b">
         <v>0</v>
       </c>
-      <c r="G224" t="inlineStr">
-        <is>
-          <t>42136 42125 20930</t>
-        </is>
-      </c>
+      <c r="G224" t="inlineStr"/>
       <c r="H224" t="inlineStr"/>
       <c r="I224" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix CLO=unavailable pricing, truncated descriptions, missing schedules
- CLO availability: a section closed in round 1 with no clearing price (CLO @ 0)
  is now 'unavailable', not free. New students (Y1) use the New-Students seats
  column, returning (Y2) use Phase 1. Placed cards and the section picker show
  'Unavailable' instead of a misleading 0/price; unavailable cost is excluded
  from the quarter spend. (e.g. 43120 & 32210 Winter are unavailable for Y1.)
- Descriptions: extract from the left text column (two-column catalog layout)
  so long descriptions are no longer truncated by the schedule interleaving
  (truncated-looking 67 -> 15).
- Schedule: fall back to the bid 'Day and Time' when the catalog lacks one;
  parser now handles full weekday names (e.g. 'Wednesday, 08:30 am - 11:30 am').
</commit_message>
<xml_diff>
--- a/build/curriculum.xlsx
+++ b/build/curriculum.xlsx
@@ -1295,6 +1295,11 @@
           <t>Heltzer, Wendy</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Tuesday, 08:30 am - 11:30 am</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
@@ -1722,6 +1727,11 @@
           <t>Le, Anthony</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Thursday, 6:00 pm - 9:00 pm</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
@@ -10876,7 +10886,7 @@
       <c r="I101" t="inlineStr"/>
       <c r="J101" t="inlineStr"/>
       <c r="L101" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M101" t="b">
         <v>0</v>
@@ -10973,7 +10983,7 @@
       <c r="I102" t="inlineStr"/>
       <c r="J102" t="inlineStr"/>
       <c r="L102" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M102" t="b">
         <v>0</v>
@@ -12090,6 +12100,11 @@
           <t>Misra, Sanjog</t>
         </is>
       </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Wednesday, 08:30 am - 11:30 am</t>
+        </is>
+      </c>
       <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr"/>
       <c r="L113" t="b">
@@ -12188,6 +12203,11 @@
           <t>Campos, Christopher</t>
         </is>
       </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Monday, 08:30 am - 11:30 am</t>
+        </is>
+      </c>
       <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr"/>
       <c r="K114" t="inlineStr">
@@ -20710,6 +20730,11 @@
           <t>Hsieh, Chang-Tai</t>
         </is>
       </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Saturday, 1:30 pm - 4:30 pm</t>
+        </is>
+      </c>
       <c r="I193" t="inlineStr"/>
       <c r="J193" t="inlineStr">
         <is>
@@ -20920,6 +20945,11 @@
           <t>Conway, Jacob; Kamenica, Emir</t>
         </is>
       </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Wednesday, 01:20 pm - 02:50 pm</t>
+        </is>
+      </c>
       <c r="I195" t="inlineStr"/>
       <c r="J195" t="inlineStr"/>
       <c r="L195" t="b">
@@ -22682,6 +22712,11 @@
           <t>Richert, Eric</t>
         </is>
       </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>Thursday,Tuesday, 09:30 am - 10:50 am</t>
+        </is>
+      </c>
       <c r="I212" t="inlineStr"/>
       <c r="J212" t="inlineStr">
         <is>
@@ -26724,6 +26759,11 @@
           <t>Parrish, Priya</t>
         </is>
       </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>Thursday, 1:30 pm - 4:30 pm</t>
+        </is>
+      </c>
       <c r="I251" t="inlineStr"/>
       <c r="J251" t="inlineStr"/>
       <c r="K251" t="inlineStr">
@@ -29495,7 +29535,7 @@
       <c r="I278" t="inlineStr"/>
       <c r="J278" t="inlineStr"/>
       <c r="L278" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M278" t="b">
         <v>0</v>
@@ -37080,6 +37120,11 @@
           <t>Rajan, Raghuram</t>
         </is>
       </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>Thursday, 08:30 am - 11:30 am</t>
+        </is>
+      </c>
       <c r="I347" t="inlineStr"/>
       <c r="J347" t="inlineStr">
         <is>
@@ -37628,6 +37673,11 @@
       <c r="G352" t="inlineStr">
         <is>
           <t>Vishny, Robert</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>Thursday, 01:30 pm - 04:30 pm</t>
         </is>
       </c>
       <c r="I352" t="inlineStr"/>
@@ -52833,6 +52883,11 @@
           <t>Wu, George</t>
         </is>
       </c>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>Thursday, 08:30 am - 11:30 am</t>
+        </is>
+      </c>
       <c r="I496" t="inlineStr">
         <is>
           <t>38103</t>
@@ -66751,7 +66806,7 @@
       <c r="I626" t="inlineStr"/>
       <c r="J626" t="inlineStr"/>
       <c r="L626" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M626" t="b">
         <v>0</v>
@@ -69666,9 +69721,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>SCHEDULE
-INTERNAL INFORMATION FOR STRATEGIC DECISIONS (30005) - HANNA, J.&gt;&gt;
-We develop your ability to analyze the economic costs of important
+          <t>We develop your ability to analyze the economic costs of important
 decisions within a firm. These decisions include make vs. buy, abandon vs.
 continue, setting transfer prices, and evaluating employee performance, to
 name a few. When you leave the course, you will understand key costing
@@ -69726,7 +69779,30 @@
 which financial statements are produced. It will benefit students that want to
 become bankers, investors, analysts, or any other job that requires more than
 a superficial understanding of financial reporting. The course is also a good
-replacement for B30000 for MBA students that have already taken an</t>
+replacement for B30000 for MBA students that have already taken an
+introductory accounting class (the online pre-MBA accounting class is a great
+preparation for the class).
+We will not limit our study to the financial statements per se. We will also work
+with supplemental disclosures, which help the user to interpret the financial
+statements and to understand better the economic transactions that gave rise
+to them. The techniques we will employ will be useful for variety of purposes
+including (but not limited to) equity, credit, and complex deals (such as MA)
+analysis. Although this course does not cover forecasting, valuation, or models
+of complex deals, a thorough understanding of financial reporting issues is
+critical to being able to use such techniques. As a result, this course will be
+especially useful as a prelude to Financial Statement Analysis (B30130),
+Advanced Financial Analysis and Valuation for Global Firms (B30131), and Deal
+Structuring and Financial Reporting Implications (B30122).
+Topics covered typically include: pro forma financial statements; convertible
+instruments; EPS; stock-based compensation accounting; accounting for
+investments; accounting for income taxes; lease accounting; foreign currency
+translation. Where significant, differences between US GAAP and international
+standards (IFRS) will be highlighted.
+Class discussions will draw from actual financial statements. Answers to five
+cases based on actual financial statements must be submitted. There will be
+two in-person exams (Weeks 5 and 10).
+The course is also likely to prove useful to those preparing to take the CFA or
+CPA exams.</t>
         </is>
       </c>
     </row>
@@ -69888,7 +69964,16 @@
 investments.
 Main topics to be covered include: (1) Financial Reporting and Tax implications
 of influence and control situations; (2) Financial reporting and Tax Implications
-of M&amp;A deals; (3) Financial reporting and tax implications for restructuring via</t>
+of M&amp;A deals; (3) Financial reporting and tax implications for restructuring via
+sales, spin-offs, and equity carve-outs; (4) Financial reporting implications and
+Tax implications for distressed firms operating in bankruptcy and emerging
+from bankruptcy (5) Building Merger Consequences and Restructuring models
+to evaluate the feasibility of deals. Here is a video introduction for the course.
+1st Class Assignment is mandatory. It requires you to build a statement of cash
+flows. It is available here.  Note that if it is your responsibility to submit the 1st
+class assignment even if you are not registered for the course by the 1st day of
+class but intend to do so. You may submit it via email to me or to the teaching
+assistant.</t>
         </is>
       </c>
     </row>
@@ -69961,7 +70046,13 @@
 proximity to financial distress.
 [6]   Sensibly Forecast Full Sets of Financial Statements.  Learn how to sensibly
 construct full sets of forecasted financial statements in order to arrive at
-economically well-founded quantitative answers to financing, investing or</t>
+economically well-founded quantitative answers to financing, investing or
+valuation questions.  Know how to avoid the errors and dubious judgments
+Wall Street analysts often make when they forecast financial statements.
+[7]   Sensibly Value a Firm and Its Equity.  Learn how good FSAV can help you
+arrive at sensible DCF + multiples measures of enterprise and equity value. 
+Recognize and avoid the errors and dubious economic judgments that
+managers &amp; Wall Street analysts make when they do DCF valuations.</t>
         </is>
       </c>
     </row>
@@ -70157,7 +70248,33 @@
 id=56fa8c00-49ac-4b5d-8e4c-b41f00eb791f
 This course provides the core set of tools and strategies related to the work of
 a Chief Financial Officer (CFO) at a private, entrepreneurial company as well as
-to the work of those who provide funding to the company, work for the</t>
+to the work of those who provide funding to the company, work for the
+company, or are founders of the company. The course follows the life-cycle of
+a company that begins as a start-up, and covers the accounting-related
+financial metrics, and the managerial, financial and tax accounting issues that
+are centrally important for an entrepreneur in the private firm environment.
+We will cover topics relevant at the earliest stages of a business, such as setting
+up the initial accounting infrastructure, through to the growth stage (including
+the role of Generative AI in aiding rapid scaling with fewer employees), and
+finally to the company’s exit. The exit would typically be to a strategic buyer, a
+private equity firm or via an IPO, Direct Listing, or SPAC. The course will be of
+particular interest to those who may become start-up founders or key
+employees as well as to those who may invest in early stage firms.
+Selected topics:
+Setting up the initial infrastructure for the information system used by a
+start-up, including tracking the equity capitalization (i.e., the capitalization
+table).
+Structuring and accounting for equity based employee compensation, for
+founders and employees.
+Reporting key performance indicators to the company, the board of
+directors and investors such as venture capital and private equity funds.
+Issues to consider during the growth phase, including the role of GenAI in
+aiding rapid scaling with fewer employees.
+Sale process, working capital adjustment, and roll-over equity for a
+management team.
+Accounting and applying for debt as a private company, such as bank
+debt, venture debt, and account receivable lines of credit.
+Accounting information required for a fundraising process.</t>
         </is>
       </c>
     </row>
@@ -70207,7 +70324,10 @@
 Main topics to be covered include: (1) Financial Reporting and Tax implications
 of influence and control situations; (2) Financial reporting and Tax Implications
 of M&amp;A deals; (3) Financial reporting and tax implications for restructuring via
-sales, spin-offs, and equity carve-outs; (4) Financial reporting implications and</t>
+sales, spin-offs, and equity carve-outs; (4) Financial reporting implications and
+Tax implications for distressed firms operating in bankruptcy and emerging
+from bankruptcy (5) Building Merger Consequences and Restructuring models
+to evaluate the feasibility of deals. Here is a video introduction for the course.</t>
         </is>
       </c>
     </row>
@@ -70491,7 +70611,58 @@
 order to present yourself such that others’ perceptions more accurately reflect
 what you intend.
 • To identify your emotions and how to utilize them as an important source of
-information and guide to your interpersonal choices.</t>
+information and guide to your interpersonal choices.
+• To navigate the emotions of others and learn how to be more aware of and
+sensitive to them.
+• To identify the widely varied and equally valuable leadership roles that
+emerge in the life of a group.
+Improving personal knowledge and abilities in these areas is crucial to
+becoming a more effective manager in today’s increasingly complex, diverse,
+international and exceedingly inter-dependent business climate.
+Commitment
+Because of the highly interactive nature of this course, it is essential that all
+students make a commitment to the course from the beginning and attend all
+sessions. Course shopping is actively discouraged. If you attend the first class
+and decide not to return, you have robbed another student of the opportunity
+to take the course, as we cannot backfill a spot after the first class meeting.
+Failure to attend the first class will result in an automatic drop.
+Scheduling Details
+Attendance at each 3-hour class, as well as at a residential weekend intensive
+retreat (off-site), is required. Attendance at this retreat, in its entirety, is
+mandatory and non-negotiable.  Several meetings with a small group of fellow
+students outside of class will also be required throughout the quarter.
+Enrollment in the course is by application
+Apply online. The application period opens on Monday February 2, 2026 at
+9:00am. Applications are due by ­Sunday February 8, 2026 at 11:59 pm. You will
+be notified of your enrollment status no later than Monday February 16, 2026
+at 5:00 pm. The more sections you indicate you can commit to, the better your
+chances of landing a spot. But please do not include sections that you cannot
+completely commit to or that you would prefer not to attend. An invitation to a
+section is for that section only. There is no section swapping once you are
+offered a spot.
+Format and Course Materials
+The format of the class will include discussion, experiential exercises, small-
+group support meetings outside of class, short lectures, T-Group and the
+retreat weekend. There is one required text for this class (see "Materials"), and
+links to all other course readings will be included in the syllabus.
+Autumn 2023 Information Session
+An in-person information session for this class may be offered but has yet to
+be scheduled.  In the meantime, please use this link to view a previous session:
+View recording of Spring 2020 Info Session.
+Spring Section Specifics
+Weekly class:
+Section 04: Wednesdays 8:30 am - 11:30 am. All classes take place at
+Harper.
+Section 05: Wednesdays 1:30 am - 4:30 am. All classes take place at
+Harper.
+Weekend Intensive Retreat: This is a mandatory, off-site retreat.
+Transportation, meals and lodging are all provided. The Friday session begins
+at 6:45 pm (allow for travel time and dinner); Sunday session ends at 12:30 pm.
+Section 04: Friday, May 8 through Sunday, May 10.
+Section 05: Friday, May 15 through Sunday, May 17.
+Small Group Meetings: Students will meet in small subgroups up to four times
+throughout the quarter. These meetings are to be scheduled at mutually
+agreeable times by the students.</t>
         </is>
       </c>
     </row>
@@ -70538,7 +70709,53 @@
 2. I am my best when I play my roles as my authentic-self. I can experiment
 and adopt new leadership qualities that are rooted in my personal values.
 3. I am self-driven. I take personal responsibility for doing the work and
-expanding my leadership qualities.</t>
+expanding my leadership qualities.
+4. I will continue work on my leadership behaviors into the future. I put in
+place good habits for ongoing development/learning following the work
+started in The Leadership Studio.
+During the Studio, each student builds upon their current leadership strengths
+and learns how to harness many more of their leadership qualities and
+abilities. They gain greater confidence in their ability to have the impact they
+desire and to continue growing and evolving as they face new demands as
+leaders. To this end, the Leadership Studio explores leadership from nine
+perspectives. These provide valuable inputs for a leadership journey that is
+truly actionable and lasting.
+This work is accomplished through a learning environment built upon three
+interwoven tracks:
+Exposure to research and new knowledge in a Classroom track
+Applying knowledge and leadership goals in a Rehearsal Hall track
+Experiments with enhancing leadership skills in a Fieldwork track.
+The class is not recorded to keep it as a safe place for experimenting and
+sharing. Students must attend in person: there is no Zoom participation
+allowance.  Because of the high participation requirement of the class,
+students are required to put away laptops, tablets, and smart phones for all
+Rehearsal Hall sessions. 
+We have assembled a teaching ensemble drawn from different areas of
+expertise that will remain involved in supporting students throughout the
+quarter. This team consists of academics, practitioners from the worlds of
+business, music, theater and improv, as well as coaches who bring a
+disciplined, scientific methodology to ongoing practice.
+Attention! This is not a class in which faculty and students play traditional, well-
+defined roles. They will instead be co-creating the experience. Students should
+sign up for the Studio if they are committed to their own personal
+development with learning tailored to each person.
+Four comments from students who have completed the course may be
+instructive:
+“The Studio will teach you two things, which can have a lasting impact in your
+life: a) A framework for self improvement based on trying new things, collecting
+data and reflecting; and b) The notion that you can be flexible on the personal
+qualities you will draw on for each situation.”
+“This is a class that goes beyond business. It impacts every aspect of life. It is
+an essential course to take to be an effective leader and learn how to become
+one.”
+“It is what you put into it. This can be a profound experience for some, and
+useless for others who do not take it seriously.”
+“Unlike any Booth class I’ve taken, you must be ready to be fully present and
+ready to make a real change in your behavior.”
+Given the experiential nature of the Leadership Studio, please view a recording
+of the information session held Friday, February 13 at 12:00pm CST to provide
+more insights into the Studio experience. You will hear from a former student
+along with three members of the teaching and coaching team.</t>
         </is>
       </c>
     </row>
@@ -70558,7 +70775,7 @@
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
@@ -70566,7 +70783,63 @@
         <is>
           <t>As a leader there are few things more vital to your success and fulfillment than
 the ability to grow as you encounter new challenges or become aware of
-outdated patterns of behaviors.</t>
+outdated patterns of behaviors.
+The principal goal of this course is to learn how to guide your own
+development and make personal change. This ability is a form of self-
+leadership and is one of the foundations of a rewarding career and a
+meaningful life. The benefits of this class are twofold.
+The first benefit is that you will define and make progress on a personal
+development goal of your choosing.
+Most of us harbor a list of things we would like to work on and change about
+ourselves. We often carry these desires for years without making much
+progress. This class creates a space in which you can finally realize your desires
+for growth and change. A sample of development goals Booth students’ have
+identified includes:
+Leaning into disagreements and conflict with others rather than avoiding
+Developing a stronger, more self-assured interpersonal presence
+Reworking interpersonal habits that derail interactions with others
+Developing habits and skills that enable more easily and comfortably
+connecting with others
+Managing one’s reactions and frustrations that get in the way of working
+effectively with others
+The second benefit is that you will learn a set of ideas and tactics for guiding
+your development in the future.
+As you work on your own development goal, you will apply approaches
+introduced in class. These approaches are designed to help you make progress
+on their current development goals; and, these same approaches are portable
+so that you can also apply them to future development goals, long after the
+course is over. Some of the approaches covered in class include:
+Taking stock of your most pressing development needs
+Engaging your thoughts, emotions, and behaviors to create actionable
+development goals
+Reworking ineffective patterns of behavior
+Dealing with your own resistance to making desired change
+Initiating and sustaining action over time to make progress
+It is important to note that Leadership Lab requires a deeper level of
+engagement than many classes.
+Broadly speaking, the focus of the course concerns human development and
+introduces a valuable set of ideas on this topic. Yet, the heart of the class
+concerns the ways in which you apply these ideas to yourself. The class
+consists of activities, assignments, and interactions that involve analyzing your
+desires for yourself, better understanding what others need from you, learning
+to work with your own thoughts and emotions, generating meaningful goals
+for yourself, on-going effort to make desired changes, and supporting your
+fellow classmates as they engage in the same kind of work. The personal
+nature of the work we do in this class relies on a willingness to try difficult
+things, to be vulnerable, and to take responsibility for your own development.
+Curriculum Video
+View video for more details about the course. Note: CNet credentials required
+to view.
+Enrollment in the course is by application
+Apply online here. The application period open is now open. Please submit
+your application by end of day on Sunday, February 19. You will be notified of
+your enrollment status on Tuesday, February 21st.
+Format
+The format of the class will include in-class discussion, experiential exercises,
+and short lectures. One of the most important parts of class are the
+assignments in between classes which involve experimenting with new
+behaviors in ways that may feel unfamiliar and/or challenging. Both are
+considered essential parts of the class experience.</t>
         </is>
       </c>
     </row>
@@ -70597,7 +70870,30 @@
 students who want to align who they are with how they lead—without
 sacrificing credibility, coherence, or performance. Designed for complex, high-
 stakes environments, the course integrates personal values, social identity, and
-behavioral data into a disciplined and strategic leadership decision framework.</t>
+behavioral data into a disciplined and strategic leadership decision framework.
+Drawing on behavioral science, values-based assessments (Hogan MVPI), and
+experiential learning, students learn to ALIGN before they lead:
+·       A — Assess: Examine values, motives, identity data, and behavioral
+drivers.
+·       L — Locate: Identify the structural dynamics, incentives, risks, and
+performance expectations shaping the moment.
+·       I — Interrogate:: Surface mental models, defaults, blind spots, and
+assumptions.
+·       G — Generate Signal: Determine what leadership stance to take, what to
+disclose or withhold, and how to act in alignment with both identity and
+context.
+·       N — Navigate: Make a deliberate leadership choice informed by both
+identity and context.
+Through professionally led table coaching, structured feedback, and narrative-
+based reflection (including podcast-based assignments), students translate
+self-insight into disciplined action—emphasizing decision-making and
+execution in environments shaped by competing expectations and real-world
+constraint.
+By the end of the course, students produce an ALIGN Strategy Portfolio—a
+cohesive body of work integrating leadership identity, peer feedback,
+contextual analysis, and a structured 90-day implementation plan designed for
+immediate application in their workplace, internships, entrepreneurial
+ventures, or professional transitions.</t>
         </is>
       </c>
     </row>
@@ -70668,7 +70964,12 @@
 classmates as they engage in the same kind of work. The personal nature of
 the work we do in this class relies on a willingness to try difficult things, to be
 vulnerable, and to take responsibility for your own development.
-Format</t>
+Format
+The format of the class will include in-class discussion, experiential exercises,
+and short lectures. One of the most important parts of class are the
+assignments in between classes which involve experimenting with new
+behaviors in ways that may feel unfamiliar and/or challenging. Both are
+considered essential parts of the class experience.</t>
         </is>
       </c>
     </row>
@@ -70706,7 +71007,34 @@
 lack of equity and the widening wealth gap in America's most vulnerable
 neighborhoods.
 Aided by current social, political and economic constructs, developers
-contribute to gentrification through large investments that build structures,</t>
+contribute to gentrification through large investments that build structures,
+not opportunity. The result is generations of residents being displaced rapidly -
+-the same residents that contributed to the culture and economic success that
+makes development in a location so appealing.
+This course involves an in-depth exploration and analyses of the above
+conditions and how we can work to develop a new reality in real estate
+development, one that does not displace people and values diversity and
+inclusion in order to create healthy communities. To start, to develop without
+displacement sufficient housing must be available for existing residents. One
+possible solution, and the one that is the focus of this class, is to assemble
+adjacent parcels so that new taller and denser development can be
+constructed. Admittedly not without its own controversies, this scenario
+envisions new residential units designed to meet the needs of existing
+residents and owners, as well as providing additional workforce housing and
+adding market-rate renters. Existing landowners can enter their properties into
+long-term leases with the developer ensuring a continual income stream while
+retaining ownership of the property. In addition to housing options, these
+developments offer ground floor retail that provide amenities for residents
+and contribute to neighborhood vibrancy and diversity. An influx of population
+can support new retail and increase available jobs. In this way development
+can be a catalyst that benefits all members of the neighborhood.
+Inner-city neighborhoods have become increasingly desirable to developers
+and to a range of new urban residents. In order to make the resulting
+development work for everyone, creative strategies must be developed that
+minimize displacement and that share benefits. Inner city revitalization is
+challenging, but through intentional strategic development and planning,
+members of marginalized communities can gain access to resources to join the
+ranks of start-up developers and take leadership roles in the process.</t>
         </is>
       </c>
     </row>
@@ -70767,7 +71095,9 @@
 Learning Outcomes: 
 1. Write basic code in Python and SQL to carry out fundamental data analysis
 tasks like data import, data cleaning, and data visualization
-2. Prompt ChatGPT and similar genAI tools to optimize your coding workflow</t>
+2. Prompt ChatGPT and similar genAI tools to optimize your coding workflow 
+3. Define data analytics fundamentals to enable you to talk intelligently with
+programmers and analysts on your team</t>
         </is>
       </c>
     </row>
@@ -70843,7 +71173,14 @@
 temporal elements to your data, through the use of maps and dynamic
 dashboards in Tableau, can be the difference between data that sits on the
 page and data that moves your audience to action.
-How are customers reacting to your ad spend, and can you make changes to</t>
+How are customers reacting to your ad spend, and can you make changes to
+your allocations more quickly to take advantage of fluctuating trends in real
+time? What’s driving customer churn, and what interventions are working right
+now? Is your bank being targeted by bad actors in a coordinated fraud
+scheme? How is your portfolio performing in real-time in relation to your risk
+metrics? Are your manufacturing processes on track, or are cost overruns and
+production delays imminent? Data visualization can improve your answers to
+all of these questions.</t>
         </is>
       </c>
     </row>
@@ -70874,7 +71211,24 @@
       <c r="I29" s="2" t="inlineStr">
         <is>
           <t>Generative AI is a pivotal advancement in the realm of artificial intelligence that
-has the potential to transform various industries, from entertainment and</t>
+has the potential to transform various industries, from entertainment and
+advertising to healthcare and education. A thorough
+understanding of Generative technologies, potential uses cases and the
+implications are going to be necessary conditions of success. This new
+technology can automate content creation, optimize processes,
+and personalize experiences but more broadly it has the capacity to synthesize
+new data, simulate scenarios, generate ideas, and even design novel solutions
+to complex problems., making it a crucial
+technology for managers across all domains.
+This course provides a comprehensive overview of Generative AI, covering its
+foundational technologies, practical applications, and broader societal
+implications. It aims to equip students with a solid
+understanding of Generative AI and its relevance to various fields, as well as
+cultivate critical thinking on the ethical, legal, and societal challenges related to
+its deployment.
+Each class will have a lecture and discussion portion as well as some
+practicum/exercise/demo portion. In addition, there will be a course projects
+where you will work on the development of a Generative AI solution.</t>
         </is>
       </c>
     </row>
@@ -70910,7 +71264,10 @@
       <c r="I30" s="2" t="inlineStr">
         <is>
           <t>This course teaches the core principles of modern microeconomics and
-illustrates their application to understanding business decisions and the</t>
+illustrates their application to understanding business decisions and the
+broader world. The course covers the following topics: supply and demand;
+consumer choice; firm behavior, including pricing and production under
+different market structures; and the effects of uncertainty.</t>
         </is>
       </c>
     </row>
@@ -71134,7 +71491,13 @@
 that studies companies and their behavior. Topics covered include production
 and productivity, pricing, demand estimation, oligopolies, equilibrium market
 structure, antitrust and regulation, vertical integration and contracting,
-strategic behavior, search and advertising, and two-sided markets. The course</t>
+strategic behavior, search and advertising, and two-sided markets. The course
+is aimed at students who are comfortable with at least intermediate-level
+microeconomics, and ideally have already taken 33001 (Microeconomics) or
+equivalent. The course material combines both theoretical and empirical
+elements, and you should be prepared for both abstract and practical
+treatments of issues. The course can also serve as a complement to, but not
+replacement for, 42001 (Competitive Strategy).</t>
         </is>
       </c>
     </row>
@@ -71174,7 +71537,61 @@
 intellectual history of capitalism, sparking active discussion of the challenges
 and opportunities facing capitalist economies today and what "capitalism" can
 and should mean going forward. 
-Course format:</t>
+Course format: 
+The format of the course is atypical. The class will follow two parallel paths.
+First, a diverse group of University of Chicago faculty will be invited to share
+their research and views, supplemented by short readings; they will discuss
+their perspectives on capitalism and its future through the lens of their
+research and areas of expertise. The second path will be that of a seminar
+course, built around readings and discussion. The seminars of 10-15 students
+and a faculty member will be taught by Brian Barry, James Carmichael, Rob
+Gertner, Caroline Grossman, John Paul Rollert, and Susana Vasquez.
+The course is 100-total units, but will be broken up into two course
+numbers/enrollments:
+33250 Perspectives on Capitalism (0 units), meets 90 minutes per week on
+Wednesdays from 5:00-6:30pm in Harper Center C-25.  Lecture format
+with speakers.
+33251 Perspectives on Capitalism Seminar (100 units), meets 90 minutes
+per week.  Small group discussion of readings at a variety of days and
+times at Harper, Gleacher, or remotely. 
+There will be a remote option for the seminar; students are required to attend
+lectures in person unless they are in a remote seminar section.
+Past faculty speakers included: 
+Marianne Bertrand, Chris P. Dialynas Distinguished Service Professor of
+Economics, Chicago Booth
+Agnes Callard, Associate Professor in Philosophy, the College
+Michael Greenstone, Milton Friedman Distinguished Professor in
+Economics, the College and the Harris School 
+Chang-tai Hsieh, Phyllis and Irwin Winkelried Professor of Economics,
+Chicago Booth
+Jonathan Levy, James Westfall Thompson Professor, History, John U. Nef
+Committee on Social Thought, and the Collegue
+Kevin Murphy, George J. Stigler Distinguished Service Professor of
+Economics, Chicago Booth, the College 
+Kenneth Pomeranz, University Professor of Modern Chinese History, the
+College
+Raghuram Rajan, Katherine Dusak Miller Distinguished Service Professor
+of Finance, Chicago Booth
+Richard Thaler, Charles R. Walgreen Distinguished Service Professor of
+Behavioral Science and Economics, Chicago Booth
+Dali Yang, William Claude Reavis Professor, Political Science
+Luigi Zingales, Robert C. McCormack Distinguished Service Professor of
+Entrepreneurship and Finance, Chicago Booth
+Information Session:
+View Info Session Recording from 2/8/24 for more details about the course.
+How to Enroll:
+Perspectives on Capitalism was previously application-based. Effective Spring
+2025, students will bid for the Seminar sections (33251). Students who bid
+successfully for 33251 will automatically be enrolled in 33250 by the Booth
+Registrar. If you are in a remote section of 33251, you will be enrolled in the
+remote section of 33250 and be expected to join the lectures remotely (live or
+asynchronously). If you are in an in-person section of 33251, you will be
+enrolled in the in-person section of 33250 and be required to attend the
+lectures in person.  Students enrolled in an in-person seminar will not be able
+to attend lectures remotely or to watch recordings except by arrangement with
+their seminar instructor, which will only be made in cases of special
+circumstances.   For questions, contact email
+BoothRegistrar@lists.chicagobooth.edu.</t>
         </is>
       </c>
     </row>
@@ -71224,7 +71641,18 @@
 First, a diverse group of University of Chicago faculty will be invited to share
 their research and views, supplemented by short readings; they will discuss
 their perspectives on capitalism and its future through the lens of their
-research and areas of expertise. The second path will be that of a seminar</t>
+research and areas of expertise. The second path will be that of a seminar
+course, built around readings and discussion. The seminars of 10-15 students
+and a faculty member will be taught by Brian Barry, James Carmichael, Rob
+Gertner, Caroline Grossman, and Susana Vasquez.
+The course is 100-total units, but will be broken up into two course
+numbers/enrollments:
+33250 Perspectives on Capitalism (0 units), meets 90 minutes per week on
+Wednesdays from 5:00-6:30pm in Harper Center C-25.  Lecture format
+with speakers.
+33251 Perspectives on Capitalism Seminar (100 units), meets 90 minutes
+per week.  Small group discussion of readings at a variety of days and
+times at Harper, Gleacher, or remotely.</t>
         </is>
       </c>
     </row>
@@ -71278,7 +71706,20 @@
 have sparked debates ranging from intellectual property protection to privacy;
 recent development in the fast-food industry and financial markets have
 triggered intense discussions about new information disclosure and consumer
-protection rules.</t>
+protection rules.
+The main purpose of this course is to better understand the non-market
+environment, and discuss firms’ strategies in light of regulatory, legal, political
+and social constraints that they face. We will discuss the rationales for
+economic regulation and describe the main tools of economic regulation (such
+as the industry conduct regulation of natural monopolies and industrial
+structure regulation imposed by antitrust laws). We also discuss firms’
+strategies in light of environmental, safety, or intellectual property concerns.
+A common thread throughout this course is that we will recognize that firms
+can also shape their non-market environment. In particular, we will discuss
+firms’ lobbying strategies and use tools from political science to guide our
+understanding of the lawmaking and rulemaking process. We will also discuss
+why and how firms may decide to self-regulate in response to activist or media
+pressures.</t>
         </is>
       </c>
     </row>
@@ -71488,7 +71929,10 @@
 targeting, positioning, pricing, and go-to-market strategy apply in the life
 sciences context. We will explore how companies create and sustain
 competitive advantage in markets where customers include patients
-providers, payers, advocacy groups and regulators.</t>
+providers, payers, advocacy groups and regulators.
+A detailed week by week syllabus is available below.  As we go along additional
+readings may be provided and we may modify the class to optimize learning
+objectives.</t>
         </is>
       </c>
     </row>
@@ -71692,7 +72136,13 @@
 also handle criticism from groups who might gain something by weakening a
 firm or industry’s reputation, or by questioning the legitimacy of the
 marketplace in which businesses operate. Critics can include rival firms,
-politicians, workers, pressure groups, journalists, customers and suppliers.</t>
+politicians, workers, pressure groups, journalists, customers and suppliers.
+The quality and accuracy of these groups’ arguments vary, but usually include
+assertions that a business or its leaders are behaving unethically or lack
+legitimacy. The ability to respond to these claims, and counter them effectively
+when the facts and arguments are on your side, is a crucial management skill.
+This is easier to do when you can think through how your assessments relate
+to broader ideas about business and capitalism.</t>
         </is>
       </c>
     </row>
@@ -72415,7 +72865,21 @@
 comprehensive. We will explore private equity from a number of perspectives,
 beginning with the entrepreneur/issuer, moving to private equity - venture
 capital, growth equity and leveraged buyout - partnerships, and finishing with
-investors in private equity partnerships.</t>
+investors in private equity partnerships.
+For each class meeting, study questions will be assigned concerning a case
+study. We will discuss these questions and the material in the case for most of
+the class period. Before each case discussion, each student will be required to
+submit a memorandum (up to two pages) of analysis and recommendations.
+Group work is encouraged, but not required on these short memoranda.
+Memoranda with up to three names on them are acceptable. We will use
+journal articles and some lectures to supplement and enhance the case
+discussions. All required cases and supplementary readings will be posted
+online in Canvas.
+Pre-assignment: Students are responsible for a memorandum for each case
+we discuss in the first class. The first class assignment is detailed in Canvas. All
+students (including those who are not registered, but are trying to add the
+course) must attend and prepare the first week. Students who do not attend
+the first week cannot take the course.</t>
         </is>
       </c>
     </row>
@@ -72454,7 +72918,23 @@
 strategic thinking skills, this course will change how you see new ideas—and
 yourself.
 At the heart of the class are nine battle-tested and tried-and-true strategy
-models and the Four Basic Questions that help you quickly and confidently</t>
+models and the Four Basic Questions that help you quickly and confidently
+assess whether any new venture is worth pursuing. You'll learn how to tell the
+difference between a business that sounds good and one that actually works,
+and how to go about building the latter.
+We'll dive into historical and contemporary case studies, debate what went
+wrong (or brilliantly right), and apply our frameworks through written memos,
+in-class exercises, and a final venture proposal you'll build with a team of your
+peers. Along the way, we'll dissect startups, carve-outs, roll-ups, and venture-
+backed plays with the same critical lens.
+This class isn't about evangelizing entrepreneurship. It's about mastering the
+judgment, discipline, and creative clarity that help great entrepreneurs
+succeed.
+By the end of the course, you'll be able to:
+Evaluate any new venture idea with clear strategic insight
+Design a business with a defensible and compelling value proposition
+Assess the risk and return of a venture for founders and investors
+Present and defend your ideas like a strategist, not a salesperson</t>
         </is>
       </c>
     </row>
@@ -72512,7 +72992,40 @@
 applicable to all types of businesses, whether B2B, B2C or deep technology
 based on fundamental scientific research. YourCo projects range from
 software and digital solutions, to consumer products, to services, to industrial
-applications and beyond.</t>
+applications and beyond. 
+AI is fundamentally changing how ventures are built, enabling founders and
+teams to move faster, test ideas more efficiently, and build products with fewer
+resources. As such, the use of AI tools is encouraged throughout this course.
+As part of the YourCo assignment and class discussions, students will explore
+how AI can be used to accelerate customer discovery, refine positioning and
+messaging, develop investor pitch materials, and support decision-making.
+Please note that students are expected to use AI responsibly and thoughtfully,
+applying their own judgment, critical thinking, and domain insight when
+evaluating and refining AI-generated outputs.
+Students will have the unique opportunity to engage with distinguished guest
+entrepreneurs and investors who will share their firsthand experiences in
+building and scaling businesses. These guest speakers bring real-world
+insights, offering perspectives that complement and enrich the course
+material. By interacting with successful founders and industry leaders,
+students will gain a deeper understanding of the challenges, opportunities,
+and decision-making processes that shape entrepreneurial ventures. These
+sessions provide a rare chance to ask questions, seek mentorship, and build
+connections with seasoned professionals. Historically, students have found this
+component of the course to be immensely valuable, as it brings theoretical
+concepts to life in a way that no textbook or lecture alone can.
+Students will also have the opportunity to practice the art of fundraising in a
+supportive environment designed for learning and growth. Students will refine
+their storytelling, articulate their value proposition, and present their venture
+to investors and experienced entrepreneurs, receiving direct feedback on both
+their business model and their pitch delivery. 
+Through class lectures, YourCo assignments, real-world cases, and guest
+fireside chats, the course covers the multidimensional aspects of
+entrepreneurship as both a mindset and a process that can be practiced and
+improved. 
+NOTE: WEEK 1 CLASS ATTENDANCE IS MANDATORY. IF YOU ARE CONSIDERING
+ADDING THE COURSE BUT DO NOT YET HAVE A SEAT, YOU MUST ATTEND THE
+FIRST CLASS IN ORDER TO REGISTER DURING DROP/ADD. PLEASE EMAIL ME IF
+YOU AREN’T YET REGISTERED BUT WANT TO ATTEND CLASS 1.</t>
         </is>
       </c>
     </row>
@@ -72542,17 +73055,21 @@
       <c r="H70" t="inlineStr"/>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>SCHEDULE
-SPECIAL TOPICS IN ENTREPRENEURSHIP: DEVELOPING A NEW VENTURE (NEW
-VENTURE CHALLENGE) (34104) - TEBBE, MARK&gt;&gt;
-This course is designed to allow students who have advanced to the second
-round of the New Venture Challenge to develop their ideas into businesses.
-Student teams will work largely on their own to develop their businesses.
-The class meetings consist primarily of business presentations. Venture
-capitalists, private investors, and entrepreneurs will help critique and improve
-the ideas and businesses during the presentations. The class meetings also will
-include sessions on presentation skills, financial modeling, and legal
-considerations in a new venture.</t>
+          <t>This course is designed to allow students who have advanced to the second
+round of the New Venture Challenge to develop their ideas into full business
+plans. Student teams will work largely on their own to develop their business
+plans and are encouraged to meet individually with the class coaches and
+faculty.
+The class meetings consist primarily of plan presentations. Venture capitalists,
+private investors, and entrepreneurs will also help critique and improve the
+plans during the presentations. The class sessions also will include workshops
+on the legal considerations of a new venture, developing marketing and sales
+plans, developing financial projections and presentation skills.
+Preassignment: An orientation meeting for all teams that have advanced to the
+second round of the New Venture Challenge will be held during winter quarter.
+Students should come to this meeting ready to present an elevator pitch of
+their ideas. Students will also be required to present their business model
+during the first weeks of class.</t>
         </is>
       </c>
     </row>
@@ -72670,7 +73187,73 @@
 and a lack of practical frameworks for success. Outperformers have learned to
 develop a deeper understanding of what motivates (and irritates) end users,
 challenge biases in their organizations and themselves, and follow a
-repeatable and scalable path to new insights and reduced innovation risks.</t>
+repeatable and scalable path to new insights and reduced innovation risks.
+This course is designed to provide proven frameworks, practical applications,
+and an emphasis on helping each participant develop the innovative mindsets
+and skillsets required for innovative problem-solving in organizations big and
+small.
+Through hands-on activities, case studies, and actionable strategies, this
+course will equip participants with the tools, mindsets, and frameworks to
+develop meaningfully unique ideas, systematically identify and mitigate the
+unique risks to each, and build the resulting innovative concepts into
+competitive advantage. Particular attention will include how to innovate with AI
+inside an enterprise setting.
+You’ll learn to: 
+Foster a culture of experimentation, risk-taking, and collaboration.
+Empower teams to solve problems creatively and resourcefully.
+Implement practical methods to reduce risk and drive innovation quickly
+and inexpensively.
+Align innovation efforts with strategic goals to ensure measurable impact.
+This course is for leaders and managers who want their core professional
+skillset to include how to identify and solve unique problems. Participants will
+learn to develop innovative concepts for products, services, and processes, de-
+risk them, and foster higher engagement in their teams, accelerate growth,
+and navigate complexity with confidence.
+Course Design
+This course explores four skillset themes that are crucial to leading innovation
+and change in an organization.
+· Theme 1: Discovery and Creation– You will practice the skills that are required
+to see the world through a different lens, to identify opportunities and
+potential sources of disruption, and to create non-obvious solutions to
+problems. We will explore these skills and practice flexing these muscles
+through in-class exercises and group homework assignments.  Creativity and
+structured problem-solving will be heavily emphasized throughout the entire
+class.
+ · Theme 2: De-Risking and Execution – Not knowing how to manage risk is a
+leading reason why companies kill breakthrough innovation. We will explore
+why this happens and learn tactical tools you can employ as a leader to
+manage risk and execute innovation despite the unknowns.
+· Theme 3: Communication and Influence – Communicating new or complex
+ideas and bringing others along to support you is crucial to making innovation
+happen. In this portion of the class we will explore how to employ alternative
+strategies such as visual communication and storytelling in your pursuit of
+communicating your ideas and influencing others.
+· Theme 4: Innovation Infrastructure – This portion of the class will explore
+operational topics surrounding innovation with a focus on how to develop a
+sustainable innovation strategy supported by the right capabilities, structure,
+and culture. We will discuss various organizational and strategic models for
+executing innovation, and the challenges of execution within established
+enterprises.
+Readings and asynchronous lectures will be assigned prior to each class to
+introduce content. Classroom time will be spent applying the course concepts
+through case discussions, in-class activities, and guest speakers. Students will
+also work in teams on hands-on group assignments throughout the quarter
+that parallel course content and enable you to apply skills learned in class.
+Learning Objectives
+This class is designed to build on other business and course skills to make you
+a more creative and ambidextrous thinker. The objective is to arm you with a
+toolkit for leading innovation and growth in the context of high risk, nebulous,
+and highly uncertain innovation initiatives.  We will cover the foundational
+principles of user-centered design and prototyping through the context of
+solving business problems broadly, however traditional product development
+tools and frameworks are not the focus of the class. Specific learning outcomes
+of this course include becoming:
+· A stronger innovation practitioner (greater proficiency of using innovation
+skills and tools)
+· A more effective manager of innovation (ability to manage the process and
+connect the right people/recourses/thinking to make things happen)
+· A more inspirational leader of innovation (greater ability to think creatively,
+teach others, and inspire others)</t>
         </is>
       </c>
     </row>
@@ -72734,7 +73317,16 @@
 entrepreneurship.
 Overarching Goal
 The goal of this course is to make you as efficient and effective in selling
-(persuasion) as possible, so that when you are spending time selling, not a</t>
+(persuasion) as possible, so that when you are spending time selling, not a
+moment is wasted. Why? Because as an entrepreneur (and a human), the way
+you spend your time determines success and failure.
+Learning Objectives
+You will be able to:
+•Understand the key phases of the entrepreneurial selling process, and identify
+the most common failure points in the process
+•Construct a sales toolkit for your venture
+•Build a set of sales skills and disciplines that will serve you in any career
+context (and in life...)</t>
         </is>
       </c>
     </row>
@@ -72770,7 +73362,40 @@
       <c r="I74" s="2" t="inlineStr">
         <is>
           <t>Impact investing plays an expanding role in deploying financial resources to
-address social problems through market-based interventions. Impact investing</t>
+address social problems through market-based interventions. Impact investing
+includes both “non-concessionary” or “market-rate” investments that target
+risk-adjusted market-rate returns and “impact-first” or “catalytic” investments
+that anticipate lower than market returns.  
+Impact investing presents several intellectually interesting and practically
+important issues. Learning the strategies and mechanics of impact investing
+provide an opportunity to apply frameworks from corporate finance,
+microeconomics, and strategy to an interesting and rapidly evolving sector.
+There are rich questions about the market for impact investors -- who they are,
+how to market to them, and how to structure funds to attract them. We will
+study the “impact” of impact investing, as well as the financial returns and risks
+of such investments. 
+Students will work in teams of four to six to develop and pitch an impact
+investment fund. Group assignments will help each team identify opportunity
+drivers and a thesis, an investment strategy, an impact management and
+measurement framework, a pipeline of companies, and prospective investors.
+Each group’s final presentation will be in the form of a presentation to a group
+of potential investors. 
+The course also brings practitioners to the classroom, offering candid
+presentations from leading fund managers pursuing impact strategies within
+venture capital, real estate, private credit, and private equity. Individual
+assignments ask students to connect what they heard with the practice of
+finding deals and constructing appropriate impact metrics. Participation is a
+significant component of the course, with the expectation that students come
+prepared to ask questions and contribute insights.
+This class complements the existing curriculum in corporate finance and
+private equity (Corporate Finance, Entrepreneurial Finance and Private Equity,
+Commercializing Innovation). Consistent with our curricular philosophy in
+other social enterprise courses, this is not a substitute “social” version of an
+existing course, but will focus on differences between the social and traditional
+institutions. Although no individual student needs to have a deep finance
+background, we will ensure that each team has at least one member with rich
+knowledge/experience. All students should have some working knowledge of
+finance and financial institutions.</t>
         </is>
       </c>
     </row>
@@ -72872,7 +73497,40 @@
 entrepreneurial ventures – namely, can the problem be validated by the target
 users, customers, beneficiaries, and, is the proposed venture the best solution
 to address this problem.  Determining the best business model for a social
-venture can be very challenging. Social entrepreneurs must address the likely</t>
+venture can be very challenging. Social entrepreneurs must address the likely
+source of funding, whether or how much to charge beneficiaries, other
+revenue streams, identify initial target beneficiaries, and often work within
+complex private, public, and nonprofit value networks.
+Much of class time will be devoted to group exercises to implement
+frameworks to answer these questions for the students’ venture ideas as well
+as a set of case study examples we will use throughout the course.
+In addition, there will be occasional class discussions on the role of social
+entrepreneurship for developing and scaling innovative solutions to society’s
+problems and alternative pathways for social innovation.
+This class is a key component of the Rustandy Center for Social Sector
+Innovation’s Social Venture Studio program. Promising ventures coming out of
+this class will be invited to participate in winter quarter programming at the
+Rustandy Center which will prepare student-led teams for the John Edwardson
+’72 Social New Venture Challenge in the upcoming spring quarter or in
+subsequent years. In the SNVC, teams have the opportunity to build out their
+ventures, develop and refine a pitch for potential investors/philanthropists,
+and present their ideas to successful social entrepreneurs and, and potentially
+receive seed funding to support the launch of the new venture.
+Grading will be based on class participation and peer collaboration, a final
+presentation, and a final meeting with the instructors to review their venture
+project. There will be no exams.
+Interested students should apply via the online application. The initial
+application deadline for returning students is 5:00pm August 19. Students who
+apply by this deadline will be notified of application decisions on August 22
+before bidding starts. We will continue to accept applications from all students
+(Booth and non-Booth) through September 19 and will make decisions on a
+rolling basis (within three business days from submission). 
+Non-Booth students are encouraged to apply for the course. We expect at least
+one team member from each venture to enroll in the course. Other team
+members are welcome to enroll or audit. For non-Booth teams, if degree
+requirements make it challenging for any student to enroll in the course, we
+will allow all team members to audit with the understanding that they will
+complete all work as if they were enrolled.</t>
         </is>
       </c>
     </row>
@@ -72928,7 +73586,10 @@
 lecturer-in-management at Stanford University’s Graduate School of Business
 since 2014 and Adjunct Professor of Entrepreneurship at the University of
 Chicago’s Booth Business School since 2019. Ms. Rapp earned a B.A. in Political
-Science and the History of Art from Yale University in 2000 and an M.B.A. from</t>
+Science and the History of Art from Yale University in 2000 and an M.B.A. from
+Stanford University’s Graduate School of Business in 2005. She is the author of
+Amazon Bestseller, Leadership and Life Hacks: Insights from a Mom, Wife,
+Entrepreneur &amp; Executive (ForbesBooks, October 2019).</t>
         </is>
       </c>
     </row>
@@ -72965,7 +73626,44 @@
 tend to outperform and outlast their counterparts (Harvard Business Review,
 2012). Admittedly amorphous, the course will begin by exploring the ambiguity
 of defining closely held businesses.  Next, the course will focus on why and
-how closely held businesses can achieve these extraordinary results so that</t>
+how closely held businesses can achieve these extraordinary results so that
+students can apply these practices to their own careers and families,
+regardless of the type of business.
+AUDIENCE:
+If you are interested or intrigued by the idea of having financial and
+operational independence in your business and your life, this course is for
+you.  This class is aimed towards students who are interested in exploring
+alternate paths to independence and entrepreneurship afforded by closely
+held and family businesses.  We will explore the benefits of stewarding a
+business to preserve and create generational wealth, while also maintaining
+maximum control over your business and, more importantly, your personal
+values and life.  This course will introduce concepts relevant to investors,
+owners and operators who are interested in exploring or considering a long
+term or perpetual hold period perspective, with a focus on creating and
+maintaining profitability.  This class will target students who are intending to
+manage a closely held business, either their own family’s or someone else’s, or
+those who will engage with closely held businesses through consulting, private
+wealth management, mergers and acquisitions, banking, etc. The course will
+also be relevant to students who are interested in acquiring a closely held
+business.  
+CLASS MODEL / PHILSOPHY OF THE COURSE:
+This course will provide a theoretical and practical understanding of closely
+held businesses and long term ownership (15+ years). It will draw on concepts
+gained from other courses (managerial decision making, behavioral /
+relationship dynamics, tax strategy, and organizational practices and
+structures) and analyze them within the context of the closely held business
+and long term ownership. 
+This course surveys many topics related to closely held businesses and long
+term ownership. It aims to establish a foundational knowledge that inspires
+connections to other business courses. The course will mix theory (through
+cases and assigned readings) with practice (through guest presentations and
+student participation). Through participation and in-class conversations, the
+course will provide a forum where students with previous exposure to closely
+held businesses can share their experiences and best practices. Through these
+open discussions on potentially difficult topics (sibling rivalry, compensation,
+corruption, power dynamics, ethical dilemmas, etc.) students will have the
+opportunity to learn as much from their peers as from their professors, guest
+speakers and readings.</t>
         </is>
       </c>
     </row>
@@ -73006,7 +73704,41 @@
 required for new venture creation.
 As the capstone project for the course, students from Booth, the Physical
 Sciences Division and the Biological Sciences Division will work collaboratively
-to create business plans and pitch decks based on intellectual property</t>
+to create business plans and pitch decks based on intellectual property
+available for license from universities. At the conclusion of the course, their
+learnings will provide a roadmap for their own entrepreneurial ambitions, and
+some may have business plans they choose to take forward.
+Structurally, in the first three weeks of this course, students will learn and
+apply business and science frameworks to a challenging life-sciences case.
+Once the approach is solidified, students will identify intellectual property from
+universities across the country that they find compelling and then apply the
+structures they learned to create their own business plans and pitch decks
+based on the intellectual property they identified. In both the case study and
+the final project, business, medical and science students will work together in
+teams to leverage their individual expertise. Many students find this
+collaboration between business and science to be a highly valuable learning
+experience. During the course, guest lecturers including entrepreneurs,
+investors, IP and licensing attorneys will help students construct the roadmap
+to venture creation.
+The specific learning objectives of this course are highlighted below:
+?      A framework to create and evaluate research programs
+?      A framework to create and evaluate research-driven business plans
+?      Business and science students will learn to collaborate across knowledge
+domains
+?      How to create and evaluate financial models for entrepreneurial, research-
+driven businesses
+?      The fundamentals of intellectual property and licensing
+?      The creative process and challenges at the earliest stages of research-
+driven entrepreneurship
+?      Solid foundation for students to begin their entrepreneurial journeys 
+Course Procedures
+It is not necessary for Booth students to have a background in the sciences or
+for science students to have a background in business. However, the
+expectation is that each member is an active participant. Peer assessments
+make a substantial impact on individual grades. Please be sure you can
+regularly accommodate team meetings outside the classroom and devote the
+time necessary, roughly 6-8 hours per week. The course is also highly
+participatory, so attendance is expected. Please arrive before the class starts.</t>
         </is>
       </c>
     </row>
@@ -73092,7 +73824,46 @@
 effective, pleasurable user experiences, to provide tangible, ethical benefits to
 users/consumers.
 In particular, the course will consider user experiences in 4 domains:
-health/fitness, urban mobility, self-expression, and entertainment.</t>
+health/fitness, urban mobility, self-expression, and entertainment.
+LEARNING OUTCOMES
+The goal of the course is to envisage future, innovative, intelligent, integrated
+product-service offerings, and develop an interdisciplinary method to design
+satisfactory user experiences.
+The course addresses competences that can be applied to product managers,
+tech leaders, and top management.
+From this course, students will learn to:
+Understand product/service systems, integrating physical and digital
+experiences
+Assess the business value of positive, efficient, pleasurable user
+experiences
+Use tools and processes to develop human-driven innovation
+Integrate multi-disciplinary teams comprising business, engineering and
+design in small to large organizations
+Envisage future product/service systems based on agentic AI, to enable
+innovative user experiences
+COURSE FORMAT
+The course has a hands-on, interdisciplinary, creative format, combining the
+perspectives of Experience Design, Technology Innovation, and Business
+Disruption.
+The course has a combination of lectures, teamwork in class, and individual
+homework.
+TEAMWORK CLASS PROJECTS
+Students will be graded by the faculty at a large percentage on their overall
+performance on the group projects.
+Process and creativity will be balanced. Individual work and teamwork will be
+evaluated both in the use of tools and processes and in generating inspiring
+results.
+The faculty cares about the quality of your work on the project itself, the way in
+which you work within a multi-disciplinary group, and the documentation and
+presentation of your team’s work product.
+The faculty’s primary concern is that all team members have meaningful tasks,
+and that students deliver on these tasks for the team. First, teams have
+responsibility to assign tasks to all members, and to make sure everybody is
+engaged and actively participating. members and determine, on a weekly basis
+and as a team, whether these tasks were fulfilled, culminating with a brief
+weekly report submitted to the faculty. Failure to complete tasks appropriately
+will negatively impact grades. Second, each student will be asked to candidly
+evaluate your team members.</t>
         </is>
       </c>
     </row>
@@ -73144,7 +73915,16 @@
 executives, investment bankers and finance executives. 
 Topic areas will include:
 1. Use of structure to shape, allocate and underwrite risk/return
-(attach/detach levels, embedded options and convexity, etc).</t>
+(attach/detach levels, embedded options and convexity, etc).
+2. Tax considerations in structuring, including differing tax treatment of
+economically similar instruments, transactions and investment strategies.
+3. Fund and portfolio level structuring, GP and LP (taxable and tax-exempt)
+investor perspectives, including blocker strategies.
+4. Incorporating tax attributes and after-tax returns into underwriting and
+performance measurement, from direct investments to fund investments
+to portfolio construction.
+5. Recent innovations in tax-aware investment strategies and investment
+products.</t>
         </is>
       </c>
     </row>
@@ -73189,7 +73969,44 @@
 examples to see how investment decisions are made in practice.
 HOW YOU LEARN
 This course combines academic rigor with practical efficiency.
-You’ll complete focused readings, short cases, and analytical exercises before</t>
+You’ll complete focused readings, short cases, and analytical exercises before
+each session.
+In-class presentations help you connect the dots and build a clear conceptual
+framework.
+Expect 6-7 hours of preparation per week in addition to class attendance.
+WHERE IT MATTERS
+Relevant for careers in asset management, private equity, infrastructure, real
+estate, private debt, consulting, and private banking.
+You’ll learn to think like an investor — understanding how capital providers
+evaluate, structure, and fund opportunities.
+The skills you gain will enhance your professional confidence and provide an
+edge in interviews for investment-related roles.
+WHO SHOULD TAKE THIS COURSE
+There are no formal prerequisites, but students who have taken private
+equity–focused classes or have prior internship or industry experience will find
+it easier to navigate and absorb the substantial volume of material.
+The course is designed for those with a serious interest in private markets and
+a willingness to engage consistently throughout the quarter.
+COURSE FORMAT &amp; ASSESSMENT
+This is a lecture-based course supported by ongoing analytical work.
+Assessment is based on class participation, short analytical assignments, two
+group projects, weekly graded quizzes, and a final exam.
+Continuous engagement is essential — this is not a class where students can
+“coast” early and catch up just before midterms or finals. Steady effort
+throughout the term is key to success.
+INSTRUCTOR PERSPECTIVE
+Private markets have evolved from niche strategies into a core pillar of global
+capital formation.
+This course helps you understand how institutional investors think, how funds
+are structured, and how value is created — knowledge that remains relevant
+across economic cycles.
+Students also gain insight into the forces shaping the industry, including how
+key players are driving disintermediation within the financial sector.
+Exposure to some of the most current industry practices and playbooks has
+helped past students secure internships and full-time roles in leading private
+markets firms.
+*** You an find additional information on the  course webpage  which will be
+available from Nov. 26 onwards***</t>
         </is>
       </c>
     </row>
@@ -73242,7 +74059,28 @@
 initial operating period, Unicorns blessed with vast amounts of capital for rapid
 expansion yet in need of ideas and data on how to best spend it, private
 businesses looking for growth, and turnaround opportunities which can make
-good acquisition targets for buy-out entrepreneurs.</t>
+good acquisition targets for buy-out entrepreneurs.
+     As a workshop we will solve strategy puzzles in class together which means
+student groups presenting solutions in real time. This allows us to build the
+frameworks required to think strategically. Each student will be required to
+carefully analyze assigned cases, stay current in "The Wall Street Journal,"
+together with a study group, present a well developed strategy proposal on
+how to solve real issues with an existing company, and write an individual term
+paper outlining strategy for a company or organization in trouble.
+     Because of the complexity of forever time, we do not build generic models
+of success as we do in New Venture Strategy. Instead we concentrate on
+taming the inherent challenges of operating without time limits. Cases used in
+New Venture Strategy will not be used in this course, nor will the NVS
+frameworks.The cognitive science underpinnings of New Venture Strategy will
+remain although we will look at the foundations of the Advanced NVS
+Workshop when possible with new examples to illustrate the central concepts. 
+     By the end of the quarter, students should have an idea of how to formulate
+strategy for an existing business looking for growth, and how to realistically
+assess inherent risk in various options. We will practice how best to make all-
+important strategy presentations to board members of the enterprise or
+organization.
+     Our goal is to develop an unconscious common sense about strategy
+beyond a start-up's initial operating period.</t>
         </is>
       </c>
     </row>
@@ -73293,7 +74131,11 @@
 please be prepared for role playing, at any point in the class, as Professors
 Agnew and O’Connor strongly believe in trying to make some of the concepts
 as applicable as possible. Grading here will be based primarily on the quality of
-the ideas with which you bring to class. Most class meetings will have guest</t>
+the ideas with which you bring to class. Most class meetings will have guest
+speakers as “real life” entrepreneurs and investors are critical to the
+understanding of class material and frameworks. Active involvement and
+engagement with the guest speakers will be factored into the class
+participation grade.</t>
         </is>
       </c>
     </row>
@@ -73469,7 +74311,14 @@
 adjust their learning in preparation for more in-depth class debate.
 Grades are based on host firm evaluations, classroom participation, individual
 assignments, case write-ups and a final project. The course cannot be taken
-pass/fail and may not be audited.</t>
+pass/fail and may not be audited.
+Students will be selected for the course through a competitive
+screening/interviewing process, which begins by submitting a resume and a
+questionnaire in a process conducted by the Polsky Center. The host firms
+choose interns. All students who secure an internship through the program are
+required to take the class due to federal laws relating to unpaid internships.
+More information on the selection process can be found on the Private Equity
+Lab website.</t>
         </is>
       </c>
     </row>
@@ -73522,7 +74371,14 @@
 opportunity fund in which the team looks to create an investment thesis which
 is more complex, potentially more narrow and seeks to creatively exploit a
 perceived mispricing.
-The overarching goal of the Real Estate Lab is to provide participating students</t>
+The overarching goal of the Real Estate Lab is to provide participating students
+with the latitude to examine/research investment strategies in which they are
+interested and to stimulate the investigation of companies and/or strategies
+that enables those students to “hit the ground running” with one or more
+investment ideas that they might hopefully deploy in the future. Accordingly,
+the Real Estate Lab attempts to place few constraints on the students’
+creativity.
+Please see syllabus link for additional details regarding this course.</t>
         </is>
       </c>
     </row>
@@ -73603,7 +74459,34 @@
 customers and stakeholders while defining and running their business, you will
 do the same in this class!
 This class will include a combination of lectures, team presentations,
-discussions, and in-class discussions. Class time will be highly interactive with</t>
+discussions, and in-class discussions. Class time will be highly interactive with
+students expected to actively participate by sharing insights and solutions.
+Students are only allowed to participate in their registered section. As
+members of a lab class, students will work in student-only teams to conduct
+interviews, perform observations, and work closely with industry experts and
+stakeholders as well as their other core team members. Group work is
+essential to the design process and will be extensive in this course. Participants
+should expect to meet with their assigned group multiple times outside of the
+classroom and should anticipate investing a minimum of seven hours per
+week.  
+By the end of the course, you will have acquired reusable business innovation
+skills and tools to:
+1. discover problem areas worth exploring,
+2. discriminate between strong and weak business ideas, 
+3. refine possible business ideas by iteratively exploring solutions, 
+4. enhance these ideas with customer and market feedback, 
+5. outline a viable business model on a Business Model Canvas, 
+6. rapidly test, iterate and execute on your defined business model, and
+7. effectively communicate the needs for growing your business.
+Due to the group nature of this course, you will only be able to drop the class
+before the first class begins.
+As expressed by one of the Autumn 2024 students in last year’s feedback
+forms, "I am super glad that I took Entrepreneurial Discovery and would
+recommend it to first year students looking for an introduction to the
+entrepreneurial process. Leveraging Prof Tebbe’s experience and proven
+insights, we gained a framework that gave me clarity on how to identify a real
+problem that’s worth pursuing and then how to build the business core to
+make it happen."</t>
         </is>
       </c>
     </row>
@@ -73627,7 +74510,7 @@
         </is>
       </c>
       <c r="F91" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr"/>
@@ -73647,7 +74530,83 @@
 Teams composed of 3-4 students will build a new business, utilizing a lab
 technology that is sourced from a leading research lab (university or national
 lab)
-• Technologies will be sourced and vetted by a PHD Science student from the</t>
+• Technologies will be sourced and vetted by a PHD Science student from the
+University of Chicago’s Molecular Engineering, Physical Science, and Biological
+Science programs. These students participate as part of a team in the class,
+providing a unique technical capability.
+• You may have the option to continue building the business after the class and
+potentially become an equity holder.
+• You will be able to enter the business in the New Venture Challenge. A
+number of prior teams have been accepted.
+Key milestones include:
+• Determining the right technology to pursue from a large number of
+technologies, utilizing the analysis performed in the fall by the PHD team
+member.
+• Analyzing multiple commercial market opportunities for the selected
+technology to determine the path forward (i.e. which approach has best
+financial benefits and lowest risk).
+• Building a business plan, which sets the road map for commercializing the
+technology, and summarize this information in a VC pitch deck.
+• Developing a robust set of skills, tools and experiences that you can utilize
+throughout your life.
+Support &amp; Guidance:
+• Professors who will guide you through the class:
+- Jason Blumberg: Head of a leading new energy VC fund + head of a leading
+energy focused Foundation + A sought out thought leader on Critical
+Industries, Energy &amp; Cleantech issues
+- Keith Crandell: Head of one the world’s preeminent science focused VC’s –
+20+ IPO’s and Billions of $’s of value created
+• Engage with preset external advisors from the professor’s network, who will
+provide technical and/or business advice. These include leaders in industry,
+research and investments.
+• Work with a leading lab or university to understand the technology and
+receive support from your U of C IME team member.
+• Garner input from an array of referral sources and hear guest lectures from
+industry leaders.
+Actual experience with a lab technology will be augmented with classroom
+instruction focused on:
+• Issues faced by entrepreneurs as they work to commercialize a lab based
+technology.
+• Core principals and technologies that are shaping the science landscaped,
+including the structure of various representative markets and overviews of
+major and minor technologies.
+• Building a toolset to be able to effectively and efficiently develop
+commercialize plan, solve complex problems, and provide high impact advice.
+The ultimate objective of the class is to provide students with a hands-on
+experience in commercializing lab based technologies. This type of immersion
+is insightful for students considering founding a company, working in a start-
+up, consulting, venture capital and/or working in the science based industries.
+Students who join this class in order to work with one particular technology
+will not obtain the full benefit of the course. Technologies that appear exciting
+in the course marketing materials may yield unexpected challenges.
+For those interested in foundational knowledge in commercializing science or
+building a science based businesses’ (i.e. anything besides digital &amp; AI) we hope
+you’ll find this one of your best classes.
+APPLICATION:
+Admittance into the class is by application only. Prospective class participants
+need to apply to participate. Since real-world problems often cut across
+multiple disciplines and interest groups, this course draws from a pool of
+students with a wide range of backgrounds, skills and perspectives with
+experience and across multiple schools in the university.
+Please apply for the class using this link. Applications may be submitted
+anytime and will be reviewed on a rolling basis until the class is filled.  Please
+note this course is typically in very high demand, so we encourage you to apply
+early, as no additional seats will be available once capacity is reached.
+ADDITIONAL DETAIL:
+Students are expected to work 7– 10 hours out of class each week. This
+includes team and technology leads, independent and group research,
+interviews, presentation preparation and more. Individual team meetings are
+scheduled with the professor every 2 weeks or more if necessary.
+Students who elect to register for this course should consider this a
+commitment. Dropping this class after the first week is strongly discouraged.
+Part-time students are welcome, but this class requires substantial schedule
+flexibility. Students must be able to schedule frequent meetings with the Lab
+Partner, often during business hours.
+Project management is a key focus of the class. Many of the research partner
+leads may have not worked with MBA students before and consequently,
+students are expected to guide the process. Part of each class is devoted to
+discussing strategies and actual project issues in order to arrive at desired
+results.</t>
         </is>
       </c>
     </row>
@@ -73689,7 +74648,9 @@
 capital funds.  The course should therefore be broadly useful not only for
 students who are interested in working in private capital, but more broadly for
 those pursuing a career in finance, management, or consulting.
-NO SYLLABUS AVAILABLE</t>
+NO SYLLABUS AVAILABLE
+Description and/or course criteria last updated: December 04 2025
+HACKING FOR DEFENSE</t>
         </is>
       </c>
     </row>
@@ -73724,7 +74685,79 @@
       <c r="I93" s="2" t="inlineStr">
         <is>
           <t>Course Application
-Info Session:</t>
+Info Session:
+Thursday, Oct 30th, 5:15 - 6:00pm, ZOOM
+Registration Link: https://forms.gle/1QpcoYuGbsatNV3q7
+ Course Application:
+Apply here:  https://forms.gle/F4sfHpmanYTkLqgy7
+Course Timeline:
+Oct 16th - Applications Open
+Oct 24th - Info Session (ZOOM)
+Oct 28th (Monday) - Applications Close
+Nov 1 (Friday) - Admitted Students Notified
+Nov 6 (Wednesday) - Students confirm admission; we submit list to Booth
+Registrar
+Nov 11 thr Jan 3  - Virtual Team Formation Process with Faculty &amp; Project
+Onboarding
+Jan 6, 2025 - WTR Quarter Begins
+Jan 10 (Friday), 2025 - First Class Session
+**NEW for this year: Apply with an existing startup or idea to get matched with
+a government go-to-market sponsor. Submit ideas here and expect an email to
+debrief: https://forms.gle/zNFUeGRV1p5fhyaa6 
+_____
+Course Overview | Hacking for Defense is an application-based,
+entrepreneurship lab experience with a focus on government innovation.  In
+this course, the faculty source fascinating technical and operational challenges
+from across the Department of Defense and Intelligence Agencies (DoD/IC) and
+match them with interdisciplinary student R&amp;D teams from across campus.
+During the course, students will not only learn the innovation toolkit (customer
+discovery, human-centered design, prototyping, how to build an effective pitch
+deck, and leadership), but will get a chance to apply that toolkit to real-world
+problems facing one of the world’s most complex and impactful bureaucracies.
+By the end of the course, students will gain professional experience
+systematically reducing organizational uncertainties, elevating their
+professional networks, and creating breakout solutions that can gain adoption
+within a huge organization and in new markets.
+Students’ career trajectories have been meaningfully transformed by this
+course. In the course’s first six years at Uchicago (with teams of students from
+across schools), we have had 7 teams successfully advance into the various
+NVC (“New Venture Challenge”) programs, two finished in the top 4, one won
+$80k in NVC, and another that was commercially acquired within 12 months of
+starting the class. Past Projects focused on projects ranging from: logistics,
+deep-tech, data-fusion, bio-tech, AI/ML, market creation, gender equity, digital
+manufacturing, distributed knowledge management, space management, and
+cyber security. (We expect future projects will be equally compelling). In the
+course evaluations, many students said the course was the most impactful
+learning experience they’ve had during their degree programs.
+Opportunity and Experience | The innovation toolkit (lean startup, human-
+centered design, prototyping) was developed to create new value under
+conditions of extreme uncertainty. Our large institutions--both public and
+private--involve uncertainties at the cutting edge of technology and
+management with outsized implications. We believe such institutions should
+be more responsive to changing conditions and that they deserve commitment
+from the best and brightest when it comes to the application of innovation. All
+of the teams within the DoD/IC are large, complex, and as impactful on society
+as any that one can identify. These teams face intense pressure to adapt their
+missions to changing constituencies, evolving geopolitical demands,
+technology revolutions, wider social norms, and complex regulations. This
+course aims to train teams of students in how to apply the innovation toolkit to
+such organizations and their challenges. 
+Students will apply to the class and be assigned to a project sponsored by a
+top government official. In the application, students will share their current
+skills, areas of desired development, and project preferences (posted mid-
+Autumn). The class projects center on the types of problems that few
+professionals get access to throughout their careers--working directly with
+high-level policy and operational experts who are asking your team to solve
+problems they’ve been unable to address.  Each team’s goal during the course
+is to develop a viable business (“mission”) model for a dual-use new venture--
+serving customers both in government and the private sector. Students will be
+supported by both the faculty and between 8-12 expert coaches drawn from
+the national labs, relevant agencies, technology firms, and DoD affiliates. 
+Overall, the course is now organized into 3 Phases (Methods, Mindsets, and
+Landscape; Confirming Beneficiary Value; Completing the Mission Model
+Canvas). The final course output will remain a rigorous and defensible pitch to
+your team’s client agency about how to address your challenge through a dual-
+use venture.</t>
         </is>
       </c>
     </row>
@@ -73823,7 +74856,35 @@
 advantages. All leaders need far better Foresight to build optionality, both
 professionally and personally.
 I'm a professor, author and active venture investor in nearly 50 companies and
-venture funds. I look forward to envisioning, exploring and creating the future</t>
+venture funds. I look forward to envisioning, exploring and creating the future
+with all of you.
+Innovation must be a principal objective of senior management; unfortunately,
+few managers achieve the innovation competencies necessary to manage the
+innovation portfolio required by global firms to achieve growth and profitability
+objectives. This course will apply a theoretical and applied approach to
+understanding Innovation Strategy &amp; Management from the perspective of
+senior corporate leaders.
+The course will focus on innovation within business entities, from the typical
+technology and product innovation programs, to broader, process, marketing
+and other forms of innovation. The course will address innovation as a holistic
+strategic management imperative not limited to Research &amp; Development or
+New Product Development. While the course will provide a theoretical
+foundation, the focus will be on real world issues, products and systems.
+We will:
+--Build foresight for where we're going across industries as a result of
+technology
+--Examine Innovation from the perspective of corporate strategy
+--Explore the impact of a range of emerging technologies on the future of
+business and society
+- Relate Innovation to other factors such as Marketing, Risk, Structure,
+Processes and Project Management
+- Discuss best practices from a number of leading firms, including Amazon,
+Netflix, AXON, BP, Disney, Dell, Zebra Technologies, Honeywell; category-
+creating companies like Haddy.life, AXON, Interstellar Lab, Unqork; and non-
+profit/government initiatives such as the Cambodian HIV/AIDS national
+response
+- Consider what we’re trying to accomplish in the world, and WHY, both
+professionally and personally.</t>
         </is>
       </c>
     </row>
@@ -74085,7 +75146,10 @@
 decisions. The course combines a theoretical framework with applied analysis.
 Topics covered include: portfolio selection based on mean-variance analysis,
 models of risk and return (including the CAPM and multifactor models),
-performance evaluation of mutual funds and hedge funds, market efficiency</t>
+performance evaluation of mutual funds and hedge funds, market efficiency
+and the random walk hypothesis, asset pricing anomalies and behavioral
+finance, derivative security pricing (including options, futures, forwards, and
+swaps), and the term structure of interest rates.</t>
         </is>
       </c>
     </row>
@@ -74257,7 +75321,7 @@
       <c r="I105" s="2" t="inlineStr">
         <is>
           <t>This course discusses the challenges to finance progress in healthcare in the
-21  century, and the possible solutions, with a specific focus on drug
+21 century, and the possible solutions, with a specific focus on drug
 discovery. The course reviews the current framework for drug approval,
 including the economics of clinical trials, and introduces the tools used for
 investment valuation, such as decision trees, financial and real options, Monte
@@ -74267,7 +75331,8 @@
 and targeted therapies, its current challenges, and the promises offered by
 new technologies, such as machine learning and artificial intelligence, and their
 impact on healthcare finance. Case studies are used to cement the concepts
-discussed in class.</t>
+discussed in class.
+st</t>
         </is>
       </c>
     </row>
@@ -74482,7 +75547,31 @@
 Mae. In addition, a large market of exchange traded and over-the-counter
 derivative securities is available for trade in order to undertake sophisticated
 hedging strategies or to adjust the risk/return characteristics of an investment
-portfolio.</t>
+portfolio.
+This course covers models and techniques that are used to analyze fixed
+income securities their (often embedded) derivatives. By the end of the course,
+students will learn (i) the basic concepts of fixed income instruments, such as
+yield curve, forward curve, yield-to-maturity, duration, convexity; (ii) the
+modern empirical methodologies to describe Treasury bond data, such as
+"curve fitting" and factor analysis; (iii) effective hedging strategies for fixed
+income portfolios, such as duration matching, asset-liability management and
+factor neutrality; (iv) the advanced properties of bonds, such as their
+risk/return characteristics, and the best predictors of their future
+returns; (v) modeling techniques used by market participants, such as the
+models of Vasicek, Cox Ingersoll and Ross, Ho and Lee, Hull and White, Black-
+Derman-Toy, and Heath-Jarrow-Morton; and, importantly, (vi) how to use these
+methodologies in practice to value and hedge fixed income products and
+derivatives, from the traditional securities, such as Bonds, Swaps, Options,
+Caps and Floors, to the more recent products, such as Inverse Floaters, Range
+Notes, Mortgage Backed Securities.
+The key feature of this course is that it strongly emphasizes the applications of
+these methodologies to value real world fixed income products, and their
+derivatives, by focusing both on the practical difficulties of applying models to
+the data, as well as on the necessity to use computers to compute prices. The
+course, which is analytical in nature, includes many real world Case
+Studies and Data Analysis to allow students to apply these models to a wide
+range of fixed income securities as well as to understand their risk and return
+characteristics.</t>
         </is>
       </c>
     </row>
@@ -74831,7 +75920,19 @@
 broker-dealers, and sovereign funds exhibit strong demand for these
 securities. We first discuss recent trends and the investment opportunities
 offered by corporate and sovereign bonds, including callable, convertible and
-other structured securities, their risks and their expected returns. We will then</t>
+other structured securities, their risks and their expected returns. We will then
+discuss the booming U.S. private credit market, including middle market
+corporate direct lending, real estate credit, asset-based lending, specialty
+finance and infrastructure debt; its market participants, and the risk and
+investment opportunities that it offers to both corporations (who borrow) and
+investors (who lend). Students will learn to apply factor models and
+optimization techniques to analyze and construct credit portfolios, as well as
+asset allocation methods that account for illiquid assets. The class aims to
+provide economic intuition as well as quantitative tools for managing credit
+portfolios. 
+The course will benefit students who are interested in asset management,
+banking, investment banking, financial consulting, as well as corporate
+Treasurers and risk managers.</t>
         </is>
       </c>
     </row>
@@ -74889,7 +75990,86 @@
 your request and indicate the more advanced class you will be taking instead
 of 35000.  
 Frequently asked questions about Kashyap’s B35200 (Corporation Finance)
-How does your course differ from other instructors?</t>
+How does your course differ from other instructors?
+We all cover roughly the same material, so I think that many of the differences
+come down to style. I think that I probably put more emphasis on teaching you
+how to value companies than some of the other instructors. Most of the  cases
+I use involve valuation. Some of the other instructors include cases on other
+topics too. I also suspect that more of my examples are international (because
+of my research interests related to Japan and Europe). I teach the case on the
+Lehman Brothers bankruptcy in the last week of the class because it is a good
+advertisement for several of the advanced corporate finance electives.  
+Can I take 35000 concurrently?
+No that won’t work. By the second week of the term we will be using the CAPM
+and in week 3 we cover real options. You need to have completed 35000 (or an
+equivalent course) to keep up with what we will be doing.
+What have you changed since the last time you taught the course?
+I am updating a number of the examples and revising the lecture on real
+options significantly. The basic material for this class is pretty timeless.
+Why do you grade the cases?
+Because I have experimented with both grading them and not grading them
+and when they are not graded people do not take them seriously. The course is
+organized so that the cases really reinforce concepts. If students do not work
+hard on the cases then they are not going to fully learn the material. The 21
+percent weight in the overall grade is enough to penalize people who shirk but
+not hurt people who make a sincere effort.
+Why can’t all the case write-ups be done in groups?
+I require some individual effort for the same reason that I grade them in the
+first place. Having a group where the members take turns doing the work
+undermines the learning. I encourage you to discuss the cases, but I want
+everyone to have made a serious attempt on their own before any discussions
+start.
+Why don’t you give out solutions to the cases?
+I (and other instructors) want to be able to use these cases in the future. If the
+answers are distributed they will find there way into future students hands and
+ruin the cases. The handouts that I provide include all the material that you
+need to match the computations that I show.  The TA will  go over the details of
+what I put up in class in the review sessions (or with you individually or in
+groups). 
+Do I have to go to the review sessions?
+No. If you are following the lectures and understanding the homework, then do
+not bother with the reviews. If you have questions, particularly on the
+homework, these sessions are designed to help.
+How should I study for the exams?
+Start with the takeaway slides that are at the end of each lecture. You
+absolutely need to understand these points. You should then make sure you
+understand how we solved the major problems worked out in class. Finally,
+you should do the homework. If you can do all the homework problems too
+(including the case write-ups), then you will do well in the class. If you do not
+do this you are going to have trouble. The best way to check that you are ready
+is to take one of the exams from prior years that are posted on the course
+chalk web site.
+I missed class what should I do?
+Review the lecture notes carefully and then try to do the homework. If you can
+do the homework and follow the notes you should be fine. You should make a
+point of also looking over the notes of someone who was in the lecture to
+make sure you find out what I stressed. Similarly, be sure to see Alissa Aviles to
+pick up any handouts you might have missed. (If you can attend one of the
+other sections, please do that.)
+I missed an exam, can I reschedule it?
+No. It is very hard to write a fair exam and without large numbers of people
+taking an exam you cannot tell whether a makeup would be fair.
+Can I take the final early or late?
+No. I won’t have the exam written until the night before so there is no time to
+give it early. Controlling information after the exams becomes hard and I don’t
+think it is fair to permit people to take it later. If you cannot make it at the
+scheduled time find another section. (If you do miss the final you will be given
+an incomplete that you can make up by taking the final in Spring quarter.)
+Where is your office?
+Campus office is HPC 529.  When teaching at Gleacher, I grab the first office
+that I can find in the suite of faculty offices on the 4 floor.
+th
+Where are the questions for the cases?
+They are posted in Canvas.
+Do I need to buy the book?
+I realize it is expensive, but it is an excellent resource and you will be at a
+definite disadvantage if you cannot do the assigned reading. I assign very little
+reading with the presumption that you will actually do it.
+Why should I take this class?
+Knowledge of this material is essential for anyone who hopes to run a
+business. If you do not understand how to finance a company you are very
+likely to make poor management decisions. For the students who are going to
+concentrate in finance this is the foundations course to help you get ready.</t>
         </is>
       </c>
     </row>
@@ -74982,7 +76162,21 @@
 trajectory of macroeconomic crises. This course studies the design of
 consumer financial products and how business leaders more broadly can
 respond to consumers’ financing needs. 
-We begin with recent innovations in consumer finance, including FinTech</t>
+We begin with recent innovations in consumer finance, including FinTech
+business models related to underwriting, ML/AI, and alt-data, as well as recent
+developments in more traditional financial services. We then ask what makes
+these innovations successful – or not. Three main themes emerge. The first is
+an understanding of consumers’ finances: how do the risks, income, wealth,
+and decision-making of consumers affect their financial needs? The second is
+the role of the competitive and regulatory environment: market forces such as
+adverse selection are shaped by regulation and by competition, and these
+crucially affect what financial products are viable. The final theme is the
+benefits, and risks, of new technology, including ethical concerns that arise in
+the debate around financial inclusion. 
+Particular applications and markets studied in the course include credit
+scoring; ML/AI in underwriting; mortgages and rental housing; credit cards;
+student loans; regulators, banks, and non-banks in the US financial system;
+and high-risk products and consumer financial distress.</t>
         </is>
       </c>
     </row>
@@ -75022,7 +76216,15 @@
       <c r="I121" s="2" t="inlineStr">
         <is>
           <t>This course will explore the challenges of corporate finance and investment in
-an integrated (and possible de-globalizing) world economy. How should one</t>
+an integrated (and possible de-globalizing) world economy. How should one
+optimally organize the location of production, control, and financing? What
+kinds of new concerns emerge when the whole world, rather than just one's
+domestic economy, becomes the arena of decision making? How does
+corporate decision making depend on the environment one is doing business
+in? In a world that is changing fast, this course will focus on finance and
+economics, but also on geo-politics, climate change, automation, and other
+important issues confronting us today. We will also have optional guest
+lectures outside class.</t>
         </is>
       </c>
     </row>
@@ -75139,7 +76341,16 @@
 course focuses on drafting credit investment memos, where students
 investigate a company in detail to make a recommendation on originating a
 credit or investing in a credit in the secondary market. The last part of the
-course covers the rich strategic actions taken by investors in the leveraged</t>
+course covers the rich strategic actions taken by investors in the leveraged
+finance market, including liability management exercises (LMEs) and the details
+of out-of-course restructuring (distressed debt exchanges) and in-court
+restructuring (Chapter 11).
+This class is designed for students in all finance and consulting fields, but with
+a particular focus on those who want to work in financial management of
+firms, private credit, private equity, banking, corporate restructuring,
+turnaround advising, or fixed income investing. Many law students also take
+the class, given the heavy overlap of finance and legal considerations in this
+area.</t>
         </is>
       </c>
     </row>
@@ -75174,7 +76385,13 @@
       <c r="I124" s="2" t="inlineStr">
         <is>
           <t>This is an advanced course covering a variety of special topics. These topics
-should include: Understanding financial crises and the role of banks; Investor</t>
+should include: Understanding financial crises and the role of banks; Investor
+sentiment, anomalies, and market efficiency; The money management
+business and the inherent limitations of professional arbitrage; The role of
+cross-country institutional differences in explaining differences in financial
+markets and access to finance; Finance and rent-seeking: Are financial people
+overpaid?; Implications of asset price volatility for corporate finance, including
+merger waves and financial innovation.</t>
         </is>
       </c>
     </row>
@@ -75307,7 +76524,30 @@
 students interested in entrepreneurship, venture capital (VC), or private equity
 (PE)—especially growth equity—in global markets. Weekly sessions feature
 high-profile guest speakers (both founders and investors), allowing students to
-connect classroom frameworks to current practice.</t>
+connect classroom frameworks to current practice.
+The “Emerging Markets Finance and Entrepreneurship” course (EMFE) is
+organized around the life cycle of firm growth and investment in emerging
+markets, progressing from the macro and institutional context to financing
+mechanisms, deal structuring, and value realization. We begin by examining
+why emerging markets remain “emerging,” then turn to the entrepreneurial
+finance ecosystem and the different sources of capital available to founders.
+The middle section focuses on financing growth, studying how investors
+structure and manage capital across stages, sectors, and risk profiles. The final
+weeks move to exits and fund dynamics, analyzing how investors create and
+capture value and how limited partners and general partners structure their
+relationships. We will conclude with a wrap-up session and discussion of
+recent trends relevant to entrepreneurs and investors.
+The goal of the course is not to become experts on particular countries or
+regions but rather to train ourselves in the use of principles that can be
+applied to evaluate entrepreneurship and investment opportunities across
+many countries, markets, and sectors. Ultimately, the goal is to ensure you
+leave the course comfortable navigating and analyzing the rapidly expanding
+entrepreneurial finance ecosystems across emerging markets. Our case lineup
+spans a wide range of regions: four cases on Latin America, three on Asia, two
+on Africa, one on emerging Europe, and three at an international scale.
+NO SYLLABUS AVAILABLE
+Description and/or course criteria last updated: December 05 2025
+DISTRESSED DEBT INVESTING</t>
         </is>
       </c>
     </row>
@@ -75697,69 +76937,20 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>SCHEDULE
-Note: If the above link to my faculty page is not working, please click on this
-link.
-PLEASE REFER TO THE COURSE SYLLABUS FOR MORE DETAILS; if you have any
-questions about this course, please do not hesitate to email me
-at philipp.afeche@chicagobooth.edu
-OVERVIEW AND LEARNING OBJECTIVES
-The modern business world presents managers with important and
-challenging decision problems that involve complex situations, uncertainty and
-many possible options. This course focuses on managerial decision problems
-that are amenable to quantitative analysis.
-This course teaches how to systematically structure, model, analyze and
-ultimately solve such managerial decision problems using Excel spreadsheets.
-We consider problems from business areas including operations, marketing,
-finance, and strategy. For each business problem we discuss how to build an
-appropriate mathematical model to structure and formulate the problem; how
-to analyze and solve the model; and how to analyze and discuss the
-managerial interpretation of the solution.
-This course takes a practical approach that focuses on modeling, analysis and
-interpretation, rather than on developing the underlying theory or algorithms.
-We develop and use Excel spreadsheets as a modeling platform, because
-spreadsheets have become an essential medium of business analysis. Using
-Excel commands, functions, and add-ins, you learn how to select, apply and
-interpret the solution of the appropriate analytical tool, including optimization,
-simulation, and decision trees. This practical approach has proven to be
-accessible and effective for managers, who find spreadsheets to be an intuitive
-and user-friendly platform for business analysis.
-In sum, you will learn how to:
-Structure a decision problem: identifying the objective, decision
-alternatives, input parameters, and sources of uncertainty.
-Build a mathematical model to formalize the decision problem:
-Optimization models (linear, nonlinear) - for resource allocation (how
-to utilize available resources optimally)
-Simulation models - for risk analysis and incorporating uncertainty in
-problem parameters
-Decision tree models - for multiperiod sequential decision making.
-Analyze the model solution: Is the decision fairly robust, or very sensitive
-to the input parameters of the model ? What is the managerial
-interpretation of the model solution?
-Use Microsoft Excel as a platform for model building, solution, and
-analysis: Spreadsheets are a useful medium for learning the decision
-modeling concepts mentioned above without the large time investment of
-learning a general purpose programming language (like Python). In
-addition to standard Excel tools such as Goal Seek and Data Table, we will
-use add-ins such as Solver, SolverTable, Precision Tree, and @RISK. This is
-NOT a course for learning Excel, the students will be expected to go
-through a introductory tutorial of Excel before the first class. 
-The classes will comprise mini-lectures to introduce the modeling and
-analytical concepts, followed by an interactive discussion of a few (3-5)
-representative problems. We will develop the models for these problems and
-implement, solve and analyze them in Excel.
-Spring 2026
-Section: 36106-01
-T 8:30 AM-11:30 AM
-Harper Center
-C05
-In-Person Only
-Spring 2026
-Section: 36106-02
-T 1:30 PM-4:30 PM
-Harper Center
-C05
-In-Person Only</t>
+          <t>BUS 36106 is designed to sharpen students’ analytical skills and elucidate
+quantitative modeling as an aid in managerial decision-making. This new
+version of the course teaches various ways to frame, set up and solve
+managerial questions about resource allocation, revenue management,
+finance, marketing, operations, risk analysis, data analysis, and forecasting
+using Microsoft Excel, as well as various tools and add-ins. The course will
+introduce various modeling frameworks and analytical tools in optimization,
+simulation, and data analysis. Students in this course will become proficient in
+formulating relevant managerial questions in the language of optimization and
+simulation modeling, as well as in solving the resulting problems using the
+frameworks covered in the course and interpreting the results. The course
+involves hands-on active learning through in-class cases and examples,
+homework and term project which applies the tools and modeling frameworks
+learned in the course to a business problem.</t>
         </is>
       </c>
     </row>
@@ -75810,7 +77001,39 @@
 of Uber drivers to customers. There are various options for us to consider of
 how to model such a decision. And with our ability to utilize Google’s API to get
 travel time data we are able to build a decision tool that can be used in the
-enterprise.</t>
+enterprise.
+We will also learn how to build discrete event simulations with Python. This is a
+very powerful tool that can be used to simulate countless processes. For
+example, how items flow through a logistical system, customers through a
+restaurant or hospital, or a disease through a community.
+The class is a mix of modern programming tools and decision modeling. As
+such, the class can be, depending on your background, challenging and time
+consuming. Bus 36106 (Managerial Decision Modeling) is a suggested
+prerequisite for this class. A student may skip Bus 36106 if they have a good
+background in Linear Programming and basic probability and statistics (an
+Industrial Engineering major for example). Students should also have exposure
+to a modern object oriented programming language (Bus 36110 or Bus 32100
+is one way to gain such experience). For students with programming
+experience but new to Python, there is a series of tutorials available on Canvas
+to work through before our first class.
+This class is a natural follow-on to Bus 36106, Managerial Decision Modeling.
+Bus 36106 is constrained by the tools available within Excel and its limited
+ability to interact with all the information available from the internet.
+This class is also a natural companion to Bus 36110, Application Development.
+Whereas Bus 36110 covers the full-stack building of web applications, it does
+not delve into the decision making or algorithmic needs of the enterprise. A
+student who has already taken Bus 36110 will find it easy to utilize their
+knowledge of the internet and object oriented programming for this class, and
+be ready to focus on decision modeling.
+Please note that the use of ”Advanced” in the course title does not pertain to
+Python. We will not cover advanced concepts of the Python language. In fact, I
+will stick to the basics of the language so that the course is accessible to
+students with only an introduction to programming in any modern language.
+The ”Advanced” better describes that using Python rather than Excel for
+decision modeling is more challenging and advanced in its capabilities. And
+”Advanced” describes the types of models we will be able to examine here vs.
+Bus 36106 (for example stochastic optimization and discrete event simulation).
+Review the syllabus for more detailed information.</t>
         </is>
       </c>
     </row>
@@ -75868,7 +77091,40 @@
 — functions.
 2. Communicate more credibly with developers on our teams.
 3. Grow an eye for problems that can be solved with technology.
-4. Prioritize features more prudently by developing a better feel for their costs.</t>
+4. Prioritize features more prudently by developing a better feel for their costs.
+5. Research and specify changes we want made to products more clearly.
+6. Be empowered with a new, powerful, and just plain fun creative outlet.
+Course Format
+This course is entirely project-driven. We will build a series of applications
+together in class. We will start with a simple idea and learn just what we need
+about various technologies (HTML, CSS, Ruby, Rails) to make that idea real.
+We will then build a slightly more complicated idea, and deepen our
+knowledge of each topic. And then an even more complicated idea. In this way,
+we will spiral across topics picking up essential, applicable knowledge; what
+we're not going to do are deep theoretical dives into each topic, one after the
+other, without ever getting to build real stuff.
+In addition, you will build your own app idea. During the first few weeks, you
+will think of a few of your ideas and we'll then, together, select one that
+matches the scope of the course. This app will be your final project.
+The process will generally consist of the instructor demonstrating a concept in
+a tutorial app and then giving the class a challenge to practice it and think up
+questions. You are strongly encouraged to team up and work together on the
+challenges.
+Expectations
+This course is designed for a beginner who has never programmed before. It is
+our goal to make programming accessible to as many people as possible, and
+dispel the mystique that surrounds it. It's really possible, with passion and
+persistence, for a beginner to become productive very quickly with today's
+tools.
+Note: it's possible, but not always easy. If you have never seen a line of code
+before, you are going to be learning a lot of new things all at once, and so
+should plan to spend a significant amount of time. If you already have some
+programming experience, you may have to spend less time initially while we
+learn basics; but once we get into Rails, it will likely be all new to you too.
+What you can expect from us in return is a lot of support. We know it's a lot,
+and we're here for you -- one-on-one appointments, review sessions, etc. We
+all will help each other on the class discussion board. There is no such thing as
+a dumb question; we're all beginners here, learning together.</t>
         </is>
       </c>
     </row>
@@ -75916,7 +77172,16 @@
 With that, you will be well-positioned to join the community of professional
 developers, and continue learning whatever you need to ship your ideas on
 your own.
-Specifically, we will:</t>
+Specifically, we will:
+-Learn more advanced and concise ways to use the Ruby language and the
+Rails framework.
+-Write automated tests, which are essential for the long-term performance and
+code quality of a project.
+-Learn JavaScript, which will enable us to improve the responsiveness of our
+applications with real-time updates.
+-Add robust APIs to our applications, to enable additional third-party or first-
+party clients.
+-If time permits, add native iOS and Android apps using a hybrid framework.</t>
         </is>
       </c>
     </row>
@@ -76007,7 +77272,12 @@
 outcomes are subject to stochastic variability. Dynamic Programming (DP)
 provides a powerful tool for obtaining structural insight about, as well
 computing prescriptions for, such decisions. The method finds wide
-application in operations management, marketing, economics, and finance</t>
+application in operations management, marketing, economics, and finance
+among other fields. This course is intended to provide a rigorous introduction
+to the method with an emphasis on applications from these fields. When
+appropriate, finite or countable state Markovian settings will be used to obtain
+theoretical results with a minimum of technical fuss. Implementation and
+computational issues will be discussed.</t>
         </is>
       </c>
     </row>
@@ -76114,7 +77384,15 @@
         <is>
           <t>This course covers basic concepts and methods in applied probability and
 stochastic modeling. The intended audience is master's and doctoral students
-in programs such as Computer Science, Statistics, Mathematics, and those in</t>
+in programs such as Computer Science, Statistics, Mathematics, and those in
+the MS/OM Ph.D. in Booth School of Business. In terms of prerequisites, basic
+familiarity with probability theory and stochastic processes will be assumed.
+The exposition will be (mostly) rigorous, yet intentionally skirting some
+measure-theoretic details; for those interested in such details they can be
+found in measure theoretic textbooks and other courses (e.g. Measure
+Theoretic Probability sequence offered by the department of Statistics). A
+unifying theme in the course will be the use of asymptotic methods which
+constitute a powerful tool for the study of complex stochastic systems.</t>
         </is>
       </c>
     </row>
@@ -76200,7 +77478,17 @@
 the last 25 years and hope that students will also share their experiences in
 class discussions. Finally, in order to expose you to different types of marketing
 careers where concepts taught in this class can be leveraged, I typically invite
-1-2 guest speakers from a variety of industries.</t>
+1-2 guest speakers from a variety of industries.
+I strive to enhance student problem-solving and decision-making abilities and
+use marketing case studies to provide an opportunity (both written and oral) to
+help a student develop, present, and defend their own recommendations, and
+to examine and discuss the recommendations of others critically. Given the
+rigorous and highly interactive nature of class discussion, as well as
+framework-based approach used, this class is helpful to students for case
+analysis preparation. Therefore, in addition to students pursuing marketing
+careers, this class is also helpful to students pursuing consulting careers,
+developing entrepreneurial businesses, or interested in understanding and
+analyzing growth and demand strategies of a corporation.</t>
         </is>
       </c>
     </row>
@@ -76242,7 +77530,33 @@
           <t>The purpose of this course is to inform future managers, analysts, consultants,
 and advisors of the psychological processes and biases underlying consumer
 behavior, with emphasis on how to incorporate such insights into marketing
-and business strategies. Contemporary approaches to business emphasize the</t>
+and business strategies. Contemporary approaches to business emphasize the
+importance of adopting a customer focus. Marketing, in particular, begins and
+ends with the consumer—from determining consumer needs to providing
+post-purchase satisfaction.
+Of course, successful marketing and business strategies depend on a thorough
+understanding of how people think, and thus the overarching goal of this
+course is to help you think differently (and better) about how consumers arrive
+at judgments and choices and how their choices ultimately affect their well-
+being. You might think that, because you’re a consumer (we all are), your
+intuitions about the drivers of consumer behavior (including your own) are
+well-informed, but in fact, your intuitions about this stuff are often inaccurate.
+To remedy this problem, this course gives students a broad overview of
+important results from various behavioral sciences (e.g., psychology,
+marketing, economics) that clarifies how and why people perceive and process
+information, make decisions, and evaluate stuff the way they do.
+The greater understanding of consumer psychology provided in this course will
+help students to develop strategic consumer insights aimed at better meeting
+people’s needs. Moreover, because this course takes a broad psychological
+perspective, it highlights novel ideas for grabbing attention, shaping behavior,
+and changing people’s minds within and outside of traditional marketing
+contexts. Also, notably, people everywhere (i.e., not only marketers, but almost
+everybody you know) are trying to influence you all the time. This means that
+the issues covered in this class are not only of concern to marketing managers,
+but to you personally, as gaining an understanding of these issues helps you
+better understand yourself as a target of influence. The premise of the course
+is that understanding consumer psychology has powerful business and
+personal implications.</t>
         </is>
       </c>
     </row>
@@ -76366,7 +77680,10 @@
 37103 (Data-Driven Marketing). However, we will cover these topics at a faster
 pace and emphasize state-of-the-art techniques that are only briefly surveyed
 or not covered in 37103. Also, the main goal of the data assignments in 37103
-is to make the students familiar with some key concepts in data-</t>
+is to make the students familiar with some key concepts in data-
+driven marketing. This class goes above and beyond this goal and introduces
+the students to a professional data scientist’s workflow used for marketing
+decision-making.</t>
         </is>
       </c>
     </row>
@@ -76412,7 +77729,28 @@
 opportunity identification, qualitative and quantitative agile user research,
 customer insights, idea generation and evaluation, new product
 prototyping/testing/optimization, forecasting, new product branding, and
-business cases.</t>
+business cases.
+A series of group projects enables students to apply these tools on an actual
+client “Lab” project. Group projects are real-world innovation projects from
+leading company sponsors across a range of industries. Student teams work
+closely with their clients, guided by a faculty coach, to uncover unmet
+customer needs, generate ideas, develop new product/service concept
+prototypes, test those new product concepts quantitatively, and present
+recommendations to their clients.
+This course covers tech, consumer, and B2B products and services. Class
+examples and cases include mobile apps, e-commerce, software, fintech, food
+and beverage, household products, healthcare, and more. I make every effort
+to invite one or more practicing innovation experts to guest lecture.
+This course is particularly relevant for students interested in the following
+careers: Product Management (Tech), Management Consulting, Brand
+Management, Innovation, Product Marketing Management (Tech), and
+Corporate Strategy.
+Winter 2026 Application Timeline:
+Tuesday, November 4 at noon-1pm:  Webinar to give details about the
+class and application process.
+Wednesday, November 5 at midnight:  Applications are due.
+Tuesday, November 11:  Acceptances are announced. Students have 24
+hours to drop. After that, no drops are allowed.</t>
         </is>
       </c>
     </row>
@@ -76454,7 +77792,46 @@
           <t>The surge in access to detailed marketing data and analytic tools has elevated
 pricing to the forefront of corporate strategy and the driving force of strategic
 revenue growth. Emerging roles like the Chief Growth Officer (CGO) and Chief
-Revenue Officer (CRO) focus predominantly on pricing decisions. For most</t>
+Revenue Officer (CRO) focus predominantly on pricing decisions. For most
+companies, improving pricing strategy represents both a strategic goal and a
+strategic challenge. Most struggle with the same basic questions: How do we
+formulate a pricing strategy? What should we charge? Which data and
+methods should we be using to make pricing decisions? Who should be in
+charge of pricing decision-making?
+In practice, most firms still use ad hoc rules-of-thumb. The simplicity of these
+rules comes at a substantial cost to a firm’s potential profitability. Most rules
+fail to align pricing with consumers’ perceived value and underlying
+willingness-to-pay. Many firms also struggle with the delegation of pricing
+responsibility within the organization, exacerbating the use of rules-of-thumb
+that fail to deliver effective pricing decisions and monetize. The fact your
+company makes money does NOT confirm the optimization of your prices: you
+may be leaving substantial money on the table.
+This course blends marketing analytic frameworks, marketing strategy,
+microeconomic theory and customer data to formulate actionable, evidence-
+based pricing strategies. Students learn how to coordinate pricing decisions
+with the rest of the marketing value proposition. Numerous pricing structures
+are developed in the course, along with their microeconomic foundations. 
+Students learn the underlying theory for each pricing structure, along with the
+practical considerations for implementation. In several modules, students will
+use statistics and AI to implement optimized pricing decisions.
+The course combines cases and analytic assignments to teach students how to
+design and execute pricing strategies. Students work with different forms of
+data and corresponding analytic methods. The examples span a wide array of
+business contexts including services, B2B and international.
+During the quarter, there are 4 group homework assignments, 3 group case
+write-ups and 1 individual case assignment. Week 1 attendance is
+mandatory. The individual assignment is due during week 3. If you register late
+for the course, you must still submit this first assignment in class during week
+3. Failure to submit this assignment will result in a grade of zero and no
+exceptions will be made. Provisional grades can be assigned so long as
+students complete all the assignments during the quarter.
+For some of the group homework assignments, you will need to run a
+regression and/or use optimization software. Two review sessions have been
+scheduled with one of the course TAs to assist those students who are
+unfamiliar with these techniques.
+For the group assignments and group case write-ups, students need to form a
+group of 4-5 people. All group members must be registered for the same
+section. No exceptions will be made.</t>
         </is>
       </c>
     </row>
@@ -76500,7 +77877,9 @@
 concepts and use them to develop marketing strategies. You will develop this
 understanding through core readings, basic frameworks, and case studies
 involving firms such as Procter &amp; Gamble, Drunk Elephant, Coca-Cola, Unilever,
-Porsche, Nestle, Sephora, and Glossier.</t>
+Porsche, Nestle, Sephora, and Glossier.
+This course is relevant for students interested in driving consumer demand
+regardless of career path. There are no prerequisites.</t>
         </is>
       </c>
     </row>
@@ -76559,7 +77938,23 @@
 traditional marketing strategies can be adapted or restrained in light of
 purpose-driven aims. Throughout, we will analyze cases, hear from guest
 speakers, and draw on academic and industry research as well as recent
-events. The final deliverable will be a marketing plan that articulates a firm</t>
+events. The final deliverable will be a marketing plan that articulates a firm
+strategy capable of increasing societal benefit while also creating shareholder
+value.
+Course Objectives:
+Critically evaluate the business case for doing well by doing good, and the
+potential benefits and risks for businesses, shareholders, and other
+stakeholders
+Learn how to select priorities and focus areas when developing purpose-
+driven strategies in the context of profit-seeking firms
+Understand consumer preferences for purpose-driven brands, and how to
+leverage these preferences to create value
+Learn principles of behavior change and how businesses can help their
+customers directly
+Effectively brand and communicate a company’s values and the value that
+they create - understanding when it is advantageous to do so
+Develop business strategies that align with broader societal goals,
+ensuring long-term sustainability and value creation for all stakeholders</t>
         </is>
       </c>
     </row>
@@ -76607,7 +78002,26 @@
 for technology-based products. We will trace the historical evolution of Product
 Management, examine alternative organizational designs, and develop a
 rigorous understanding of the product manager’s craft, competencies, growth
-journeys, tools, and strategies to overcome challenges. The focus of this course</t>
+journeys, tools, and strategies to overcome challenges. The focus of this course
+is specifically on digital product management and the modern Product
+manager tech stack, providing a practical integration of product, design, data,
+engineering, leading cross-functional teams and going to market.
+The course emphasizes both analytical and managerial decision-making,
+including:
+Identifying and framing customer and business problems appropriate for
+product-led solutions.
+Designing product vision, strategy, and roadmaps under resource and
+organizational constraints.
+Prioritizing initiatives using data, experimentation, and financial reasoning.
+Managing product development, measurement, and iteration across the
+product lifecycle, including the emerging use of AI-enabled tools.
+Leading without authority through influence, storytelling, and cross-
+functional collaboration.
+The course uses a combination of case discussions, frameworks, applied
+exercises, and a team project in which students plan a product from concept
+through launch and evaluation. Students will leave the course with practical
+tools and a structured perspective for leading product-driven organizations
+and initiatives in both established firms and entrepreneurial settings.</t>
         </is>
       </c>
     </row>
@@ -76744,7 +78158,34 @@
 now expected to know how to select, deploy and use a variety of marketing
 software platforms &amp; services, including the latest AI-based platforms &amp; tools.
 As of last count, there are over 15,300 MarTech applications in 49 categories
-including advertising (AdTech), content marketing, marketing automation, sales</t>
+including advertising (AdTech), content marketing, marketing automation, sales
+automation, websites, social media, sales intelligence, and analytics. The best
+way to gain such expertise is for these professionals to actually build and
+execute specific digital marketing programs/strategies using various MarTech
+platforms in a lab environment.
+This lab course, DML, takes students through the process of designing and
+executing specific digital marketing program components, hands-on. They will
+work with several marketing platforms and tools including some newer AI tools
+such as ChatGPT,  for creating and managing digital presence, content and
+SEO, paid search and social media advertising, marketing analytics, &amp; other
+aspects of digital marketing.
+By the end of the course, students will have learned how to utilize key MarTech
+platforms, AI tools, and several frameworks to build out digital marketing
+programs, and by so doing, they will develop a deep understanding of what it
+really takes to design and execute digital marketing strategies and campaigns
+on their own. This course is primarily targeted at students (i) that are
+interested in marketing, MarTech and AdTech, (ii) that are aiming to be product
+managers, and (iii) that wish to start or join entrepreneurial ventures.
+Registering for this course is strictly by application only. As this is a lab course
+where students will be executing real-life projects with real companies, there is
+a limit on the number of student slots. We will host a Webinar on Friday, Aug
+15 at 12:00 Noon, Central Time. In this webinar we will provide details about
+this Lab,  the various class assignments &amp; projects that the students will
+execute, and the application process. At that time, the application form for this
+course will be made available here and via email. Details regarding the webinar
+will be made available to students a week to 10 days in advance via email.
+Once accepted into the course, students will have 72 hours to decide before
+they will be registered. Once registered, students may not drop the course.</t>
         </is>
       </c>
     </row>
@@ -76856,7 +78297,11 @@
 students are expected to read, assimilate, and discuss multiple papers on
 specific topic areas each week. Each student is expected to lead the discussion
 for an entire topic once or twice in the quarter. Responsibilities will include
-assigning discussion questions for the week, allocating readings to specific</t>
+assigning discussion questions for the week, allocating readings to specific
+classmates for detailed discussion, and synthesizing the discussion across
+readings to develop an integrative framework for research in the topic area at
+the end of that session. Students are also expected to generate research ideas
+and write a paper for the course.</t>
         </is>
       </c>
     </row>
@@ -77007,13 +78452,8 @@
       <c r="H168" t="inlineStr"/>
       <c r="I168" s="2" t="inlineStr">
         <is>
-          <t>SCHEDULE
-Spring 2026
-MARKETING RESEARCH SEMINAR (SPRING) (37912, 50 UNIT COURSE) - KRAFT,
-ANDREAS&gt;&gt;
-MANAGERIAL PSYCHOLOGY (38000) - GINZEL, LINDA&gt;&gt;
-Intensive year-long research and writing seminar for Booth Marketing PhD
-behavioral students in the 3rd year and up.</t>
+          <t>Intensive year-long research and writing seminar for Booth Marketing PhD
+quantitative students in the 3rd year and up.</t>
         </is>
       </c>
     </row>
@@ -77043,7 +78483,11 @@
 individual, interpersonal and group behaviors as they relate to organizational
 performance using the lens of social psychology. We will work together to
 develop a more complex understanding of processes such as motivation, social
-perception, interpersonal influence, effective communication, interpersonal</t>
+perception, interpersonal influence, effective communication, interpersonal
+problem solving, group decision making, commitment, and leadership. Using a
+combination of case discussions, demonstrations, role-plays, group activities,
+and lectures, our primary goal is to offer conceptual frameworks and principles
+that will help to improve your managerial and leadership effectiveness.</t>
         </is>
       </c>
     </row>
@@ -77172,7 +78616,22 @@
       <c r="I172" s="2" t="inlineStr">
         <is>
           <t>Every effective manager needs to know how to wisely manage power and
-influence. Skill in doing so enables managers to win the cooperation of others,</t>
+influence. Skill in doing so enables managers to win the cooperation of others,
+to elicit the most value from diverse organizational resources, and to
+consistently achieve goals.
+In this class, you will be introduced to conceptual models, tactical approaches,
+and self-assessment tools that can help you to manage workplace power
+dynamics more wisely and skillfully. You will learn about several different
+methods of influence, and start the process of understanding and shaping
+your own influence style. You will also explore specific, real-world examples to
+understand how power and influence might be effectively and ineffectively
+used at different stages of a person’s career. As the nature of our focal topics
+will raise difficult ethical questions, the course will also challenge you to
+examine and define your views on what will constitute the ethical exercise of
+power and influence in your work life.
+Readings in this class are extensive. Preparing thoroughly for class discussions
+and exercises with these weekly readings is essential for getting the most value
+from the class.</t>
         </is>
       </c>
     </row>
@@ -77212,7 +78671,14 @@
 benefit from feedback. In the early class sessions, we introduce basic
 negotiation concepts and tactics. In the classes that follow, we focus on specific
 aspects of the negotiation process that are important to many negotiation
-situations, such as obstacles to effective communication at the bargaining</t>
+situations, such as obstacles to effective communication at the bargaining
+table, the maximization of multiple interests, and tactics for coalition building.
+In the final set of classes, we put it all together by exploring negotiations that
+contain elements of both cooperation and competition; that is, these sessions
+involve cases where the parties can “enlarge the pie” by creating joint gains.
+Because little in business (or life) gets done without negotiation, this course
+has the potential to deliver significant upside in your professional and personal
+outcomes.</t>
         </is>
       </c>
     </row>
@@ -77247,7 +78713,29 @@
       <c r="I174" s="2" t="inlineStr">
         <is>
           <t>This course builds on 38103, Strategies and Processes of Negotiation, and is
-designed to increase your understanding of the theory and process of</t>
+designed to increase your understanding of the theory and process of
+negotiation.
+The course will include advanced topics that expand upon or were not covered
+in 38103. In particular, the course will improve your ability to deal with difficult
+negotiators and difficult negotiations. 38103 introduced the basic ideas of
+negotiations—BATNAs, effective tactics for distributive negotiations, processes
+and analytics behind the discovery of joint gains, and coalitional dynamics in
+multi-party settings. This course will discuss advanced concepts of negotiations
+by taking you through a set of negotiation exercises that are more complex
+and more authentic than the ones used in 38103. The exercises will include:
+integrative negotiations without scoring systems, dynamic negotiations,
+complex deal structuring negotiations, sustaining negotiated value, and
+negotiations that require coordination of internal and external parties.
+The more advanced deal making and deal design skills developed in this
+course should be especially useful to students whose careers will involve
+investment banking; business development; venture capital, private equity
+investment, and entrepreneurial firms; and alliances and joint ventures, as well
+as students who anticipate conducting a substantial amount of intra-
+organizational negotiations.
+The course will use a combination of role-playing simulations and case
+discussions that include topics such as strategic alliances; dysfunctional
+business relationships.
+Note: All students must attend the first week of class.</t>
         </is>
       </c>
     </row>
@@ -77415,7 +78903,9 @@
 Course Format:
 This course will involve a combination of lecture, class discussion, in-class and
 out-of-class exercises, and occasional case discussion.  There will be a take-
-home (open-book) midterm exam that you will have two hours to complete</t>
+home (open-book) midterm exam that you will have two hours to complete
+after the Week 5 class session, and a final group paper due at the scheduled
+time of the final exam.</t>
         </is>
       </c>
     </row>
@@ -77512,7 +79002,23 @@
 “pathways” (things like getting heard, getting credit, and getting second
 chances).
 We will also consider barriers to diversity efforts that must be overcome. For
-example, an organization cannot learn and improve without being willing to</t>
+example, an organization cannot learn and improve without being willing to
+acknowledge that current practices may be problematic and being willing to
+experiment with something new. Indeed, even with a good idea, implementing
+it effectively requires buy-in, ally-ship, and rigorous evaluation.
+All are welcome. I hope to encourage learning and dialogue among students
+with a variety of social identities and backgrounds and expect to hear different
+views on how firms can and should address diversity, equity, and inclusion.
+Although the class will foreground race and gender dynamics in the U.S.
+context, we will also consider other dimensions of difference (e.g., class
+background, nationality, LGBTQ identity, religion, disability, and more) and
+reflect on these topics in other countries and cultural contexts. It is vitally
+important for MBA students, who will become the leaders of domestic and
+global companies, to be informed about how to create the conditions that
+enable all people to achieve success. Students who take this course will be able
+to utilize the skills and knowledge taught when making their own career
+decisions, as well as when managing, being managed by, or collaborating with
+others of diverse backgrounds.</t>
         </is>
       </c>
     </row>
@@ -78033,7 +79539,15 @@
 networks of organizations that supply and transform materials and distribute
 final products to consumers. If designed and managed properly, these
 networks can be a crucial source of competitive advantage for both
-manufacturing and service enterprises.</t>
+manufacturing and service enterprises.
+Students will learn how to examine and improve the flow of materials and
+information through this network of suppliers, manufacturers, distributors,
+and retailers in order to match supply with demand (i.e., to get the right
+products to the right customers in the right amount and at the right time). Key
+topics include inter- and intra-firm coordination, incentive design, the impact
+of uncertainty, and the role of information technology. Special emphasis is
+given to understanding how the business context shapes managerial decisions
+regarding the strategic design and management of the supply chain.</t>
         </is>
       </c>
     </row>
@@ -78080,7 +79594,14 @@
 examples from a variety of industries including airlines, hotels, car rental
 agencies, internet/media advertising, entertainment, retailing, energy,
 commodities, freight, and manufacturing will be used to develop skills in
-designing and implementing solutions in different environments.</t>
+designing and implementing solutions in different environments.
+Students will learn how to recognize opportunities for revenue enhancement;
+how to differentiate among types of opportunities; how to segment markets
+while incorporating constrained capacity, opportunity costs, customer and
+competitor response, demand and supply uncertainty, and information
+infrastructure; how to formulate and solve for revenue management decisions
+using constrained optimization; and how to define overall implementation
+requirements.</t>
         </is>
       </c>
     </row>
@@ -78119,7 +79640,33 @@
 services. Lines of inquiry include: How to design and improve a service offering
 for sustained excellence, How to identify and overcome key challenges in
 service delivery, and How to monitor and analyze the performance of service
-entities. We consider a wide range of industries, from traditional services such</t>
+entities. We consider a wide range of industries, from traditional services such
+as restaurants and hospitals to more modern internet-based services, and
+services taken from both the public and private sector.
+We consider a service one in which the customer is involved, actively or
+passively, in the production process, and we strive to understand and leverage
+the role customers play in the process. This course draws on ideas from
+operations management (Bus 40000), but from a different perspective, that
+also includes a behavioral element. This course is a mix of softer more
+qualitative frameworks and more analytical pursuits.
+Our Service Model has four parts: The Service Offering (what customer needs
+and expectations does the service emphasize and which ones will it sacrifice?),
+Firm Value (does the service provide value for the stakeholders), Employee
+Value (does the service provide value to the employees?), and Customer Value
+(does the service provide enough value to customers to encourage them to
+play their role effectively?).
+Process Flows are used to understand the aggregated flow of customers
+through a process to address issues such as capacity utilization, throughput,
+and waiting time. We will cover the basics of process flow analysis that is also
+covered in Bus 40000, but with a focus on service processes. As such, there is
+significant overlap with the content of Bus 40000 (roughly 50%), and so a
+typical student may likely choose to take either this course or Bus 40000. This
+class’s focus on Services is for those students whose interests tend towards the
+end consumer; in comparison, Bus 40000 takes a broader view of Operations
+that include issues of production and supply chain management.
+The course has both cases and lecture. Most cases are intended to provoke
+class discussion, with the purpose of exploring our Service Framework in a
+broad sense, and also delving into particular aspects in more detail.</t>
         </is>
       </c>
     </row>
@@ -78238,7 +79785,9 @@
 Students interested in the Healthcare Analytics Laboratory (Bus 40721) are
 encouraged to enroll in this class. While this course is designed to complement
 the Healthcare Analytics Lab, it is a standalone offering and can be taken
-independently. Students seeking exposure to healthcare business analytics</t>
+independently. Students seeking exposure to healthcare business analytics
+who are unable to make the commitments the Lab requires will find it useful
+preparation for future endeavors.</t>
         </is>
       </c>
     </row>
@@ -78280,7 +79829,27 @@
 healthcare institutions.
 The Laboratory provides students with opportunities to:
 1. Apply and reinforce tools and frameworks developed elsewhere in the Booth
-curriculum</t>
+curriculum
+2. Develop leadership skills and build effectiveness in teams;
+3. Learn a healthcare context deeply through an intensive project experience
+4. Develop proficiency at presenting data analyses to executive audiences
+5. Impact real-world healthcare delivery.
+Thus, the course will help students develop the skills required to successfully
+deliver evidence-based management analytics in the real world. Projects will be
+carefully scoped, and most data will be acquired, before the course begins so
+that students can make steady progress towards clear, attainable goals.
+Students will present milestones every two weeks to the instructional team
+(which consists of the faculty instructor and graduate students who serve as
+project mentors) and, on occasion, to the entire class. Final presentations will
+be delivered to hospital executives and physician leaders.
+The course is for students interested in leveraging the academic rigor of data
+and decision analysis to improve healthcare delivery. It is an excellent course
+for those interested in careers in or related to the healthcare industry, and
+business analytics more broadly.  Students will be prepared for careers as
+consultants, analysts, or managers in the healthcare industry, or in any
+industry or career that relies on data for making important business decisions.
+Application Timeline:
+Applications for Winter 2026 are now closed.</t>
         </is>
       </c>
     </row>
@@ -78654,7 +80223,9 @@
 large-scale testing and false discovery rates, modern regression and model
 choice, machine-learning based classification,
 network analysis, language and topic models, principal components,
-clustering, Bayesian analysis, deep learning, transformers and attention.</t>
+clustering, Bayesian analysis, deep learning, transformers and attention.
+By the end of the course, students will be equipped to perform machine-
+supported intelligent data analysis and communicate findings effectively.</t>
         </is>
       </c>
     </row>
@@ -78807,12 +80378,12 @@
       <c r="I208" s="2" t="inlineStr">
         <is>
           <t>In this Ph.D.-level course, we will discuss statistical methodology with a focus
-on methods used for causal inference.   The course will review basic models
+on methods used for causal inference.  The course will review basic models
 commonly used in social science research (the linear regression model and
 linear IV model) and cover additional topics such as estimation of treatment
 effects when effects may be heterogeneous, workhorse panel data models,
 estimation using flexible/high-dimensional   methods, and group-based
-inference for dependent data.   It is assumed that students have a good
+inference for dependent data.  It is assumed that students have a good
 understanding of linear regression and methods of performing classical
 inference using asymptotic approximations for linear and nonlinear models.</t>
         </is>
@@ -78900,7 +80471,18 @@
 models followed by tools and concepts from artificial intelligence. Students will
 learn how to use deep learning to analyze a variety of complex real world
 problems. Numerous empirical examples from finance, internet analytics, and
-sports are used to illustrate the material covered. Google’s development of</t>
+sports are used to illustrate the material covered. Google’s development of
+deep neural networks and applications will be discussed in detail.
+Emphasis will be placed on understanding concepts of Bayes, AI and Deep
+Learning. The three main topics covered are: (i) Bayesian methods including
+conditional probability,hierarchical models (ii) Artificial Intelligence including
+modern regression methods such as lasso and ridge regression.
+Dimensionality reduction techniques and sparsity are central to data analysis
+(ii) Deep Learning including Neural Nets, Architecture design,Stochastic
+Gradient Descent, speeding up convergence. Throughout business and
+internet applications including machine intelligence, reinforcement learning,
+image and speech recognition will be used to illustrate the wide range of
+applications.</t>
         </is>
       </c>
     </row>
@@ -78956,7 +80538,22 @@
 uncompromising, choices of priors and likelihoods.
 Throughout the course, we will explore key principles that underpin or alleviate
 such choices towards meaningful and theoretically sound Bayesian data
-analysis.</t>
+analysis.
+Lectures will emphasize methodology, computation and theory but will also
+feature several real datasets. The goals is not to provide a compendium of
+techniques but rather to create links between various approaches and to
+explore their applicability in real life.
+The curriculum begins with traditional (parametric) Bayesian statistics and
+progressively advances through nonparametric priors, likelihood-free
+inference, and prediction-driven inference, culminating in some of the most
+cutting-edge research-driven creative developments in Bayes.
+Topics include Bayesian decision theory, Bayesian sparsity, Bayesian machine
+learning and nonparametrics, likelihood-free inference, generative Bayesian
+models, or variational and predictive inference.
+By the end of the course, students will be be able to confidently apply Bayesian
+tools in realworld settings and will have developed the theoretical and
+methodological foundation necessary to pursue both applied and methods–
+oriented research.</t>
         </is>
       </c>
     </row>
@@ -79250,7 +80847,70 @@
         <is>
           <t>This course aims to help students excel in one of the business world's most
 important competencies: the ability to construct and to deliver a powerful,
-influential narrative.</t>
+influential narrative.
+What differentiates those who are more successful interacting with bosses and
+colleagues inside an organization? How do managers create trust and change
+the attitudes and behaviors of their teams? What differentiates the
+entrepreneurs who succeed in raising money from those who fail? Why are
+some companies more successful in attracting and retaining both employees
+and customers? How do companies that are yet to turn a profit command the
+value of billions of dollars? What is the basis for effective lobbying and rule-
+shaping?
+Whether advancing in your career, leading organizations, motivating people,
+creating strong brands, building and sustaining reputations, or working
+effectively with politicians, regulators, and the media – successful managers,
+entrepreneurs, and companies share a few common, potent skills: they
+appreciate the importance of stories, they develop and maintain coherent
+strategic narratives – and they know how to tell them.
+In this course we will study the critical role of stories in driving success in many
+real-life situations. We will gain an understanding of how our reality is
+comprised of stories, we will establish a critical perspective on stories in the
+arenas of business, economics and politics, and we will study the
+characteristics of successful stories and storytellers. All the while, we will
+practice and hone the telling of our own powerful, personal stories.
+Who should take this course?
+MBA students who aspire to lead larger teams, earn promotions, and step into
+senior roles where influence matters as much as analysis. In 2026, technical
+competence is assumed. Analytical rigor is table stakes. What differentiates
+rising leaders is their ability to align people around direction and purpose. As
+responsibility expands, success depends less on having the right answer and
+more on persuading others to act on it.
+This course is especially suited for:
+Students who aspire to become general managers or CEOs and will be
+responsible for shaping organizational direction and public perception
+Founders who must raise capital, recruit top talent, and sustain belief in a
+vision through uncertainty and setbacks
+Consultants and strategists who need to reframe complex problems and
+persuade clients to commit to difficult strategic decisions
+Professionals entering highly regulated or politically visible industries
+where narrative control influences valuation and legitimacy
+Managers seeking promotion who must demonstrate strategic clarity,
+executive presence, and the ability to influence senior stakeholders
+Technically strong students in finance, engineering, analytics, or
+operations who want to strengthen their influence and leadership impact
+Anyone who expects to lead through crisis, organizational change, or rapid
+technological disruption and needs tools to build alignment under
+pressure
+Crucially, the course emphasizes storytelling as an executive capability - not
+simply the crafting of a corporate brand message. Corporate narratives can be
+delegated to marketing departments. Executive storytelling cannot. In
+moments of ambiguity or crisis, stakeholders look to leaders, not logos, for
+clarity. The way an executive explains change, articulates risk, frames
+opportunity, or defines failure often determines whether an organization gains
+alignment or fractures.
+For MBA students scanning the 2026 course catalogue, the question is not
+whether storytelling is useful, but whether it is central to leadership. In an era
+defined by competing interpretations of reality -across markets, media, and
+internal organizations - leadership is as much about meaning as it is about
+metrics. Markets are contests over interpretation as much as over resources.
+Those who can construct and communicate powerful narratives will be better
+positioned to lead in uncertain, politically complex, and fast-moving
+environments.
+This course will feature two guest lectures of leading figures from the industry.
+Students enrolled in this class will have the opportunity to learn and engage
+with guest lecturers who hold, or have held, prominent roles in large
+corporations where they effectively employed their unique storytelling skills.
+Order of topics in class are subject to change, according to guest lecture.</t>
         </is>
       </c>
     </row>
@@ -79296,7 +80956,14 @@
 students will learn about advancing artistic excellence and creative innovation
 while expanding audiences and achieving financial goals. We will survey
 settings in the not-for-profit performing and visual arts. Among the topics
-explored will be governance and management, serving multiple stakeholders,</t>
+explored will be governance and management, serving multiple stakeholders,
+managing fiscal and creative tradeoffs, standing out in real and virtual spaces,
+achieving growth amidst rising costs and diminishing revenues, and adapting
+to rapidly evolving cultural ecosystems. Students will develop their own
+perspectives on the ways in which commerce, creativity, and culture can align
+and collide in the leadership of arts organizations. Students will have the
+opportunity to grapple real-time with the unprecedented challenges facing arts
+leaders today.</t>
         </is>
       </c>
     </row>
@@ -79338,7 +81005,30 @@
 interests, priorities, and perspectives.
 These debates are more complex than determining the feasibility and
 efficiency of a particular solution in lowering emissions.  What are the costs,
-and who pays for them?  What externalities are created by these solutions, and</t>
+and who pays for them?  What externalities are created by these solutions, and
+how are they distributed?  And what happens to the industries and people
+impacted by the current fossil fuel economy, for better or worse?  How
+individuals, firms, markets, and the government come together or grow apart
+in answering these questions requires an examination through both traditional
+Business School tools and the sausage-making of politics, involving the various
+parties with a stake in the game.
+This course will attempt to address some of these issues.  However, this course
+will not focus on the firm’s perspective, which is the customary starting point
+for most Business School courses.  Instead, the course will focus on various
+governmental entities, commonly referred to as “the state.”  The firm
+represents one of the actors that influences and is influenced by the State. 
+However, we will also consider other stakeholders, including policymakers,
+politicians, financiers, lobbyists, workers, communities, and advocates.  As
+politics is an exercise in coalition building, how these actors work with or
+against each other is critical to understanding the potential solution set while
+also considering the disproportionate way climate change impacts particular
+communities and people.  To that end, the interests of a traditional profit-
+maximizing firm may conflict with those of others.
+As many students will soon be entering firms, it will be essential to align the
+fundamentals of how a firm’s agenda aligns and conflicts with the needs and
+goals of various stakeholders who also have a voice.  The course aims to
+support students in this endeavor in the field of climate and energy, but the
+skills learned apply to any regulated industry.</t>
         </is>
       </c>
     </row>
@@ -79462,7 +81152,25 @@
 influence, collaborate with, or challenge them.
 Who Should Take This Course?
 Consultants and strategists who advise organizations operating in
-complex, high-visibility markets where perception, policy, and media</t>
+complex, high-visibility markets where perception, policy, and media
+framing directly influence outcomes.
+Entrepreneurs and startup founders who need to understand how media
+narratives, platform dynamics, changing regulation and public sentiment
+affect  valuations, investor confidence, brand legitimacy, and growth.
+Students pursuing roles in technology — who must anticipate how
+algorithms, AI systems, and online discourse shape regulation,
+competition, and reputation.
+Finance professionals and investors who need to evaluate not only
+financial fundamentals but also the regulatory, media, and cultural
+environments in which companies are embedded—factors that
+increasingly determine valuation, risk, and long-term performance.
+Future leaders in highly regulated sectors such as energy, healthcare, or
+financial services, where public opinion, policy agendas, and media
+narratives define both constraints and opportunities.
+Students who want to understand the world more deeply and become
+sophisticated, critical consumers of all forms of media—from traditional
+journalism to social platforms, algorithms, and AI-powered chatbots—
+developing the discernment essential to modern leadership.</t>
         </is>
       </c>
     </row>
@@ -79513,7 +81221,12 @@
 trucks and mobility on demand services. The industry is creating a dazzling
 array of new vehicles – supercomputers on wheels – and over the next decade
 a new multi-trillion industry will emerge with new (and existing) players and
-new business models.</t>
+new business models.
+So, how might all this play out? If history is any guide, we can expect a
+shakeout among market players, resulting in clear winners and losers. With
+billions of dollars at stake, this course offers students a strategic framework—
+The Clockspeed Dilemma—providing fresh ideas and approaches to not only
+survive but thrive during periods of market disruption</t>
         </is>
       </c>
     </row>
@@ -79559,7 +81272,11 @@
 stock exchanges, futures markets, over-the-counter markets, blockchains. Even
 dating apps involve market design.
 This class will cover the key economic principles behind market design and will
-challenge students to invent ways to make markets work better.</t>
+challenge students to invent ways to make markets work better.
+Some of the specific topics we will cover include auction design, matching
+markets, platform economics, financial markets, cryptocurrencies, and
+reputation systems.
+The class will feature a mix of lectures and case studies.</t>
         </is>
       </c>
     </row>
@@ -79605,7 +81322,39 @@
 driven businesses) design strategies, choose business models, raise and
 manage money, measure results, and make trade-offs between impact and
 financial sustainability. We’ll focus on the practical tools leaders use to decide
-what to do, how to do it, and how to grow what works.</t>
+what to do, how to do it, and how to grow what works.
+Many of the basic management ideas you may already know — like marketing,
+operations, and competitive strategy — still apply. But managing for impact
+adds real complexity. Goals are harder to define, success is harder to measure,
+funding doesn’t always come from customers, and stakeholders often have
+very different priorities. These differences matter, and they shape almost every
+major decision leaders make.
+This class is designed as a survey course. You won’t become an expert in every
+topic, but you will build a solid working understanding of how social ventures
+are structured and managed, and where the hardest challenges tend to arise.
+Whether you plan to work in the nonprofit sector, in government, in impact
+investing, or in a mission-driven company, the goal is for you to leave with a
+practical framework for thinking about how impact actually gets delivered —
+not just how it gets talked about.
+Class Structure
+This is a discussion-based, case-driven course. Most weeks, you’ll prepare
+cases and readings and then use class time to apply ideas, debate trade-offs,
+and practice making real-world decisions.
+Across the quarter, we’ll cover how social sector organizations:
+Choose legal and organizational structures
+Design business and funding models
+Define their intended impact and theory of change
+Measure results and learn from data
+Work with boards and governance structures
+Think about growth, scale, partnerships, and systems change
+When helpful, we’ll compare social ventures to traditional for-profit companies
+to highlight what’s similar — and what’s not. The goal is not just to understand
+the tools, but to understand when and why certain tools work better (or worse)
+in impact-driven settings.
+By the end of the course, you should be able to look at a social sector
+organization and assess how well its strategy, funding, operations, and
+governance fit together — and whether those pieces are likely to support the
+impact the organization is trying to achieve.</t>
         </is>
       </c>
     </row>
@@ -79665,7 +81414,7 @@
         </is>
       </c>
       <c r="F226" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G226" t="inlineStr"/>
       <c r="H226" t="inlineStr"/>
@@ -79677,7 +81426,45 @@
 This lab course centers around several live consulting projects that allow
 students to consider the role of the firm in society by exploring the domains of
 Sustainability, corporate social responsibility (CSR), Environmental, Social and
-Governance (ESG), and more.</t>
+Governance (ESG), and more.
+The Winter 2026 course will include three projects, sponsored by Owens
+Corning, ThirdLove, and WM (Waste Management), all focused on elements of
+sustainability and circularity.
+Class time will be about 50% project-based, complemented by cases,
+discussions, and guest speakers who extend learnings beyond the projects.
+There will be some attention to how students work as a team and what you
+learn from that experience. 
+By application only.
+Class sessions are required and will be in-person only with no remote option.
+Final presentations will be held during Week 9 and exam week. There will be
+additional required meetings with your client outside of class, including a
+potential field trip to begin during the lunch hour prior to class and which may
+extend into the evening.
+Attendance at the first class on Tuesday January 6th is mandatory.
+Students will be divided into three assigned groups. Students will have an
+opportunity rank project preference.
+Project descriptions will be updated as available.
+Owens Corning: 
+Owens Corning’s glass reinforcements (GR) business is a leading global
+provider of solutions matching the differentiated needs of the growing
+composites industry. The 2026 project will focus on identifying opportunities
+for Sustaina® Loop, a newly launched product made with recycled glass fiber
+in data center and rebar markets.  In addition to its recycled content,
+Sustaina® Loop has a 50% lower carbon footprint compared to similar
+products currently available in the U.S. Students will explore decarbonization
+goals and market opportunities, helping Owens Corning understand how to
+best leverage the product’s sustainability advantages to create value in its  the
+data center and rebar end markets.
+Leveraging a powerful combination of material science, manufacturing
+excellence, and deep market and customer knowledge, the GR business
+provides sustainable, customer-centric solutions for the global wind, building
+and construction, thermoplastic compounding, and composites specialty
+markets. With annual revenues of approximately $1.2 billion, the business
+employs 4,000 people at 18 operations in 12 countries.
+WM (Waste Management): 
+Textile Recycling
+ThirdLove:
+Textile sustainability and circularity</t>
         </is>
       </c>
     </row>
@@ -79730,7 +81517,41 @@
 consulting (e.g., soft skills, such as leadership and interpersonal development,
 and hard skills, such as the hypothesis-driven approach, data analyses, and
 deliverable development/delivery). 
-Background:</t>
+Background:
+Professor Harry L. Davis is one of the top professors at Booth and has taught
+this course over many years. Joe Raudabaugh (Booth MBA ’17), a principle at
+Kearney, leads the effort for Kearney and is a strong supporter of experiential
+education at Booth. Adjunct Professor Craig Terrill has taught client-based lab
+classes at Booth during the last 11 years and was a senior partner in a
+management consulting firm early in his career.
+Enrollment &amp; Application:
+Consulting Lab is offered only to students in the Master in Management
+program (MiM) or Master in Finance program (MiF). Enrollment in this course is
+by application.
+1. A Zoom Informational Webinar will be held at 12-1 CST on Thursday,
+February 5, 2026. Course structure, expectations, and potential clients will
+be discussed. The webinar is optional, and students can apply without
+attending. An email will be sent to all MiM and MiF students the week prior
+with instructions for attending the webinar and a link for completing the
+application (link is also below).
+2. Application Deadline: Sunday, February 8, 2026.
+Click Here for the Application
+3. Students will be notified of acceptance by Tues, February 10.
+Class Location:
+This course will meet weekly at the Gleacher Center on Thursdays from 1:30 -
+4:30 pm. Please see the Gleacher/Booth 455 electronic boards to confirm
+location. Note below that there are three additional required meetings.
+Additional Meetings:
+In addition to the regular Thursday afternoon class sessions, there are three
+additional required meetings. If you cannot commit to attending these
+additional meetings, you should not apply for the course. Please note that the
+first one is before the spring quarter.
+Thursday, March 5, 2026: 5 pm to 7 pm, Gleacher - Initial training with
+Kearney
+Friday, March 27, 2026: 8 am to 12 pm, Gleacher - Kickoff meetings with
+Clients
+Friday, May 22, 2026: 8 am to 12 pm, Gleacher - Final Presentations to
+Clients</t>
         </is>
       </c>
     </row>
@@ -79777,7 +81598,42 @@
 addressing.
 In addition, each week students are given time to work on their client projects
 culminating in the final capstone in which students will present their findings
-and recommendations for the clients during the final week. Given the vast and</t>
+and recommendations for the clients during the final week. Given the vast and
+complicated nature of addressing economic development and wealth creation,
+we bring guest speakers who bring various perspectives that are important:
+entrepreneurs, elected officials, venture capitalists, leaders at anchor
+institutions, artists, and philanthropists, among them. Clients for the Winter
+2025 section will include:
+The Obama Presidential Center, in partnership with other South Side
+cultural institutions, is looking to explore revitalizing a tourism and brand
+strategy to support Museum Campus South.  As the Obama Presidential
+Center nears its public launch in 2026, students will develop a strategy to
+identify and amplify tourism opportunities for the broader network of
+cultural institutions that stand to benefit from significant new tourist
+activity in the broader South Side.
+The Garfield Park Community Council is working to address food
+insecurity in the broader community through a variety of strategies. 
+Having successfully recruited an anchor retailer to occupy a grocery retail
+site formerly occupied by Aldi, students will develop a retail launch,
+pricing, and customer retention strategy to ensure the success and
+profitability of the new grocery retail partner. 
+The Chicagoland Workforce Funder Alliance is a collaborative of over 30
+funders who develop and fund workforce solutions to strengthen
+workforce development strategies in the region.  This quarter, students
+will develop a strategy to support transportation access for people
+entering the workforce, in particular in the construction and trades where
+vehicle access is required to transit to work and job sites.  Students will
+explore various potential strategies including a shared fleet model, vehicle
+financing programs, or third party partnership models.
+Other project(s) TBA
+Applications for the Social Impact Lab (SIL) are now open, taught by Ghian
+Foreman and myself, Todd Connor. The course will be offered winter quarter
+on Tuesday mornings from 8:30 – 11:30am at the Harper Center. This course is
+open by application only.  Applications are due on 11/19/2025 at 5:00pm, and
+decisions will be sent out 11/21/2025.  Students applying early can also receive
+an early acceptance for course planning purposes.  The first class will be
+Tuesday, January 6th, 8:30-11:30am and is required for all enrolled
+students.  Interested students can apply here.</t>
         </is>
       </c>
     </row>
@@ -79834,7 +81690,14 @@
 Students apply individually and can work in groups of one to three. If you
 already have potential team members in mind, there is a place to note this on
 your application. This course is for anyone who has an interest in social
-entrepreneurship and wants to spend their quarter crafting their own social</t>
+entrepreneurship and wants to spend their quarter crafting their own social
+venture. It is designed to have a global feel and to feature placement partners
+and guest speakers representing a wide range of backgrounds. Note that this
+year, unlike in the previous two years, this year's course will focus fully on
+designing your own social venture ideas; there will not be an additional project
+component with partner social ventures.
+Applications are now open here and are due by Friday, November 7th at
+11:59pm CT.</t>
         </is>
       </c>
     </row>
@@ -79911,7 +81774,14 @@
 This course applies many of the concepts learned in other Booth courses.
 It is not necessary to have taken all of the classes, but we recommend
 building teams whose combined members have taken many of the
-classes.</t>
+classes.
+Students are given guidance but encouraged to think through problems
+and find their own answers.
+The simulation is designed to reflect a complex business environment. To
+run the business effectively students should expect to invest time and
+effort to (1) learn the interface, (2) analyze the business and its
+environment, (3) plan strategy and tactics, and (4) work with others to
+execute those plans in the face of competition.</t>
         </is>
       </c>
     </row>
@@ -80142,7 +82012,35 @@
 case discussions, analyzing how AI companies navigate critical decisions and
 trade-offs. Finally, students will apply these concepts and techniques through
 practical assignments, progressively designing an AI product by the end of the
-course.</t>
+course.  
+The first half of the course will be primarily focused on understanding the
+relevant frameworks to make decisions on AI products and illustrate them
+through case discussions, while the second half will be more focused on the
+practical aspects of building an AI product through hands-on application in
+class. 
+This is not a course on machine learning or generative AI—it’s a course on
+building AI products and businesses, not models or systems.
+However, AI products are highly technical, so students are expected to have at
+least a basic understanding of how AI works under the hood. The course will
+not cover fundamentals like how to train models and measure their
+performance, students are expected to be at least familiar with these topics. If
+terms like AUC, recall, or embeddings sound completely foreign, students
+should be aware that the workload to be successful in the course will be much
+higher. While recommended readings and resources will be provided for those
+who need to catch up, these concepts will not be explained in class.  
+You should NOT take this class if:
+Your main interest is to learn how to build AI models and systems. There
+are other technical classes you can take, not this one. 
+You want a lab class that will teach you to use different AI tools for product
+managers and founders. You don’t need a full term class to learn those
+tools, they are easy to learn on your own. While this class may provide a
+good opportunity to use some of those tools as part of your group project,
+we will not spend time teaching them. 
+You are not interested in frameworks and cases, you just want to build
+something. There are other pure lab courses you can take for that. This
+course takes the view that you can’t build great AI products without a
+rigorous decision-making framework, so a good part of the course is
+dedicated to teaching it.</t>
         </is>
       </c>
     </row>
@@ -80309,7 +82207,24 @@
 The course is about you, so we’ll start by identifying, practicing and refining a
 “leadership communication avatar” that captures how you want to come
 across and conveys your vision in a way that’s authentic. We’ll review and
-analyze examples of leadership communication and hear from guest speakers.</t>
+analyze examples of leadership communication and hear from guest speakers.
+Leadership communication is fundamentally different from operational and
+managerial communication. It is less about transmitting information and more
+about shaping interpretation. You will be challenged to move beyond the
+safety of describing what is, and to stake a claim about what could be. That
+shift from analyst to author, from manager to visionary, is rhetorical and
+intellectual. It requires a willingness to risk being wrong in order to lead.
+You will learn and practice articulating a vision, framing opportunities, and
+speaking persuasively about the future. Emphasis is placed on clarity, tone,
+narrative control, and intellectual authority. You will learn how to develop
+strategic foresight, use rhetorical devices to frame a vision, and how to project
+that vision in public.
+Throughout the course, we will analyze real-world examples of leadership
+speech, from quarterly earnings calls to public keynote addresses, and assess
+what makes them credible, memorable, and effective. You will be expected to
+produce work that combines expertise and insight with passion and conviction.
+The aim is not to create stylized performances, but to discover and articulate
+your own authentic leadership language.</t>
         </is>
       </c>
     </row>

</xml_diff>